<commit_message>
Update inventario_expandido.xlsx — pipeline 1206
</commit_message>
<xml_diff>
--- a/inventario_expandido.xlsx
+++ b/inventario_expandido.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Inventario" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Inventario'!$A$1:$O$487</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Inventario'!$A$1:$O$490</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -481,7 +481,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O487"/>
+  <dimension ref="A1:O490"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -14736,13 +14736,13 @@
         <v>0</v>
       </c>
       <c r="K254" s="2" t="n">
-        <v>0</v>
+        <v>415</v>
       </c>
       <c r="L254" s="2" t="n">
         <v>45</v>
       </c>
       <c r="M254" s="2" t="n">
-        <v>45</v>
+        <v>460</v>
       </c>
       <c r="N254" s="6" t="inlineStr">
         <is>
@@ -22773,13 +22773,13 @@
         <v>0</v>
       </c>
       <c r="K395" s="2" t="n">
-        <v>0</v>
+        <v>223</v>
       </c>
       <c r="L395" s="2" t="n">
         <v>53</v>
       </c>
       <c r="M395" s="2" t="n">
-        <v>53</v>
+        <v>276</v>
       </c>
       <c r="N395" s="6" t="inlineStr">
         <is>
@@ -22940,13 +22940,13 @@
         <v>0</v>
       </c>
       <c r="K398" s="2" t="n">
-        <v>0</v>
+        <v>851</v>
       </c>
       <c r="L398" s="2" t="n">
         <v>405</v>
       </c>
       <c r="M398" s="2" t="n">
-        <v>405</v>
+        <v>1256</v>
       </c>
       <c r="N398" s="6" t="inlineStr">
         <is>
@@ -23047,7 +23047,7 @@
         </is>
       </c>
       <c r="J400" s="2" t="n">
-        <v>0</v>
+        <v>178</v>
       </c>
       <c r="K400" s="2" t="n">
         <v>305</v>
@@ -23056,11 +23056,11 @@
         <v>93</v>
       </c>
       <c r="M400" s="2" t="n">
-        <v>398</v>
-      </c>
-      <c r="N400" s="6" t="inlineStr">
-        <is>
-          <t>7/10 Días</t>
+        <v>576</v>
+      </c>
+      <c r="N400" s="4" t="inlineStr">
+        <is>
+          <t>Stock</t>
         </is>
       </c>
       <c r="O400" s="2" t="n">
@@ -23338,10 +23338,10 @@
         <v>595</v>
       </c>
       <c r="L405" s="2" t="n">
-        <v>0</v>
+        <v>168</v>
       </c>
       <c r="M405" s="2" t="n">
-        <v>675</v>
+        <v>843</v>
       </c>
       <c r="N405" s="4" t="inlineStr">
         <is>
@@ -23674,7 +23674,7 @@
         </is>
       </c>
       <c r="J411" s="2" t="n">
-        <v>0</v>
+        <v>201</v>
       </c>
       <c r="K411" s="2" t="n">
         <v>1290</v>
@@ -23683,11 +23683,11 @@
         <v>3</v>
       </c>
       <c r="M411" s="2" t="n">
-        <v>1293</v>
-      </c>
-      <c r="N411" s="6" t="inlineStr">
-        <is>
-          <t>7/10 Días</t>
+        <v>1494</v>
+      </c>
+      <c r="N411" s="4" t="inlineStr">
+        <is>
+          <t>Stock</t>
         </is>
       </c>
       <c r="O411" s="2" t="n">
@@ -23731,20 +23731,20 @@
         </is>
       </c>
       <c r="J412" s="2" t="n">
-        <v>0</v>
+        <v>399</v>
       </c>
       <c r="K412" s="2" t="n">
-        <v>0</v>
+        <v>1957</v>
       </c>
       <c r="L412" s="2" t="n">
         <v>715</v>
       </c>
       <c r="M412" s="2" t="n">
-        <v>715</v>
-      </c>
-      <c r="N412" s="6" t="inlineStr">
-        <is>
-          <t>7/10 Días</t>
+        <v>3071</v>
+      </c>
+      <c r="N412" s="4" t="inlineStr">
+        <is>
+          <t>Stock</t>
         </is>
       </c>
       <c r="O412" s="2" t="n">
@@ -23788,20 +23788,20 @@
         </is>
       </c>
       <c r="J413" s="2" t="n">
-        <v>0</v>
+        <v>189</v>
       </c>
       <c r="K413" s="2" t="n">
-        <v>0</v>
+        <v>766</v>
       </c>
       <c r="L413" s="2" t="n">
         <v>131</v>
       </c>
       <c r="M413" s="2" t="n">
-        <v>131</v>
-      </c>
-      <c r="N413" s="6" t="inlineStr">
-        <is>
-          <t>7/10 Días</t>
+        <v>1086</v>
+      </c>
+      <c r="N413" s="4" t="inlineStr">
+        <is>
+          <t>Stock</t>
         </is>
       </c>
       <c r="O413" s="2" t="n">
@@ -23905,13 +23905,13 @@
         <v>300</v>
       </c>
       <c r="K415" s="2" t="n">
-        <v>0</v>
+        <v>783</v>
       </c>
       <c r="L415" s="2" t="n">
         <v>96</v>
       </c>
       <c r="M415" s="2" t="n">
-        <v>396</v>
+        <v>1179</v>
       </c>
       <c r="N415" s="4" t="inlineStr">
         <is>
@@ -24079,10 +24079,10 @@
         <v>530</v>
       </c>
       <c r="L418" s="2" t="n">
-        <v>0</v>
+        <v>282</v>
       </c>
       <c r="M418" s="2" t="n">
-        <v>621</v>
+        <v>903</v>
       </c>
       <c r="N418" s="4" t="inlineStr">
         <is>
@@ -24190,13 +24190,13 @@
         <v>128</v>
       </c>
       <c r="K420" s="2" t="n">
-        <v>0</v>
+        <v>282</v>
       </c>
       <c r="L420" s="2" t="n">
         <v>83</v>
       </c>
       <c r="M420" s="2" t="n">
-        <v>211</v>
+        <v>493</v>
       </c>
       <c r="N420" s="4" t="inlineStr">
         <is>
@@ -24247,13 +24247,13 @@
         <v>0</v>
       </c>
       <c r="K421" s="2" t="n">
-        <v>0</v>
+        <v>193</v>
       </c>
       <c r="L421" s="2" t="n">
         <v>109</v>
       </c>
       <c r="M421" s="2" t="n">
-        <v>109</v>
+        <v>302</v>
       </c>
       <c r="N421" s="6" t="inlineStr">
         <is>
@@ -24358,7 +24358,7 @@
         </is>
       </c>
       <c r="J423" s="2" t="n">
-        <v>0</v>
+        <v>157</v>
       </c>
       <c r="K423" s="2" t="n">
         <v>92</v>
@@ -24367,11 +24367,11 @@
         <v>0</v>
       </c>
       <c r="M423" s="2" t="n">
-        <v>92</v>
-      </c>
-      <c r="N423" s="6" t="inlineStr">
-        <is>
-          <t>7/10 Días</t>
+        <v>249</v>
+      </c>
+      <c r="N423" s="4" t="inlineStr">
+        <is>
+          <t>Stock</t>
         </is>
       </c>
       <c r="O423" s="2" t="n">
@@ -24438,12 +24438,12 @@
     <row r="425">
       <c r="A425" s="2" t="inlineStr">
         <is>
-          <t>NOR0032111</t>
+          <t>NOR0032110</t>
         </is>
       </c>
       <c r="B425" s="3" t="inlineStr">
         <is>
-          <t>ANGULO 80 X 40 X 1.25</t>
+          <t>ANGULO 60 X 40 X 1.5</t>
         </is>
       </c>
       <c r="C425" s="2" t="inlineStr">
@@ -24452,19 +24452,19 @@
         </is>
       </c>
       <c r="D425" s="2" t="n">
-        <v>80</v>
+        <v>60</v>
       </c>
       <c r="E425" s="2" t="n">
         <v>40</v>
       </c>
       <c r="F425" s="2" t="n">
-        <v>1.25</v>
+        <v>1.5</v>
       </c>
       <c r="G425" s="2" t="n">
         <v>6.4</v>
       </c>
       <c r="H425" s="2" t="n">
-        <v>0.4005</v>
+        <v>0.3996</v>
       </c>
       <c r="I425" s="2" t="inlineStr">
         <is>
@@ -24472,16 +24472,16 @@
         </is>
       </c>
       <c r="J425" s="2" t="n">
-        <v>77</v>
+        <v>179</v>
       </c>
       <c r="K425" s="2" t="n">
-        <v>0</v>
+        <v>226</v>
       </c>
       <c r="L425" s="2" t="n">
-        <v>0</v>
+        <v>236</v>
       </c>
       <c r="M425" s="2" t="n">
-        <v>77</v>
+        <v>641</v>
       </c>
       <c r="N425" s="4" t="inlineStr">
         <is>
@@ -24495,12 +24495,12 @@
     <row r="426">
       <c r="A426" s="2" t="inlineStr">
         <is>
-          <t>NOR0032112</t>
+          <t>NOR0032111</t>
         </is>
       </c>
       <c r="B426" s="3" t="inlineStr">
         <is>
-          <t>ANGULO 30 X 15 X 1,2</t>
+          <t>ANGULO 80 X 40 X 1.25</t>
         </is>
       </c>
       <c r="C426" s="2" t="inlineStr">
@@ -24509,19 +24509,19 @@
         </is>
       </c>
       <c r="D426" s="2" t="n">
-        <v>30</v>
+        <v>80</v>
       </c>
       <c r="E426" s="2" t="n">
-        <v>15</v>
+        <v>40</v>
       </c>
       <c r="F426" s="2" t="n">
-        <v>1.2</v>
+        <v>1.25</v>
       </c>
       <c r="G426" s="2" t="n">
         <v>6.4</v>
       </c>
       <c r="H426" s="2" t="n">
-        <v>0.142</v>
+        <v>0.4005</v>
       </c>
       <c r="I426" s="2" t="inlineStr">
         <is>
@@ -24529,35 +24529,35 @@
         </is>
       </c>
       <c r="J426" s="2" t="n">
-        <v>0</v>
+        <v>77</v>
       </c>
       <c r="K426" s="2" t="n">
-        <v>0</v>
+        <v>237</v>
       </c>
       <c r="L426" s="2" t="n">
-        <v>60</v>
+        <v>252</v>
       </c>
       <c r="M426" s="2" t="n">
-        <v>60</v>
-      </c>
-      <c r="N426" s="6" t="inlineStr">
-        <is>
-          <t>7/10 Días</t>
+        <v>566</v>
+      </c>
+      <c r="N426" s="4" t="inlineStr">
+        <is>
+          <t>Stock</t>
         </is>
       </c>
       <c r="O426" s="2" t="n">
-        <v>0.97</v>
+        <v>2.72</v>
       </c>
     </row>
     <row r="427">
       <c r="A427" s="2" t="inlineStr">
         <is>
-          <t>NOR0032115</t>
+          <t>NOR0032112</t>
         </is>
       </c>
       <c r="B427" s="3" t="inlineStr">
         <is>
-          <t>ANGULO 100 X 40 X 1,8</t>
+          <t>ANGULO 30 X 15 X 1,2</t>
         </is>
       </c>
       <c r="C427" s="2" t="inlineStr">
@@ -24566,19 +24566,19 @@
         </is>
       </c>
       <c r="D427" s="2" t="n">
-        <v>100</v>
+        <v>30</v>
       </c>
       <c r="E427" s="2" t="n">
-        <v>40</v>
+        <v>15</v>
       </c>
       <c r="F427" s="2" t="n">
-        <v>1.8</v>
+        <v>1.2</v>
       </c>
       <c r="G427" s="2" t="n">
         <v>6.4</v>
       </c>
       <c r="H427" s="2" t="n">
-        <v>0.672</v>
+        <v>0.142</v>
       </c>
       <c r="I427" s="2" t="inlineStr">
         <is>
@@ -24586,16 +24586,16 @@
         </is>
       </c>
       <c r="J427" s="2" t="n">
-        <v>144</v>
+        <v>191</v>
       </c>
       <c r="K427" s="2" t="n">
-        <v>40</v>
+        <v>212</v>
       </c>
       <c r="L427" s="2" t="n">
-        <v>138</v>
+        <v>60</v>
       </c>
       <c r="M427" s="2" t="n">
-        <v>322</v>
+        <v>463</v>
       </c>
       <c r="N427" s="4" t="inlineStr">
         <is>
@@ -24603,18 +24603,18 @@
         </is>
       </c>
       <c r="O427" s="2" t="n">
-        <v>4.57</v>
+        <v>0.97</v>
       </c>
     </row>
     <row r="428">
       <c r="A428" s="2" t="inlineStr">
         <is>
-          <t>NOR0032116</t>
+          <t>NOR0032115</t>
         </is>
       </c>
       <c r="B428" s="3" t="inlineStr">
         <is>
-          <t>ANGULO 25 X 1.5</t>
+          <t>ANGULO 100 X 40 X 1,8</t>
         </is>
       </c>
       <c r="C428" s="2" t="inlineStr">
@@ -24623,19 +24623,19 @@
         </is>
       </c>
       <c r="D428" s="2" t="n">
-        <v>25</v>
+        <v>100</v>
       </c>
       <c r="E428" s="2" t="n">
-        <v>25</v>
+        <v>40</v>
       </c>
       <c r="F428" s="2" t="n">
-        <v>1.5</v>
+        <v>1.8</v>
       </c>
       <c r="G428" s="2" t="n">
-        <v>6</v>
+        <v>6.4</v>
       </c>
       <c r="H428" s="2" t="n">
-        <v>0.1982</v>
+        <v>0.672</v>
       </c>
       <c r="I428" s="2" t="inlineStr">
         <is>
@@ -24643,35 +24643,35 @@
         </is>
       </c>
       <c r="J428" s="2" t="n">
-        <v>0</v>
+        <v>144</v>
       </c>
       <c r="K428" s="2" t="n">
-        <v>282</v>
+        <v>40</v>
       </c>
       <c r="L428" s="2" t="n">
-        <v>282</v>
+        <v>138</v>
       </c>
       <c r="M428" s="2" t="n">
-        <v>564</v>
-      </c>
-      <c r="N428" s="6" t="inlineStr">
-        <is>
-          <t>7/10 Días</t>
+        <v>322</v>
+      </c>
+      <c r="N428" s="4" t="inlineStr">
+        <is>
+          <t>Stock</t>
         </is>
       </c>
       <c r="O428" s="2" t="n">
-        <v>1.35</v>
+        <v>4.57</v>
       </c>
     </row>
     <row r="429">
       <c r="A429" s="2" t="inlineStr">
         <is>
-          <t>NOR0032117</t>
+          <t>NOR0032116</t>
         </is>
       </c>
       <c r="B429" s="3" t="inlineStr">
         <is>
-          <t>ANGULO 50 X 25 X 1,7</t>
+          <t>ANGULO 25 X 1.5</t>
         </is>
       </c>
       <c r="C429" s="2" t="inlineStr">
@@ -24680,19 +24680,19 @@
         </is>
       </c>
       <c r="D429" s="2" t="n">
-        <v>50</v>
+        <v>25</v>
       </c>
       <c r="E429" s="2" t="n">
         <v>25</v>
       </c>
       <c r="F429" s="2" t="n">
-        <v>1.7</v>
+        <v>1.5</v>
       </c>
       <c r="G429" s="2" t="n">
-        <v>6.4</v>
+        <v>6</v>
       </c>
       <c r="H429" s="2" t="n">
-        <v>0.338</v>
+        <v>0.1982</v>
       </c>
       <c r="I429" s="2" t="inlineStr">
         <is>
@@ -24700,35 +24700,35 @@
         </is>
       </c>
       <c r="J429" s="2" t="n">
-        <v>80</v>
+        <v>0</v>
       </c>
       <c r="K429" s="2" t="n">
-        <v>0</v>
+        <v>282</v>
       </c>
       <c r="L429" s="2" t="n">
-        <v>31</v>
+        <v>282</v>
       </c>
       <c r="M429" s="2" t="n">
-        <v>111</v>
-      </c>
-      <c r="N429" s="4" t="inlineStr">
-        <is>
-          <t>Stock</t>
+        <v>564</v>
+      </c>
+      <c r="N429" s="6" t="inlineStr">
+        <is>
+          <t>7/10 Días</t>
         </is>
       </c>
       <c r="O429" s="2" t="n">
-        <v>2.3</v>
+        <v>1.35</v>
       </c>
     </row>
     <row r="430">
       <c r="A430" s="2" t="inlineStr">
         <is>
-          <t>NOR0032120</t>
+          <t>NOR0032117</t>
         </is>
       </c>
       <c r="B430" s="3" t="inlineStr">
         <is>
-          <t>ANGULO 53 X 28 X 1.5 CH.</t>
+          <t>ANGULO 50 X 25 X 1,7</t>
         </is>
       </c>
       <c r="C430" s="2" t="inlineStr">
@@ -24737,19 +24737,19 @@
         </is>
       </c>
       <c r="D430" s="2" t="n">
-        <v>53</v>
+        <v>50</v>
       </c>
       <c r="E430" s="2" t="n">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="F430" s="2" t="n">
-        <v>1.5</v>
+        <v>1.7</v>
       </c>
       <c r="G430" s="2" t="n">
         <v>6.4</v>
       </c>
       <c r="H430" s="2" t="n">
-        <v>0.32</v>
+        <v>0.338</v>
       </c>
       <c r="I430" s="2" t="inlineStr">
         <is>
@@ -24757,56 +24757,56 @@
         </is>
       </c>
       <c r="J430" s="2" t="n">
-        <v>0</v>
+        <v>80</v>
       </c>
       <c r="K430" s="2" t="n">
-        <v>50</v>
+        <v>283</v>
       </c>
       <c r="L430" s="2" t="n">
-        <v>0</v>
+        <v>31</v>
       </c>
       <c r="M430" s="2" t="n">
-        <v>50</v>
-      </c>
-      <c r="N430" s="6" t="inlineStr">
-        <is>
-          <t>7/10 Días</t>
+        <v>394</v>
+      </c>
+      <c r="N430" s="4" t="inlineStr">
+        <is>
+          <t>Stock</t>
         </is>
       </c>
       <c r="O430" s="2" t="n">
-        <v>2.18</v>
+        <v>2.3</v>
       </c>
     </row>
     <row r="431">
       <c r="A431" s="2" t="inlineStr">
         <is>
-          <t>NOR0032200</t>
+          <t>NOR0032120</t>
         </is>
       </c>
       <c r="B431" s="3" t="inlineStr">
         <is>
-          <t>TUBO CUADRADO 16 X 1.3</t>
+          <t>ANGULO 53 X 28 X 1.5 CH.</t>
         </is>
       </c>
       <c r="C431" s="2" t="inlineStr">
         <is>
-          <t>TUBO CUADRADO</t>
+          <t>ANGULO</t>
         </is>
       </c>
       <c r="D431" s="2" t="n">
-        <v>16</v>
+        <v>53</v>
       </c>
       <c r="E431" s="2" t="n">
-        <v>16</v>
+        <v>28</v>
       </c>
       <c r="F431" s="2" t="n">
-        <v>1.3</v>
+        <v>1.5</v>
       </c>
       <c r="G431" s="2" t="n">
         <v>6.4</v>
       </c>
       <c r="H431" s="2" t="n">
-        <v>0.206</v>
+        <v>0.32</v>
       </c>
       <c r="I431" s="2" t="inlineStr">
         <is>
@@ -24814,35 +24814,35 @@
         </is>
       </c>
       <c r="J431" s="2" t="n">
-        <v>137</v>
+        <v>0</v>
       </c>
       <c r="K431" s="2" t="n">
-        <v>510</v>
+        <v>50</v>
       </c>
       <c r="L431" s="2" t="n">
-        <v>82</v>
+        <v>0</v>
       </c>
       <c r="M431" s="2" t="n">
-        <v>729</v>
-      </c>
-      <c r="N431" s="4" t="inlineStr">
-        <is>
-          <t>Stock</t>
+        <v>50</v>
+      </c>
+      <c r="N431" s="6" t="inlineStr">
+        <is>
+          <t>7/10 Días</t>
         </is>
       </c>
       <c r="O431" s="2" t="n">
-        <v>1.4</v>
+        <v>2.18</v>
       </c>
     </row>
     <row r="432">
       <c r="A432" s="2" t="inlineStr">
         <is>
-          <t>NOR0032201</t>
+          <t>NOR0032200</t>
         </is>
       </c>
       <c r="B432" s="3" t="inlineStr">
         <is>
-          <t>TUBO CUADRADO 20 X 1,3</t>
+          <t>TUBO CUADRADO 16 X 1.3</t>
         </is>
       </c>
       <c r="C432" s="2" t="inlineStr">
@@ -24851,19 +24851,19 @@
         </is>
       </c>
       <c r="D432" s="2" t="n">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="E432" s="2" t="n">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="F432" s="2" t="n">
         <v>1.3</v>
       </c>
       <c r="G432" s="2" t="n">
-        <v>6</v>
+        <v>6.4</v>
       </c>
       <c r="H432" s="2" t="n">
-        <v>0.2624</v>
+        <v>0.206</v>
       </c>
       <c r="I432" s="2" t="inlineStr">
         <is>
@@ -24871,35 +24871,35 @@
         </is>
       </c>
       <c r="J432" s="2" t="n">
-        <v>0</v>
+        <v>137</v>
       </c>
       <c r="K432" s="2" t="n">
-        <v>2</v>
+        <v>510</v>
       </c>
       <c r="L432" s="2" t="n">
-        <v>0</v>
+        <v>82</v>
       </c>
       <c r="M432" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="N432" s="5" t="inlineStr">
-        <is>
-          <t>Sin stock</t>
+        <v>729</v>
+      </c>
+      <c r="N432" s="4" t="inlineStr">
+        <is>
+          <t>Stock</t>
         </is>
       </c>
       <c r="O432" s="2" t="n">
-        <v>1.78</v>
+        <v>1.4</v>
       </c>
     </row>
     <row r="433">
       <c r="A433" s="2" t="inlineStr">
         <is>
-          <t>NOR0032202</t>
+          <t>NOR0032201</t>
         </is>
       </c>
       <c r="B433" s="3" t="inlineStr">
         <is>
-          <t>TUBO CUADRADO 25 X 1.3</t>
+          <t>TUBO CUADRADO 20 X 1,3</t>
         </is>
       </c>
       <c r="C433" s="2" t="inlineStr">
@@ -24908,10 +24908,10 @@
         </is>
       </c>
       <c r="D433" s="2" t="n">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="E433" s="2" t="n">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="F433" s="2" t="n">
         <v>1.3</v>
@@ -24920,7 +24920,7 @@
         <v>6</v>
       </c>
       <c r="H433" s="2" t="n">
-        <v>0.332</v>
+        <v>0.2624</v>
       </c>
       <c r="I433" s="2" t="inlineStr">
         <is>
@@ -24931,32 +24931,32 @@
         <v>0</v>
       </c>
       <c r="K433" s="2" t="n">
-        <v>55</v>
+        <v>2</v>
       </c>
       <c r="L433" s="2" t="n">
-        <v>46</v>
+        <v>0</v>
       </c>
       <c r="M433" s="2" t="n">
-        <v>101</v>
-      </c>
-      <c r="N433" s="6" t="inlineStr">
-        <is>
-          <t>7/10 Días</t>
+        <v>2</v>
+      </c>
+      <c r="N433" s="5" t="inlineStr">
+        <is>
+          <t>Sin stock</t>
         </is>
       </c>
       <c r="O433" s="2" t="n">
-        <v>2.26</v>
+        <v>1.78</v>
       </c>
     </row>
     <row r="434">
       <c r="A434" s="2" t="inlineStr">
         <is>
-          <t>NOR0032202</t>
+          <t>NOR0032201</t>
         </is>
       </c>
       <c r="B434" s="3" t="inlineStr">
         <is>
-          <t>TUBO CUADRADO 25 X 1.3</t>
+          <t>TUBO CUADRADO 20 X 1,3</t>
         </is>
       </c>
       <c r="C434" s="2" t="inlineStr">
@@ -24965,10 +24965,10 @@
         </is>
       </c>
       <c r="D434" s="2" t="n">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="E434" s="2" t="n">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="F434" s="2" t="n">
         <v>1.3</v>
@@ -24977,7 +24977,7 @@
         <v>6.4</v>
       </c>
       <c r="H434" s="2" t="n">
-        <v>0.332</v>
+        <v>0.2624</v>
       </c>
       <c r="I434" s="2" t="inlineStr">
         <is>
@@ -24988,13 +24988,13 @@
         <v>0</v>
       </c>
       <c r="K434" s="2" t="n">
-        <v>0</v>
+        <v>347</v>
       </c>
       <c r="L434" s="2" t="n">
-        <v>24</v>
+        <v>157</v>
       </c>
       <c r="M434" s="2" t="n">
-        <v>24</v>
+        <v>504</v>
       </c>
       <c r="N434" s="6" t="inlineStr">
         <is>
@@ -25002,18 +25002,18 @@
         </is>
       </c>
       <c r="O434" s="2" t="n">
-        <v>2.26</v>
+        <v>1.78</v>
       </c>
     </row>
     <row r="435">
       <c r="A435" s="2" t="inlineStr">
         <is>
-          <t>NOR0032203</t>
+          <t>NOR0032202</t>
         </is>
       </c>
       <c r="B435" s="3" t="inlineStr">
         <is>
-          <t>TUBO CUADRADO 30 X 1.3</t>
+          <t>TUBO CUADRADO 25 X 1.3</t>
         </is>
       </c>
       <c r="C435" s="2" t="inlineStr">
@@ -25022,19 +25022,19 @@
         </is>
       </c>
       <c r="D435" s="2" t="n">
-        <v>30</v>
+        <v>25</v>
       </c>
       <c r="E435" s="2" t="n">
-        <v>30</v>
+        <v>25</v>
       </c>
       <c r="F435" s="2" t="n">
         <v>1.3</v>
       </c>
       <c r="G435" s="2" t="n">
-        <v>6.4</v>
+        <v>6</v>
       </c>
       <c r="H435" s="2" t="n">
-        <v>0.402</v>
+        <v>0.332</v>
       </c>
       <c r="I435" s="2" t="inlineStr">
         <is>
@@ -25042,16 +25042,16 @@
         </is>
       </c>
       <c r="J435" s="2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K435" s="2" t="n">
-        <v>0</v>
+        <v>55</v>
       </c>
       <c r="L435" s="2" t="n">
-        <v>119</v>
+        <v>46</v>
       </c>
       <c r="M435" s="2" t="n">
-        <v>121</v>
+        <v>101</v>
       </c>
       <c r="N435" s="6" t="inlineStr">
         <is>
@@ -25059,18 +25059,18 @@
         </is>
       </c>
       <c r="O435" s="2" t="n">
-        <v>2.73</v>
+        <v>2.26</v>
       </c>
     </row>
     <row r="436">
       <c r="A436" s="2" t="inlineStr">
         <is>
-          <t>NOR0032204</t>
+          <t>NOR0032202</t>
         </is>
       </c>
       <c r="B436" s="3" t="inlineStr">
         <is>
-          <t>TUBO CUADRADO 40 X 1.3</t>
+          <t>TUBO CUADRADO 25 X 1.3</t>
         </is>
       </c>
       <c r="C436" s="2" t="inlineStr">
@@ -25079,10 +25079,10 @@
         </is>
       </c>
       <c r="D436" s="2" t="n">
-        <v>40</v>
+        <v>25</v>
       </c>
       <c r="E436" s="2" t="n">
-        <v>40</v>
+        <v>25</v>
       </c>
       <c r="F436" s="2" t="n">
         <v>1.3</v>
@@ -25091,7 +25091,7 @@
         <v>6.4</v>
       </c>
       <c r="H436" s="2" t="n">
-        <v>0.543</v>
+        <v>0.332</v>
       </c>
       <c r="I436" s="2" t="inlineStr">
         <is>
@@ -25099,35 +25099,35 @@
         </is>
       </c>
       <c r="J436" s="2" t="n">
-        <v>0</v>
+        <v>218</v>
       </c>
       <c r="K436" s="2" t="n">
-        <v>66</v>
+        <v>239</v>
       </c>
       <c r="L436" s="2" t="n">
-        <v>0</v>
+        <v>24</v>
       </c>
       <c r="M436" s="2" t="n">
-        <v>66</v>
-      </c>
-      <c r="N436" s="6" t="inlineStr">
-        <is>
-          <t>7/10 Días</t>
+        <v>481</v>
+      </c>
+      <c r="N436" s="4" t="inlineStr">
+        <is>
+          <t>Stock</t>
         </is>
       </c>
       <c r="O436" s="2" t="n">
-        <v>3.69</v>
+        <v>2.26</v>
       </c>
     </row>
     <row r="437">
       <c r="A437" s="2" t="inlineStr">
         <is>
-          <t>NOR0032205</t>
+          <t>NOR0032203</t>
         </is>
       </c>
       <c r="B437" s="3" t="inlineStr">
         <is>
-          <t>TUBO CUADRADO 45 X 1.5</t>
+          <t>TUBO CUADRADO 30 X 1.3</t>
         </is>
       </c>
       <c r="C437" s="2" t="inlineStr">
@@ -25136,19 +25136,19 @@
         </is>
       </c>
       <c r="D437" s="2" t="n">
-        <v>45</v>
+        <v>30</v>
       </c>
       <c r="E437" s="2" t="n">
-        <v>45</v>
+        <v>30</v>
       </c>
       <c r="F437" s="2" t="n">
-        <v>1.5</v>
+        <v>1.3</v>
       </c>
       <c r="G437" s="2" t="n">
-        <v>6</v>
+        <v>6.4</v>
       </c>
       <c r="H437" s="2" t="n">
-        <v>0.705</v>
+        <v>0.402</v>
       </c>
       <c r="I437" s="2" t="inlineStr">
         <is>
@@ -25156,35 +25156,35 @@
         </is>
       </c>
       <c r="J437" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K437" s="2" t="n">
-        <v>2</v>
+        <v>263</v>
       </c>
       <c r="L437" s="2" t="n">
-        <v>3</v>
+        <v>119</v>
       </c>
       <c r="M437" s="2" t="n">
-        <v>5</v>
-      </c>
-      <c r="N437" s="5" t="inlineStr">
-        <is>
-          <t>Sin stock</t>
+        <v>384</v>
+      </c>
+      <c r="N437" s="6" t="inlineStr">
+        <is>
+          <t>7/10 Días</t>
         </is>
       </c>
       <c r="O437" s="2" t="n">
-        <v>4.79</v>
+        <v>2.73</v>
       </c>
     </row>
     <row r="438">
       <c r="A438" s="2" t="inlineStr">
         <is>
-          <t>NOR0032205</t>
+          <t>NOR0032204</t>
         </is>
       </c>
       <c r="B438" s="3" t="inlineStr">
         <is>
-          <t>TUBO CUADRADO 45 X 1.5</t>
+          <t>TUBO CUADRADO 40 X 1.3</t>
         </is>
       </c>
       <c r="C438" s="2" t="inlineStr">
@@ -25193,19 +25193,19 @@
         </is>
       </c>
       <c r="D438" s="2" t="n">
-        <v>45</v>
+        <v>40</v>
       </c>
       <c r="E438" s="2" t="n">
-        <v>45</v>
+        <v>40</v>
       </c>
       <c r="F438" s="2" t="n">
-        <v>1.5</v>
+        <v>1.3</v>
       </c>
       <c r="G438" s="2" t="n">
         <v>6.4</v>
       </c>
       <c r="H438" s="2" t="n">
-        <v>0.705</v>
+        <v>0.543</v>
       </c>
       <c r="I438" s="2" t="inlineStr">
         <is>
@@ -25213,35 +25213,35 @@
         </is>
       </c>
       <c r="J438" s="2" t="n">
-        <v>0</v>
+        <v>169</v>
       </c>
       <c r="K438" s="2" t="n">
-        <v>139</v>
+        <v>66</v>
       </c>
       <c r="L438" s="2" t="n">
-        <v>59</v>
+        <v>191</v>
       </c>
       <c r="M438" s="2" t="n">
-        <v>198</v>
-      </c>
-      <c r="N438" s="6" t="inlineStr">
-        <is>
-          <t>7/10 Días</t>
+        <v>426</v>
+      </c>
+      <c r="N438" s="4" t="inlineStr">
+        <is>
+          <t>Stock</t>
         </is>
       </c>
       <c r="O438" s="2" t="n">
-        <v>4.79</v>
+        <v>3.69</v>
       </c>
     </row>
     <row r="439">
       <c r="A439" s="2" t="inlineStr">
         <is>
-          <t>NOR0032206</t>
+          <t>NOR0032205</t>
         </is>
       </c>
       <c r="B439" s="3" t="inlineStr">
         <is>
-          <t>TUBO CUADRADO 50 X 1,3</t>
+          <t>TUBO CUADRADO 45 X 1.5</t>
         </is>
       </c>
       <c r="C439" s="2" t="inlineStr">
@@ -25250,19 +25250,19 @@
         </is>
       </c>
       <c r="D439" s="2" t="n">
-        <v>50</v>
+        <v>45</v>
       </c>
       <c r="E439" s="2" t="n">
-        <v>50</v>
+        <v>45</v>
       </c>
       <c r="F439" s="2" t="n">
-        <v>1.3</v>
+        <v>1.5</v>
       </c>
       <c r="G439" s="2" t="n">
         <v>6</v>
       </c>
       <c r="H439" s="2" t="n">
-        <v>0.6830000000000001</v>
+        <v>0.705</v>
       </c>
       <c r="I439" s="2" t="inlineStr">
         <is>
@@ -25273,32 +25273,32 @@
         <v>0</v>
       </c>
       <c r="K439" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="L439" s="2" t="n">
-        <v>36</v>
+        <v>3</v>
       </c>
       <c r="M439" s="2" t="n">
-        <v>36</v>
-      </c>
-      <c r="N439" s="6" t="inlineStr">
-        <is>
-          <t>7/10 Días</t>
+        <v>5</v>
+      </c>
+      <c r="N439" s="5" t="inlineStr">
+        <is>
+          <t>Sin stock</t>
         </is>
       </c>
       <c r="O439" s="2" t="n">
-        <v>4.64</v>
+        <v>4.79</v>
       </c>
     </row>
     <row r="440">
       <c r="A440" s="2" t="inlineStr">
         <is>
-          <t>NOR0032206</t>
+          <t>NOR0032205</t>
         </is>
       </c>
       <c r="B440" s="3" t="inlineStr">
         <is>
-          <t>TUBO CUADRADO 50 X 1,3</t>
+          <t>TUBO CUADRADO 45 X 1.5</t>
         </is>
       </c>
       <c r="C440" s="2" t="inlineStr">
@@ -25307,19 +25307,19 @@
         </is>
       </c>
       <c r="D440" s="2" t="n">
-        <v>50</v>
+        <v>45</v>
       </c>
       <c r="E440" s="2" t="n">
-        <v>50</v>
+        <v>45</v>
       </c>
       <c r="F440" s="2" t="n">
-        <v>1.3</v>
+        <v>1.5</v>
       </c>
       <c r="G440" s="2" t="n">
         <v>6.4</v>
       </c>
       <c r="H440" s="2" t="n">
-        <v>0.6830000000000001</v>
+        <v>0.705</v>
       </c>
       <c r="I440" s="2" t="inlineStr">
         <is>
@@ -25327,35 +25327,35 @@
         </is>
       </c>
       <c r="J440" s="2" t="n">
-        <v>19</v>
+        <v>0</v>
       </c>
       <c r="K440" s="2" t="n">
-        <v>67</v>
+        <v>139</v>
       </c>
       <c r="L440" s="2" t="n">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="M440" s="2" t="n">
-        <v>147</v>
-      </c>
-      <c r="N440" s="4" t="inlineStr">
-        <is>
-          <t>Stock</t>
+        <v>198</v>
+      </c>
+      <c r="N440" s="6" t="inlineStr">
+        <is>
+          <t>7/10 Días</t>
         </is>
       </c>
       <c r="O440" s="2" t="n">
-        <v>4.64</v>
+        <v>4.79</v>
       </c>
     </row>
     <row r="441">
       <c r="A441" s="2" t="inlineStr">
         <is>
-          <t>NOR0032207</t>
+          <t>NOR0032206</t>
         </is>
       </c>
       <c r="B441" s="3" t="inlineStr">
         <is>
-          <t>TUBO CUADRADO 60 X 1,3</t>
+          <t>TUBO CUADRADO 50 X 1,3</t>
         </is>
       </c>
       <c r="C441" s="2" t="inlineStr">
@@ -25364,19 +25364,19 @@
         </is>
       </c>
       <c r="D441" s="2" t="n">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="E441" s="2" t="n">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="F441" s="2" t="n">
         <v>1.3</v>
       </c>
       <c r="G441" s="2" t="n">
-        <v>6.4</v>
+        <v>6</v>
       </c>
       <c r="H441" s="2" t="n">
-        <v>0.8235</v>
+        <v>0.6830000000000001</v>
       </c>
       <c r="I441" s="2" t="inlineStr">
         <is>
@@ -25384,16 +25384,16 @@
         </is>
       </c>
       <c r="J441" s="2" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="K441" s="2" t="n">
-        <v>82</v>
+        <v>0</v>
       </c>
       <c r="L441" s="2" t="n">
-        <v>94</v>
+        <v>36</v>
       </c>
       <c r="M441" s="2" t="n">
-        <v>181</v>
+        <v>36</v>
       </c>
       <c r="N441" s="6" t="inlineStr">
         <is>
@@ -25401,18 +25401,18 @@
         </is>
       </c>
       <c r="O441" s="2" t="n">
-        <v>5.6</v>
+        <v>4.64</v>
       </c>
     </row>
     <row r="442">
       <c r="A442" s="2" t="inlineStr">
         <is>
-          <t>NOR0032208</t>
+          <t>NOR0032206</t>
         </is>
       </c>
       <c r="B442" s="3" t="inlineStr">
         <is>
-          <t>TUBO CUADRADO 70 X 1,3</t>
+          <t>TUBO CUADRADO 50 X 1,3</t>
         </is>
       </c>
       <c r="C442" s="2" t="inlineStr">
@@ -25421,10 +25421,10 @@
         </is>
       </c>
       <c r="D442" s="2" t="n">
-        <v>70</v>
+        <v>50</v>
       </c>
       <c r="E442" s="2" t="n">
-        <v>70</v>
+        <v>50</v>
       </c>
       <c r="F442" s="2" t="n">
         <v>1.3</v>
@@ -25433,7 +25433,7 @@
         <v>6.4</v>
       </c>
       <c r="H442" s="2" t="n">
-        <v>0.96454</v>
+        <v>0.6830000000000001</v>
       </c>
       <c r="I442" s="2" t="inlineStr">
         <is>
@@ -25441,35 +25441,35 @@
         </is>
       </c>
       <c r="J442" s="2" t="n">
-        <v>0</v>
+        <v>19</v>
       </c>
       <c r="K442" s="2" t="n">
-        <v>23</v>
+        <v>67</v>
       </c>
       <c r="L442" s="2" t="n">
-        <v>41</v>
+        <v>61</v>
       </c>
       <c r="M442" s="2" t="n">
-        <v>64</v>
-      </c>
-      <c r="N442" s="6" t="inlineStr">
-        <is>
-          <t>7/10 Días</t>
+        <v>147</v>
+      </c>
+      <c r="N442" s="4" t="inlineStr">
+        <is>
+          <t>Stock</t>
         </is>
       </c>
       <c r="O442" s="2" t="n">
-        <v>6.56</v>
+        <v>4.64</v>
       </c>
     </row>
     <row r="443">
       <c r="A443" s="2" t="inlineStr">
         <is>
-          <t>NOR0032209</t>
+          <t>NOR0032207</t>
         </is>
       </c>
       <c r="B443" s="3" t="inlineStr">
         <is>
-          <t>TUBO CUADRADO 80 X 1,5</t>
+          <t>TUBO CUADRADO 60 X 1,3</t>
         </is>
       </c>
       <c r="C443" s="2" t="inlineStr">
@@ -25478,19 +25478,19 @@
         </is>
       </c>
       <c r="D443" s="2" t="n">
-        <v>80</v>
+        <v>60</v>
       </c>
       <c r="E443" s="2" t="n">
-        <v>80</v>
+        <v>60</v>
       </c>
       <c r="F443" s="2" t="n">
-        <v>1.5</v>
+        <v>1.3</v>
       </c>
       <c r="G443" s="2" t="n">
         <v>6.4</v>
       </c>
       <c r="H443" s="2" t="n">
-        <v>1.2717</v>
+        <v>0.8235</v>
       </c>
       <c r="I443" s="2" t="inlineStr">
         <is>
@@ -25498,35 +25498,35 @@
         </is>
       </c>
       <c r="J443" s="2" t="n">
-        <v>11</v>
+        <v>5</v>
       </c>
       <c r="K443" s="2" t="n">
-        <v>58</v>
+        <v>82</v>
       </c>
       <c r="L443" s="2" t="n">
-        <v>6</v>
+        <v>94</v>
       </c>
       <c r="M443" s="2" t="n">
-        <v>75</v>
-      </c>
-      <c r="N443" s="4" t="inlineStr">
-        <is>
-          <t>Stock</t>
+        <v>181</v>
+      </c>
+      <c r="N443" s="6" t="inlineStr">
+        <is>
+          <t>7/10 Días</t>
         </is>
       </c>
       <c r="O443" s="2" t="n">
-        <v>8.65</v>
+        <v>5.6</v>
       </c>
     </row>
     <row r="444">
       <c r="A444" s="2" t="inlineStr">
         <is>
-          <t>NOR0032210</t>
+          <t>NOR0032208</t>
         </is>
       </c>
       <c r="B444" s="3" t="inlineStr">
         <is>
-          <t>TUBO CUADRADO 100 X 1,9</t>
+          <t>TUBO CUADRADO 70 X 1,3</t>
         </is>
       </c>
       <c r="C444" s="2" t="inlineStr">
@@ -25535,19 +25535,19 @@
         </is>
       </c>
       <c r="D444" s="2" t="n">
-        <v>100</v>
+        <v>70</v>
       </c>
       <c r="E444" s="2" t="n">
-        <v>100</v>
+        <v>70</v>
       </c>
       <c r="F444" s="2" t="n">
-        <v>1.9</v>
+        <v>1.3</v>
       </c>
       <c r="G444" s="2" t="n">
-        <v>6</v>
+        <v>6.4</v>
       </c>
       <c r="H444" s="2" t="n">
-        <v>2.0142</v>
+        <v>0.96454</v>
       </c>
       <c r="I444" s="2" t="inlineStr">
         <is>
@@ -25555,35 +25555,35 @@
         </is>
       </c>
       <c r="J444" s="2" t="n">
-        <v>44</v>
+        <v>0</v>
       </c>
       <c r="K444" s="2" t="n">
-        <v>1</v>
+        <v>23</v>
       </c>
       <c r="L444" s="2" t="n">
-        <v>72</v>
+        <v>41</v>
       </c>
       <c r="M444" s="2" t="n">
-        <v>117</v>
-      </c>
-      <c r="N444" s="4" t="inlineStr">
-        <is>
-          <t>Stock</t>
+        <v>64</v>
+      </c>
+      <c r="N444" s="6" t="inlineStr">
+        <is>
+          <t>7/10 Días</t>
         </is>
       </c>
       <c r="O444" s="2" t="n">
-        <v>13.7</v>
+        <v>6.56</v>
       </c>
     </row>
     <row r="445">
       <c r="A445" s="2" t="inlineStr">
         <is>
-          <t>NOR0032210</t>
+          <t>NOR0032209</t>
         </is>
       </c>
       <c r="B445" s="3" t="inlineStr">
         <is>
-          <t>TUBO CUADRADO 100 X 1,9</t>
+          <t>TUBO CUADRADO 80 X 1,5</t>
         </is>
       </c>
       <c r="C445" s="2" t="inlineStr">
@@ -25592,19 +25592,19 @@
         </is>
       </c>
       <c r="D445" s="2" t="n">
-        <v>100</v>
+        <v>80</v>
       </c>
       <c r="E445" s="2" t="n">
-        <v>100</v>
+        <v>80</v>
       </c>
       <c r="F445" s="2" t="n">
-        <v>1.9</v>
+        <v>1.5</v>
       </c>
       <c r="G445" s="2" t="n">
         <v>6.4</v>
       </c>
       <c r="H445" s="2" t="n">
-        <v>2.0142</v>
+        <v>1.2717</v>
       </c>
       <c r="I445" s="2" t="inlineStr">
         <is>
@@ -25612,35 +25612,35 @@
         </is>
       </c>
       <c r="J445" s="2" t="n">
-        <v>0</v>
+        <v>11</v>
       </c>
       <c r="K445" s="2" t="n">
-        <v>40</v>
+        <v>58</v>
       </c>
       <c r="L445" s="2" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="M445" s="2" t="n">
-        <v>42</v>
-      </c>
-      <c r="N445" s="6" t="inlineStr">
-        <is>
-          <t>7/10 Días</t>
+        <v>75</v>
+      </c>
+      <c r="N445" s="4" t="inlineStr">
+        <is>
+          <t>Stock</t>
         </is>
       </c>
       <c r="O445" s="2" t="n">
-        <v>13.7</v>
+        <v>8.65</v>
       </c>
     </row>
     <row r="446">
       <c r="A446" s="2" t="inlineStr">
         <is>
-          <t>NOR0032211</t>
+          <t>NOR0032210</t>
         </is>
       </c>
       <c r="B446" s="3" t="inlineStr">
         <is>
-          <t>TUBO CUADRADO 35 X 1.3</t>
+          <t>TUBO CUADRADO 100 X 1,9</t>
         </is>
       </c>
       <c r="C446" s="2" t="inlineStr">
@@ -25649,19 +25649,19 @@
         </is>
       </c>
       <c r="D446" s="2" t="n">
-        <v>35</v>
+        <v>100</v>
       </c>
       <c r="E446" s="2" t="n">
-        <v>35</v>
+        <v>100</v>
       </c>
       <c r="F446" s="2" t="n">
-        <v>1.3</v>
+        <v>1.9</v>
       </c>
       <c r="G446" s="2" t="n">
-        <v>6.4</v>
+        <v>6</v>
       </c>
       <c r="H446" s="2" t="n">
-        <v>0.475</v>
+        <v>2.0142</v>
       </c>
       <c r="I446" s="2" t="inlineStr">
         <is>
@@ -25669,35 +25669,35 @@
         </is>
       </c>
       <c r="J446" s="2" t="n">
-        <v>4</v>
+        <v>44</v>
       </c>
       <c r="K446" s="2" t="n">
-        <v>81</v>
+        <v>1</v>
       </c>
       <c r="L446" s="2" t="n">
-        <v>260</v>
+        <v>72</v>
       </c>
       <c r="M446" s="2" t="n">
-        <v>345</v>
-      </c>
-      <c r="N446" s="6" t="inlineStr">
-        <is>
-          <t>7/10 Días</t>
+        <v>117</v>
+      </c>
+      <c r="N446" s="4" t="inlineStr">
+        <is>
+          <t>Stock</t>
         </is>
       </c>
       <c r="O446" s="2" t="n">
-        <v>3.23</v>
+        <v>13.7</v>
       </c>
     </row>
     <row r="447">
       <c r="A447" s="2" t="inlineStr">
         <is>
-          <t>NOR0032212</t>
+          <t>NOR0032210</t>
         </is>
       </c>
       <c r="B447" s="3" t="inlineStr">
         <is>
-          <t>TUBO CUADRADO 120 X 2</t>
+          <t>TUBO CUADRADO 100 X 1,9</t>
         </is>
       </c>
       <c r="C447" s="2" t="inlineStr">
@@ -25706,19 +25706,19 @@
         </is>
       </c>
       <c r="D447" s="2" t="n">
-        <v>120</v>
+        <v>100</v>
       </c>
       <c r="E447" s="2" t="n">
-        <v>120</v>
+        <v>100</v>
       </c>
       <c r="F447" s="2" t="n">
-        <v>2</v>
+        <v>1.9</v>
       </c>
       <c r="G447" s="2" t="n">
         <v>6.4</v>
       </c>
       <c r="H447" s="2" t="n">
-        <v>2.549</v>
+        <v>2.0142</v>
       </c>
       <c r="I447" s="2" t="inlineStr">
         <is>
@@ -25726,35 +25726,35 @@
         </is>
       </c>
       <c r="J447" s="2" t="n">
-        <v>26</v>
+        <v>0</v>
       </c>
       <c r="K447" s="2" t="n">
-        <v>50</v>
+        <v>40</v>
       </c>
       <c r="L447" s="2" t="n">
-        <v>52</v>
+        <v>2</v>
       </c>
       <c r="M447" s="2" t="n">
-        <v>128</v>
-      </c>
-      <c r="N447" s="4" t="inlineStr">
-        <is>
-          <t>Stock</t>
+        <v>42</v>
+      </c>
+      <c r="N447" s="6" t="inlineStr">
+        <is>
+          <t>7/10 Días</t>
         </is>
       </c>
       <c r="O447" s="2" t="n">
-        <v>17.33</v>
+        <v>13.7</v>
       </c>
     </row>
     <row r="448">
       <c r="A448" s="2" t="inlineStr">
         <is>
-          <t>NOR0032213</t>
+          <t>NOR0032211</t>
         </is>
       </c>
       <c r="B448" s="3" t="inlineStr">
         <is>
-          <t>TUBO CUADRADO 40 X 1.5</t>
+          <t>TUBO CUADRADO 35 X 1.3</t>
         </is>
       </c>
       <c r="C448" s="2" t="inlineStr">
@@ -25763,19 +25763,19 @@
         </is>
       </c>
       <c r="D448" s="2" t="n">
-        <v>40</v>
+        <v>35</v>
       </c>
       <c r="E448" s="2" t="n">
-        <v>40</v>
+        <v>35</v>
       </c>
       <c r="F448" s="2" t="n">
-        <v>1.5</v>
+        <v>1.3</v>
       </c>
       <c r="G448" s="2" t="n">
         <v>6.4</v>
       </c>
       <c r="H448" s="2" t="n">
-        <v>0.624</v>
+        <v>0.475</v>
       </c>
       <c r="I448" s="2" t="inlineStr">
         <is>
@@ -25783,16 +25783,16 @@
         </is>
       </c>
       <c r="J448" s="2" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="K448" s="2" t="n">
-        <v>0</v>
+        <v>81</v>
       </c>
       <c r="L448" s="2" t="n">
-        <v>37</v>
+        <v>260</v>
       </c>
       <c r="M448" s="2" t="n">
-        <v>37</v>
+        <v>345</v>
       </c>
       <c r="N448" s="6" t="inlineStr">
         <is>
@@ -25800,39 +25800,39 @@
         </is>
       </c>
       <c r="O448" s="2" t="n">
-        <v>4.24</v>
+        <v>3.23</v>
       </c>
     </row>
     <row r="449">
       <c r="A449" s="2" t="inlineStr">
         <is>
-          <t>NOR0032300</t>
+          <t>NOR0032212</t>
         </is>
       </c>
       <c r="B449" s="3" t="inlineStr">
         <is>
-          <t>RECTANGULAR 20 X 10 X 1.3</t>
+          <t>TUBO CUADRADO 120 X 2</t>
         </is>
       </c>
       <c r="C449" s="2" t="inlineStr">
         <is>
-          <t>TUBO RECTANGULAR</t>
+          <t>TUBO CUADRADO</t>
         </is>
       </c>
       <c r="D449" s="2" t="n">
-        <v>20</v>
+        <v>120</v>
       </c>
       <c r="E449" s="2" t="n">
-        <v>10</v>
+        <v>120</v>
       </c>
       <c r="F449" s="2" t="n">
-        <v>1.3</v>
+        <v>2</v>
       </c>
       <c r="G449" s="2" t="n">
         <v>6.4</v>
       </c>
       <c r="H449" s="2" t="n">
-        <v>0.16594</v>
+        <v>2.549</v>
       </c>
       <c r="I449" s="2" t="inlineStr">
         <is>
@@ -25840,16 +25840,16 @@
         </is>
       </c>
       <c r="J449" s="2" t="n">
-        <v>79</v>
+        <v>26</v>
       </c>
       <c r="K449" s="2" t="n">
-        <v>0</v>
+        <v>50</v>
       </c>
       <c r="L449" s="2" t="n">
-        <v>0</v>
+        <v>52</v>
       </c>
       <c r="M449" s="2" t="n">
-        <v>79</v>
+        <v>128</v>
       </c>
       <c r="N449" s="4" t="inlineStr">
         <is>
@@ -25857,39 +25857,39 @@
         </is>
       </c>
       <c r="O449" s="2" t="n">
-        <v>1.13</v>
+        <v>17.33</v>
       </c>
     </row>
     <row r="450">
       <c r="A450" s="2" t="inlineStr">
         <is>
-          <t>NOR0032301</t>
+          <t>NOR0032213</t>
         </is>
       </c>
       <c r="B450" s="3" t="inlineStr">
         <is>
-          <t>RECTANGULAR 30 X 15 X 1.3</t>
+          <t>TUBO CUADRADO 40 X 1.5</t>
         </is>
       </c>
       <c r="C450" s="2" t="inlineStr">
         <is>
-          <t>TUBO RECTANGULAR</t>
+          <t>TUBO CUADRADO</t>
         </is>
       </c>
       <c r="D450" s="2" t="n">
-        <v>30</v>
+        <v>40</v>
       </c>
       <c r="E450" s="2" t="n">
-        <v>15</v>
+        <v>40</v>
       </c>
       <c r="F450" s="2" t="n">
-        <v>1.3</v>
+        <v>1.5</v>
       </c>
       <c r="G450" s="2" t="n">
         <v>6.4</v>
       </c>
       <c r="H450" s="2" t="n">
-        <v>0.298</v>
+        <v>0.624</v>
       </c>
       <c r="I450" s="2" t="inlineStr">
         <is>
@@ -25897,35 +25897,35 @@
         </is>
       </c>
       <c r="J450" s="2" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="K450" s="2" t="n">
         <v>0</v>
       </c>
       <c r="L450" s="2" t="n">
-        <v>0</v>
+        <v>37</v>
       </c>
       <c r="M450" s="2" t="n">
-        <v>7</v>
-      </c>
-      <c r="N450" s="5" t="inlineStr">
-        <is>
-          <t>Sin stock</t>
+        <v>37</v>
+      </c>
+      <c r="N450" s="6" t="inlineStr">
+        <is>
+          <t>7/10 Días</t>
         </is>
       </c>
       <c r="O450" s="2" t="n">
-        <v>2.03</v>
+        <v>4.24</v>
       </c>
     </row>
     <row r="451">
       <c r="A451" s="2" t="inlineStr">
         <is>
-          <t>NOR0032302</t>
+          <t>NOR0032300</t>
         </is>
       </c>
       <c r="B451" s="3" t="inlineStr">
         <is>
-          <t>RECTANGULAR 30 x 20 X 1,2</t>
+          <t>RECTANGULAR 20 X 10 X 1.3</t>
         </is>
       </c>
       <c r="C451" s="2" t="inlineStr">
@@ -25934,19 +25934,19 @@
         </is>
       </c>
       <c r="D451" s="2" t="n">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="E451" s="2" t="n">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="F451" s="2" t="n">
-        <v>1.2</v>
+        <v>1.3</v>
       </c>
       <c r="G451" s="2" t="n">
         <v>6.4</v>
       </c>
       <c r="H451" s="2" t="n">
-        <v>0.3078</v>
+        <v>0.16594</v>
       </c>
       <c r="I451" s="2" t="inlineStr">
         <is>
@@ -25954,16 +25954,16 @@
         </is>
       </c>
       <c r="J451" s="2" t="n">
-        <v>42</v>
+        <v>79</v>
       </c>
       <c r="K451" s="2" t="n">
-        <v>118</v>
+        <v>343</v>
       </c>
       <c r="L451" s="2" t="n">
-        <v>0</v>
+        <v>498</v>
       </c>
       <c r="M451" s="2" t="n">
-        <v>160</v>
+        <v>920</v>
       </c>
       <c r="N451" s="4" t="inlineStr">
         <is>
@@ -25971,18 +25971,18 @@
         </is>
       </c>
       <c r="O451" s="2" t="n">
-        <v>2.09</v>
+        <v>1.13</v>
       </c>
     </row>
     <row r="452">
       <c r="A452" s="2" t="inlineStr">
         <is>
-          <t>NOR0032303</t>
+          <t>NOR0032301</t>
         </is>
       </c>
       <c r="B452" s="3" t="inlineStr">
         <is>
-          <t>RECTANGULAR 40 X 20 X 1,3</t>
+          <t>RECTANGULAR 30 X 15 X 1.3</t>
         </is>
       </c>
       <c r="C452" s="2" t="inlineStr">
@@ -25991,10 +25991,10 @@
         </is>
       </c>
       <c r="D452" s="2" t="n">
-        <v>40</v>
+        <v>30</v>
       </c>
       <c r="E452" s="2" t="n">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="F452" s="2" t="n">
         <v>1.3</v>
@@ -26003,7 +26003,7 @@
         <v>6.4</v>
       </c>
       <c r="H452" s="2" t="n">
-        <v>0.402</v>
+        <v>0.298</v>
       </c>
       <c r="I452" s="2" t="inlineStr">
         <is>
@@ -26011,16 +26011,16 @@
         </is>
       </c>
       <c r="J452" s="2" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="K452" s="2" t="n">
-        <v>111</v>
+        <v>309</v>
       </c>
       <c r="L452" s="2" t="n">
-        <v>180</v>
+        <v>233</v>
       </c>
       <c r="M452" s="2" t="n">
-        <v>292</v>
+        <v>549</v>
       </c>
       <c r="N452" s="6" t="inlineStr">
         <is>
@@ -26028,18 +26028,18 @@
         </is>
       </c>
       <c r="O452" s="2" t="n">
-        <v>2.73</v>
+        <v>2.03</v>
       </c>
     </row>
     <row r="453">
       <c r="A453" s="2" t="inlineStr">
         <is>
-          <t>NOR0032304</t>
+          <t>NOR0032302</t>
         </is>
       </c>
       <c r="B453" s="3" t="inlineStr">
         <is>
-          <t>RECTANGULAR 50 X 20 X 1.3</t>
+          <t>RECTANGULAR 30 x 20 X 1,2</t>
         </is>
       </c>
       <c r="C453" s="2" t="inlineStr">
@@ -26048,19 +26048,19 @@
         </is>
       </c>
       <c r="D453" s="2" t="n">
-        <v>50</v>
+        <v>30</v>
       </c>
       <c r="E453" s="2" t="n">
         <v>20</v>
       </c>
       <c r="F453" s="2" t="n">
-        <v>1.3</v>
+        <v>1.2</v>
       </c>
       <c r="G453" s="2" t="n">
         <v>6.4</v>
       </c>
       <c r="H453" s="2" t="n">
-        <v>0.474</v>
+        <v>0.3078</v>
       </c>
       <c r="I453" s="2" t="inlineStr">
         <is>
@@ -26068,16 +26068,16 @@
         </is>
       </c>
       <c r="J453" s="2" t="n">
-        <v>54</v>
+        <v>42</v>
       </c>
       <c r="K453" s="2" t="n">
-        <v>31</v>
+        <v>118</v>
       </c>
       <c r="L453" s="2" t="n">
-        <v>29</v>
+        <v>267</v>
       </c>
       <c r="M453" s="2" t="n">
-        <v>114</v>
+        <v>427</v>
       </c>
       <c r="N453" s="4" t="inlineStr">
         <is>
@@ -26085,18 +26085,18 @@
         </is>
       </c>
       <c r="O453" s="2" t="n">
-        <v>3.22</v>
+        <v>2.09</v>
       </c>
     </row>
     <row r="454">
       <c r="A454" s="2" t="inlineStr">
         <is>
-          <t>NOR0032305</t>
+          <t>NOR0032303</t>
         </is>
       </c>
       <c r="B454" s="3" t="inlineStr">
         <is>
-          <t>RECTANGULAR 60 X 20 X 1,3</t>
+          <t>RECTANGULAR 40 X 20 X 1,3</t>
         </is>
       </c>
       <c r="C454" s="2" t="inlineStr">
@@ -26105,7 +26105,7 @@
         </is>
       </c>
       <c r="D454" s="2" t="n">
-        <v>60</v>
+        <v>40</v>
       </c>
       <c r="E454" s="2" t="n">
         <v>20</v>
@@ -26117,7 +26117,7 @@
         <v>6.4</v>
       </c>
       <c r="H454" s="2" t="n">
-        <v>0.5427</v>
+        <v>0.402</v>
       </c>
       <c r="I454" s="2" t="inlineStr">
         <is>
@@ -26125,35 +26125,35 @@
         </is>
       </c>
       <c r="J454" s="2" t="n">
-        <v>98</v>
+        <v>1</v>
       </c>
       <c r="K454" s="2" t="n">
-        <v>117</v>
+        <v>111</v>
       </c>
       <c r="L454" s="2" t="n">
-        <v>83</v>
+        <v>180</v>
       </c>
       <c r="M454" s="2" t="n">
-        <v>298</v>
-      </c>
-      <c r="N454" s="4" t="inlineStr">
-        <is>
-          <t>Stock</t>
+        <v>292</v>
+      </c>
+      <c r="N454" s="6" t="inlineStr">
+        <is>
+          <t>7/10 Días</t>
         </is>
       </c>
       <c r="O454" s="2" t="n">
-        <v>3.69</v>
+        <v>2.73</v>
       </c>
     </row>
     <row r="455">
       <c r="A455" s="2" t="inlineStr">
         <is>
-          <t>NOR0032306</t>
+          <t>NOR0032304</t>
         </is>
       </c>
       <c r="B455" s="3" t="inlineStr">
         <is>
-          <t>RECTANGULAR 70 X 20 X 1.3</t>
+          <t>RECTANGULAR 50 X 20 X 1.3</t>
         </is>
       </c>
       <c r="C455" s="2" t="inlineStr">
@@ -26162,7 +26162,7 @@
         </is>
       </c>
       <c r="D455" s="2" t="n">
-        <v>70</v>
+        <v>50</v>
       </c>
       <c r="E455" s="2" t="n">
         <v>20</v>
@@ -26174,7 +26174,7 @@
         <v>6.4</v>
       </c>
       <c r="H455" s="2" t="n">
-        <v>0.6129</v>
+        <v>0.474</v>
       </c>
       <c r="I455" s="2" t="inlineStr">
         <is>
@@ -26182,16 +26182,16 @@
         </is>
       </c>
       <c r="J455" s="2" t="n">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="K455" s="2" t="n">
-        <v>82</v>
+        <v>31</v>
       </c>
       <c r="L455" s="2" t="n">
-        <v>9</v>
+        <v>29</v>
       </c>
       <c r="M455" s="2" t="n">
-        <v>144</v>
+        <v>114</v>
       </c>
       <c r="N455" s="4" t="inlineStr">
         <is>
@@ -26199,18 +26199,18 @@
         </is>
       </c>
       <c r="O455" s="2" t="n">
-        <v>4.17</v>
+        <v>3.22</v>
       </c>
     </row>
     <row r="456">
       <c r="A456" s="2" t="inlineStr">
         <is>
-          <t>NOR0032307</t>
+          <t>NOR0032305</t>
         </is>
       </c>
       <c r="B456" s="3" t="inlineStr">
         <is>
-          <t>RECTANGULAR 80 X 20 X 1.3</t>
+          <t>RECTANGULAR 60 X 20 X 1,3</t>
         </is>
       </c>
       <c r="C456" s="2" t="inlineStr">
@@ -26219,7 +26219,7 @@
         </is>
       </c>
       <c r="D456" s="2" t="n">
-        <v>80</v>
+        <v>60</v>
       </c>
       <c r="E456" s="2" t="n">
         <v>20</v>
@@ -26231,7 +26231,7 @@
         <v>6.4</v>
       </c>
       <c r="H456" s="2" t="n">
-        <v>0.6831</v>
+        <v>0.5427</v>
       </c>
       <c r="I456" s="2" t="inlineStr">
         <is>
@@ -26239,35 +26239,35 @@
         </is>
       </c>
       <c r="J456" s="2" t="n">
-        <v>1</v>
+        <v>98</v>
       </c>
       <c r="K456" s="2" t="n">
-        <v>61</v>
+        <v>117</v>
       </c>
       <c r="L456" s="2" t="n">
-        <v>95</v>
+        <v>83</v>
       </c>
       <c r="M456" s="2" t="n">
-        <v>157</v>
-      </c>
-      <c r="N456" s="6" t="inlineStr">
-        <is>
-          <t>7/10 Días</t>
+        <v>298</v>
+      </c>
+      <c r="N456" s="4" t="inlineStr">
+        <is>
+          <t>Stock</t>
         </is>
       </c>
       <c r="O456" s="2" t="n">
-        <v>4.65</v>
+        <v>3.69</v>
       </c>
     </row>
     <row r="457">
       <c r="A457" s="2" t="inlineStr">
         <is>
-          <t>NOR0032308</t>
+          <t>NOR0032306</t>
         </is>
       </c>
       <c r="B457" s="3" t="inlineStr">
         <is>
-          <t>RECTANGULAR 100 X 40 X 1.5</t>
+          <t>RECTANGULAR 70 X 20 X 1.3</t>
         </is>
       </c>
       <c r="C457" s="2" t="inlineStr">
@@ -26276,19 +26276,19 @@
         </is>
       </c>
       <c r="D457" s="2" t="n">
-        <v>100</v>
+        <v>70</v>
       </c>
       <c r="E457" s="2" t="n">
-        <v>40</v>
+        <v>20</v>
       </c>
       <c r="F457" s="2" t="n">
-        <v>1.5</v>
+        <v>1.3</v>
       </c>
       <c r="G457" s="2" t="n">
-        <v>6</v>
+        <v>6.4</v>
       </c>
       <c r="H457" s="2" t="n">
-        <v>1.1097</v>
+        <v>0.6129</v>
       </c>
       <c r="I457" s="2" t="inlineStr">
         <is>
@@ -26296,35 +26296,35 @@
         </is>
       </c>
       <c r="J457" s="2" t="n">
-        <v>0</v>
+        <v>53</v>
       </c>
       <c r="K457" s="2" t="n">
-        <v>0</v>
+        <v>82</v>
       </c>
       <c r="L457" s="2" t="n">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="M457" s="2" t="n">
-        <v>13</v>
-      </c>
-      <c r="N457" s="6" t="inlineStr">
-        <is>
-          <t>7/10 Días</t>
+        <v>144</v>
+      </c>
+      <c r="N457" s="4" t="inlineStr">
+        <is>
+          <t>Stock</t>
         </is>
       </c>
       <c r="O457" s="2" t="n">
-        <v>7.55</v>
+        <v>4.17</v>
       </c>
     </row>
     <row r="458">
       <c r="A458" s="2" t="inlineStr">
         <is>
-          <t>NOR0032308</t>
+          <t>NOR0032307</t>
         </is>
       </c>
       <c r="B458" s="3" t="inlineStr">
         <is>
-          <t>RECTANGULAR 100 X 40 X 1.5</t>
+          <t>RECTANGULAR 80 X 20 X 1.3</t>
         </is>
       </c>
       <c r="C458" s="2" t="inlineStr">
@@ -26333,19 +26333,19 @@
         </is>
       </c>
       <c r="D458" s="2" t="n">
-        <v>100</v>
+        <v>80</v>
       </c>
       <c r="E458" s="2" t="n">
-        <v>40</v>
+        <v>20</v>
       </c>
       <c r="F458" s="2" t="n">
-        <v>1.5</v>
+        <v>1.3</v>
       </c>
       <c r="G458" s="2" t="n">
         <v>6.4</v>
       </c>
       <c r="H458" s="2" t="n">
-        <v>1.1097</v>
+        <v>0.6831</v>
       </c>
       <c r="I458" s="2" t="inlineStr">
         <is>
@@ -26353,13 +26353,13 @@
         </is>
       </c>
       <c r="J458" s="2" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="K458" s="2" t="n">
-        <v>89</v>
+        <v>61</v>
       </c>
       <c r="L458" s="2" t="n">
-        <v>60</v>
+        <v>95</v>
       </c>
       <c r="M458" s="2" t="n">
         <v>157</v>
@@ -26370,18 +26370,18 @@
         </is>
       </c>
       <c r="O458" s="2" t="n">
-        <v>7.55</v>
+        <v>4.65</v>
       </c>
     </row>
     <row r="459">
       <c r="A459" s="2" t="inlineStr">
         <is>
-          <t>NOR0032309</t>
+          <t>NOR0032308</t>
         </is>
       </c>
       <c r="B459" s="3" t="inlineStr">
         <is>
-          <t>RECTANGULAR 100 X 45 X 1.7</t>
+          <t>RECTANGULAR 100 X 40 X 1.5</t>
         </is>
       </c>
       <c r="C459" s="2" t="inlineStr">
@@ -26393,16 +26393,16 @@
         <v>100</v>
       </c>
       <c r="E459" s="2" t="n">
-        <v>45</v>
+        <v>40</v>
       </c>
       <c r="F459" s="2" t="n">
-        <v>1.7</v>
+        <v>1.5</v>
       </c>
       <c r="G459" s="2" t="n">
         <v>6</v>
       </c>
       <c r="H459" s="2" t="n">
-        <v>1.528</v>
+        <v>1.1097</v>
       </c>
       <c r="I459" s="2" t="inlineStr">
         <is>
@@ -26413,32 +26413,32 @@
         <v>0</v>
       </c>
       <c r="K459" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L459" s="2" t="n">
-        <v>0</v>
+        <v>13</v>
       </c>
       <c r="M459" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="N459" s="5" t="inlineStr">
-        <is>
-          <t>Sin stock</t>
+        <v>13</v>
+      </c>
+      <c r="N459" s="6" t="inlineStr">
+        <is>
+          <t>7/10 Días</t>
         </is>
       </c>
       <c r="O459" s="2" t="n">
-        <v>10.39</v>
+        <v>7.55</v>
       </c>
     </row>
     <row r="460">
       <c r="A460" s="2" t="inlineStr">
         <is>
-          <t>NOR0032310</t>
+          <t>NOR0032308</t>
         </is>
       </c>
       <c r="B460" s="3" t="inlineStr">
         <is>
-          <t>RECTANGULAR 120 X 40 X 1.9</t>
+          <t>RECTANGULAR 100 X 40 X 1.5</t>
         </is>
       </c>
       <c r="C460" s="2" t="inlineStr">
@@ -26447,19 +26447,19 @@
         </is>
       </c>
       <c r="D460" s="2" t="n">
-        <v>120</v>
+        <v>100</v>
       </c>
       <c r="E460" s="2" t="n">
         <v>40</v>
       </c>
       <c r="F460" s="2" t="n">
-        <v>1.9</v>
+        <v>1.5</v>
       </c>
       <c r="G460" s="2" t="n">
         <v>6.4</v>
       </c>
       <c r="H460" s="2" t="n">
-        <v>1.604</v>
+        <v>1.1097</v>
       </c>
       <c r="I460" s="2" t="inlineStr">
         <is>
@@ -26467,16 +26467,16 @@
         </is>
       </c>
       <c r="J460" s="2" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="K460" s="2" t="n">
-        <v>42</v>
+        <v>89</v>
       </c>
       <c r="L460" s="2" t="n">
-        <v>23</v>
+        <v>60</v>
       </c>
       <c r="M460" s="2" t="n">
-        <v>65</v>
+        <v>157</v>
       </c>
       <c r="N460" s="6" t="inlineStr">
         <is>
@@ -26484,18 +26484,18 @@
         </is>
       </c>
       <c r="O460" s="2" t="n">
-        <v>10.91</v>
+        <v>7.55</v>
       </c>
     </row>
     <row r="461">
       <c r="A461" s="2" t="inlineStr">
         <is>
-          <t>NOR0032311</t>
+          <t>NOR0032309</t>
         </is>
       </c>
       <c r="B461" s="3" t="inlineStr">
         <is>
-          <t>RECTANGULAR 60 X 40 X 1.3</t>
+          <t>RECTANGULAR 100 X 45 X 1.7</t>
         </is>
       </c>
       <c r="C461" s="2" t="inlineStr">
@@ -26504,19 +26504,19 @@
         </is>
       </c>
       <c r="D461" s="2" t="n">
-        <v>60</v>
+        <v>100</v>
       </c>
       <c r="E461" s="2" t="n">
-        <v>40</v>
+        <v>45</v>
       </c>
       <c r="F461" s="2" t="n">
-        <v>1.3</v>
+        <v>1.7</v>
       </c>
       <c r="G461" s="2" t="n">
-        <v>6.4</v>
+        <v>6</v>
       </c>
       <c r="H461" s="2" t="n">
-        <v>0.6831</v>
+        <v>1.528</v>
       </c>
       <c r="I461" s="2" t="inlineStr">
         <is>
@@ -26524,35 +26524,35 @@
         </is>
       </c>
       <c r="J461" s="2" t="n">
-        <v>11</v>
+        <v>0</v>
       </c>
       <c r="K461" s="2" t="n">
-        <v>149</v>
+        <v>1</v>
       </c>
       <c r="L461" s="2" t="n">
-        <v>45</v>
+        <v>0</v>
       </c>
       <c r="M461" s="2" t="n">
-        <v>205</v>
-      </c>
-      <c r="N461" s="4" t="inlineStr">
-        <is>
-          <t>Stock</t>
+        <v>1</v>
+      </c>
+      <c r="N461" s="5" t="inlineStr">
+        <is>
+          <t>Sin stock</t>
         </is>
       </c>
       <c r="O461" s="2" t="n">
-        <v>4.65</v>
+        <v>10.39</v>
       </c>
     </row>
     <row r="462">
       <c r="A462" s="2" t="inlineStr">
         <is>
-          <t>NOR0032312</t>
+          <t>NOR0032310</t>
         </is>
       </c>
       <c r="B462" s="3" t="inlineStr">
         <is>
-          <t>RECTANGULAR 80 X 40 X 1.5</t>
+          <t>RECTANGULAR 120 X 40 X 1.9</t>
         </is>
       </c>
       <c r="C462" s="2" t="inlineStr">
@@ -26561,19 +26561,19 @@
         </is>
       </c>
       <c r="D462" s="2" t="n">
-        <v>80</v>
+        <v>120</v>
       </c>
       <c r="E462" s="2" t="n">
         <v>40</v>
       </c>
       <c r="F462" s="2" t="n">
-        <v>1.5</v>
+        <v>1.9</v>
       </c>
       <c r="G462" s="2" t="n">
         <v>6.4</v>
       </c>
       <c r="H462" s="2" t="n">
-        <v>0.948</v>
+        <v>1.604</v>
       </c>
       <c r="I462" s="2" t="inlineStr">
         <is>
@@ -26584,13 +26584,13 @@
         <v>0</v>
       </c>
       <c r="K462" s="2" t="n">
-        <v>124</v>
+        <v>42</v>
       </c>
       <c r="L462" s="2" t="n">
-        <v>151</v>
+        <v>23</v>
       </c>
       <c r="M462" s="2" t="n">
-        <v>275</v>
+        <v>65</v>
       </c>
       <c r="N462" s="6" t="inlineStr">
         <is>
@@ -26598,18 +26598,18 @@
         </is>
       </c>
       <c r="O462" s="2" t="n">
-        <v>6.45</v>
+        <v>10.91</v>
       </c>
     </row>
     <row r="463">
       <c r="A463" s="2" t="inlineStr">
         <is>
-          <t>NOR0032313</t>
+          <t>NOR0032311</t>
         </is>
       </c>
       <c r="B463" s="3" t="inlineStr">
         <is>
-          <t>RECTANGULAR 50 X 25 X 1.5</t>
+          <t>RECTANGULAR 60 X 40 X 1.3</t>
         </is>
       </c>
       <c r="C463" s="2" t="inlineStr">
@@ -26618,19 +26618,19 @@
         </is>
       </c>
       <c r="D463" s="2" t="n">
-        <v>50</v>
+        <v>60</v>
       </c>
       <c r="E463" s="2" t="n">
-        <v>25</v>
+        <v>40</v>
       </c>
       <c r="F463" s="2" t="n">
-        <v>1.5</v>
+        <v>1.3</v>
       </c>
       <c r="G463" s="2" t="n">
-        <v>6</v>
+        <v>6.4</v>
       </c>
       <c r="H463" s="2" t="n">
-        <v>0.583</v>
+        <v>0.6831</v>
       </c>
       <c r="I463" s="2" t="inlineStr">
         <is>
@@ -26638,35 +26638,35 @@
         </is>
       </c>
       <c r="J463" s="2" t="n">
-        <v>0</v>
+        <v>11</v>
       </c>
       <c r="K463" s="2" t="n">
-        <v>0</v>
+        <v>149</v>
       </c>
       <c r="L463" s="2" t="n">
-        <v>39</v>
+        <v>45</v>
       </c>
       <c r="M463" s="2" t="n">
-        <v>39</v>
-      </c>
-      <c r="N463" s="6" t="inlineStr">
-        <is>
-          <t>7/10 Días</t>
+        <v>205</v>
+      </c>
+      <c r="N463" s="4" t="inlineStr">
+        <is>
+          <t>Stock</t>
         </is>
       </c>
       <c r="O463" s="2" t="n">
-        <v>3.96</v>
+        <v>4.65</v>
       </c>
     </row>
     <row r="464">
       <c r="A464" s="2" t="inlineStr">
         <is>
-          <t>NOR0032313</t>
+          <t>NOR0032312</t>
         </is>
       </c>
       <c r="B464" s="3" t="inlineStr">
         <is>
-          <t>RECTANGULAR 50 X 25 X 1.5</t>
+          <t>RECTANGULAR 80 X 40 X 1.5</t>
         </is>
       </c>
       <c r="C464" s="2" t="inlineStr">
@@ -26675,10 +26675,10 @@
         </is>
       </c>
       <c r="D464" s="2" t="n">
-        <v>50</v>
+        <v>80</v>
       </c>
       <c r="E464" s="2" t="n">
-        <v>25</v>
+        <v>40</v>
       </c>
       <c r="F464" s="2" t="n">
         <v>1.5</v>
@@ -26687,7 +26687,7 @@
         <v>6.4</v>
       </c>
       <c r="H464" s="2" t="n">
-        <v>0.583</v>
+        <v>0.948</v>
       </c>
       <c r="I464" s="2" t="inlineStr">
         <is>
@@ -26695,35 +26695,35 @@
         </is>
       </c>
       <c r="J464" s="2" t="n">
-        <v>25</v>
+        <v>0</v>
       </c>
       <c r="K464" s="2" t="n">
-        <v>121</v>
+        <v>124</v>
       </c>
       <c r="L464" s="2" t="n">
-        <v>78</v>
+        <v>151</v>
       </c>
       <c r="M464" s="2" t="n">
-        <v>224</v>
-      </c>
-      <c r="N464" s="4" t="inlineStr">
-        <is>
-          <t>Stock</t>
+        <v>275</v>
+      </c>
+      <c r="N464" s="6" t="inlineStr">
+        <is>
+          <t>7/10 Días</t>
         </is>
       </c>
       <c r="O464" s="2" t="n">
-        <v>3.96</v>
+        <v>6.45</v>
       </c>
     </row>
     <row r="465">
       <c r="A465" s="2" t="inlineStr">
         <is>
-          <t>NOR0032314</t>
+          <t>NOR0032313</t>
         </is>
       </c>
       <c r="B465" s="3" t="inlineStr">
         <is>
-          <t>RECTANGULAR 60 X 10 X 1.3</t>
+          <t>RECTANGULAR 50 X 25 X 1.5</t>
         </is>
       </c>
       <c r="C465" s="2" t="inlineStr">
@@ -26732,19 +26732,19 @@
         </is>
       </c>
       <c r="D465" s="2" t="n">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="E465" s="2" t="n">
-        <v>10</v>
+        <v>25</v>
       </c>
       <c r="F465" s="2" t="n">
-        <v>1.3</v>
+        <v>1.5</v>
       </c>
       <c r="G465" s="2" t="n">
-        <v>6.4</v>
+        <v>6</v>
       </c>
       <c r="H465" s="2" t="n">
-        <v>0.473</v>
+        <v>0.583</v>
       </c>
       <c r="I465" s="2" t="inlineStr">
         <is>
@@ -26752,35 +26752,35 @@
         </is>
       </c>
       <c r="J465" s="2" t="n">
-        <v>16</v>
+        <v>0</v>
       </c>
       <c r="K465" s="2" t="n">
         <v>0</v>
       </c>
       <c r="L465" s="2" t="n">
-        <v>148</v>
+        <v>39</v>
       </c>
       <c r="M465" s="2" t="n">
-        <v>164</v>
-      </c>
-      <c r="N465" s="4" t="inlineStr">
-        <is>
-          <t>Stock</t>
+        <v>39</v>
+      </c>
+      <c r="N465" s="6" t="inlineStr">
+        <is>
+          <t>7/10 Días</t>
         </is>
       </c>
       <c r="O465" s="2" t="n">
-        <v>3.22</v>
+        <v>3.96</v>
       </c>
     </row>
     <row r="466">
       <c r="A466" s="2" t="inlineStr">
         <is>
-          <t>NOR0032315</t>
+          <t>NOR0032313</t>
         </is>
       </c>
       <c r="B466" s="3" t="inlineStr">
         <is>
-          <t>RECTANGULAR 100 X 20 X 1.5</t>
+          <t>RECTANGULAR 50 X 25 X 1.5</t>
         </is>
       </c>
       <c r="C466" s="2" t="inlineStr">
@@ -26789,10 +26789,10 @@
         </is>
       </c>
       <c r="D466" s="2" t="n">
-        <v>100</v>
+        <v>50</v>
       </c>
       <c r="E466" s="2" t="n">
-        <v>20</v>
+        <v>25</v>
       </c>
       <c r="F466" s="2" t="n">
         <v>1.5</v>
@@ -26801,7 +26801,7 @@
         <v>6.4</v>
       </c>
       <c r="H466" s="2" t="n">
-        <v>0.95118</v>
+        <v>0.583</v>
       </c>
       <c r="I466" s="2" t="inlineStr">
         <is>
@@ -26809,16 +26809,16 @@
         </is>
       </c>
       <c r="J466" s="2" t="n">
-        <v>11</v>
+        <v>25</v>
       </c>
       <c r="K466" s="2" t="n">
-        <v>0</v>
+        <v>121</v>
       </c>
       <c r="L466" s="2" t="n">
-        <v>44</v>
+        <v>78</v>
       </c>
       <c r="M466" s="2" t="n">
-        <v>55</v>
+        <v>224</v>
       </c>
       <c r="N466" s="4" t="inlineStr">
         <is>
@@ -26826,18 +26826,18 @@
         </is>
       </c>
       <c r="O466" s="2" t="n">
-        <v>6.47</v>
+        <v>3.96</v>
       </c>
     </row>
     <row r="467">
       <c r="A467" s="2" t="inlineStr">
         <is>
-          <t>NOR0032316</t>
+          <t>NOR0032314</t>
         </is>
       </c>
       <c r="B467" s="3" t="inlineStr">
         <is>
-          <t>RECTANGULAR 120 X 20 X 1.5</t>
+          <t>RECTANGULAR 60 X 10 X 1.3</t>
         </is>
       </c>
       <c r="C467" s="2" t="inlineStr">
@@ -26846,19 +26846,19 @@
         </is>
       </c>
       <c r="D467" s="2" t="n">
-        <v>120</v>
+        <v>60</v>
       </c>
       <c r="E467" s="2" t="n">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="F467" s="2" t="n">
-        <v>1.5</v>
+        <v>1.3</v>
       </c>
       <c r="G467" s="2" t="n">
         <v>6.4</v>
       </c>
       <c r="H467" s="2" t="n">
-        <v>1.114</v>
+        <v>0.473</v>
       </c>
       <c r="I467" s="2" t="inlineStr">
         <is>
@@ -26866,16 +26866,16 @@
         </is>
       </c>
       <c r="J467" s="2" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="K467" s="2" t="n">
+        <v>319</v>
+      </c>
+      <c r="L467" s="2" t="n">
         <v>148</v>
       </c>
-      <c r="L467" s="2" t="n">
-        <v>15</v>
-      </c>
       <c r="M467" s="2" t="n">
-        <v>182</v>
+        <v>483</v>
       </c>
       <c r="N467" s="4" t="inlineStr">
         <is>
@@ -26883,18 +26883,18 @@
         </is>
       </c>
       <c r="O467" s="2" t="n">
-        <v>7.58</v>
+        <v>3.22</v>
       </c>
     </row>
     <row r="468">
       <c r="A468" s="2" t="inlineStr">
         <is>
-          <t>NOR0032319</t>
+          <t>NOR0032315</t>
         </is>
       </c>
       <c r="B468" s="3" t="inlineStr">
         <is>
-          <t>RECTANGULAR 50 X 15 X 1.2</t>
+          <t>RECTANGULAR 100 X 20 X 1.5</t>
         </is>
       </c>
       <c r="C468" s="2" t="inlineStr">
@@ -26903,19 +26903,19 @@
         </is>
       </c>
       <c r="D468" s="2" t="n">
-        <v>50</v>
+        <v>100</v>
       </c>
       <c r="E468" s="2" t="n">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="F468" s="2" t="n">
-        <v>1.2</v>
+        <v>1.5</v>
       </c>
       <c r="G468" s="2" t="n">
         <v>6.4</v>
       </c>
       <c r="H468" s="2" t="n">
-        <v>0.406</v>
+        <v>0.95118</v>
       </c>
       <c r="I468" s="2" t="inlineStr">
         <is>
@@ -26923,35 +26923,35 @@
         </is>
       </c>
       <c r="J468" s="2" t="n">
-        <v>0</v>
+        <v>11</v>
       </c>
       <c r="K468" s="2" t="n">
-        <v>0</v>
+        <v>338</v>
       </c>
       <c r="L468" s="2" t="n">
-        <v>61</v>
+        <v>44</v>
       </c>
       <c r="M468" s="2" t="n">
-        <v>61</v>
-      </c>
-      <c r="N468" s="6" t="inlineStr">
-        <is>
-          <t>7/10 Días</t>
+        <v>393</v>
+      </c>
+      <c r="N468" s="4" t="inlineStr">
+        <is>
+          <t>Stock</t>
         </is>
       </c>
       <c r="O468" s="2" t="n">
-        <v>2.76</v>
+        <v>6.47</v>
       </c>
     </row>
     <row r="469">
       <c r="A469" s="2" t="inlineStr">
         <is>
-          <t>NOR0032320</t>
+          <t>NOR0032316</t>
         </is>
       </c>
       <c r="B469" s="3" t="inlineStr">
         <is>
-          <t>RECTANGULAR 120 X 40 X 1.5</t>
+          <t>RECTANGULAR 120 X 20 X 1.5</t>
         </is>
       </c>
       <c r="C469" s="2" t="inlineStr">
@@ -26963,16 +26963,16 @@
         <v>120</v>
       </c>
       <c r="E469" s="2" t="n">
-        <v>40</v>
+        <v>20</v>
       </c>
       <c r="F469" s="2" t="n">
         <v>1.5</v>
       </c>
       <c r="G469" s="2" t="n">
-        <v>6</v>
+        <v>6.4</v>
       </c>
       <c r="H469" s="2" t="n">
-        <v>1.272</v>
+        <v>1.114</v>
       </c>
       <c r="I469" s="2" t="inlineStr">
         <is>
@@ -26980,35 +26980,35 @@
         </is>
       </c>
       <c r="J469" s="2" t="n">
-        <v>0</v>
+        <v>19</v>
       </c>
       <c r="K469" s="2" t="n">
-        <v>0</v>
+        <v>148</v>
       </c>
       <c r="L469" s="2" t="n">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="M469" s="2" t="n">
-        <v>20</v>
-      </c>
-      <c r="N469" s="6" t="inlineStr">
-        <is>
-          <t>7/10 Días</t>
+        <v>182</v>
+      </c>
+      <c r="N469" s="4" t="inlineStr">
+        <is>
+          <t>Stock</t>
         </is>
       </c>
       <c r="O469" s="2" t="n">
-        <v>8.65</v>
+        <v>7.58</v>
       </c>
     </row>
     <row r="470">
       <c r="A470" s="2" t="inlineStr">
         <is>
-          <t>NOR0032320</t>
+          <t>NOR0032319</t>
         </is>
       </c>
       <c r="B470" s="3" t="inlineStr">
         <is>
-          <t>RECTANGULAR 120 X 40 X 1.5</t>
+          <t>RECTANGULAR 50 X 15 X 1.2</t>
         </is>
       </c>
       <c r="C470" s="2" t="inlineStr">
@@ -27017,19 +27017,19 @@
         </is>
       </c>
       <c r="D470" s="2" t="n">
-        <v>120</v>
+        <v>50</v>
       </c>
       <c r="E470" s="2" t="n">
-        <v>40</v>
+        <v>15</v>
       </c>
       <c r="F470" s="2" t="n">
-        <v>1.5</v>
+        <v>1.2</v>
       </c>
       <c r="G470" s="2" t="n">
         <v>6.4</v>
       </c>
       <c r="H470" s="2" t="n">
-        <v>1.272</v>
+        <v>0.406</v>
       </c>
       <c r="I470" s="2" t="inlineStr">
         <is>
@@ -27037,35 +27037,35 @@
         </is>
       </c>
       <c r="J470" s="2" t="n">
-        <v>28</v>
+        <v>0</v>
       </c>
       <c r="K470" s="2" t="n">
-        <v>0</v>
+        <v>199</v>
       </c>
       <c r="L470" s="2" t="n">
-        <v>0</v>
+        <v>61</v>
       </c>
       <c r="M470" s="2" t="n">
-        <v>28</v>
-      </c>
-      <c r="N470" s="4" t="inlineStr">
-        <is>
-          <t>Stock</t>
+        <v>260</v>
+      </c>
+      <c r="N470" s="6" t="inlineStr">
+        <is>
+          <t>7/10 Días</t>
         </is>
       </c>
       <c r="O470" s="2" t="n">
-        <v>8.65</v>
+        <v>2.76</v>
       </c>
     </row>
     <row r="471">
       <c r="A471" s="2" t="inlineStr">
         <is>
-          <t>NOR0032321</t>
+          <t>NOR0032320</t>
         </is>
       </c>
       <c r="B471" s="3" t="inlineStr">
         <is>
-          <t>RECTANGULAR 150 X 20 X 1.5</t>
+          <t>RECTANGULAR 120 X 40 X 1.5</t>
         </is>
       </c>
       <c r="C471" s="2" t="inlineStr">
@@ -27074,19 +27074,19 @@
         </is>
       </c>
       <c r="D471" s="2" t="n">
-        <v>150</v>
+        <v>120</v>
       </c>
       <c r="E471" s="2" t="n">
-        <v>20</v>
+        <v>40</v>
       </c>
       <c r="F471" s="2" t="n">
         <v>1.5</v>
       </c>
       <c r="G471" s="2" t="n">
-        <v>6.4</v>
+        <v>6</v>
       </c>
       <c r="H471" s="2" t="n">
-        <v>1.353</v>
+        <v>1.272</v>
       </c>
       <c r="I471" s="2" t="inlineStr">
         <is>
@@ -27094,35 +27094,35 @@
         </is>
       </c>
       <c r="J471" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K471" s="2" t="n">
         <v>0</v>
       </c>
       <c r="L471" s="2" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="M471" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="N471" s="5" t="inlineStr">
-        <is>
-          <t>Sin stock</t>
+        <v>20</v>
+      </c>
+      <c r="N471" s="6" t="inlineStr">
+        <is>
+          <t>7/10 Días</t>
         </is>
       </c>
       <c r="O471" s="2" t="n">
-        <v>9.199999999999999</v>
+        <v>8.65</v>
       </c>
     </row>
     <row r="472">
       <c r="A472" s="2" t="inlineStr">
         <is>
-          <t>NOR0032323</t>
+          <t>NOR0032320</t>
         </is>
       </c>
       <c r="B472" s="3" t="inlineStr">
         <is>
-          <t>RECTANGULAR 100 X 50 X 1.5</t>
+          <t>RECTANGULAR 120 X 40 X 1.5</t>
         </is>
       </c>
       <c r="C472" s="2" t="inlineStr">
@@ -27131,10 +27131,10 @@
         </is>
       </c>
       <c r="D472" s="2" t="n">
-        <v>100</v>
+        <v>120</v>
       </c>
       <c r="E472" s="2" t="n">
-        <v>50</v>
+        <v>40</v>
       </c>
       <c r="F472" s="2" t="n">
         <v>1.5</v>
@@ -27143,7 +27143,7 @@
         <v>6.4</v>
       </c>
       <c r="H472" s="2" t="n">
-        <v>1.195</v>
+        <v>1.272</v>
       </c>
       <c r="I472" s="2" t="inlineStr">
         <is>
@@ -27151,35 +27151,35 @@
         </is>
       </c>
       <c r="J472" s="2" t="n">
-        <v>0</v>
+        <v>28</v>
       </c>
       <c r="K472" s="2" t="n">
-        <v>43</v>
+        <v>0</v>
       </c>
       <c r="L472" s="2" t="n">
         <v>0</v>
       </c>
       <c r="M472" s="2" t="n">
-        <v>43</v>
-      </c>
-      <c r="N472" s="6" t="inlineStr">
-        <is>
-          <t>7/10 Días</t>
+        <v>28</v>
+      </c>
+      <c r="N472" s="4" t="inlineStr">
+        <is>
+          <t>Stock</t>
         </is>
       </c>
       <c r="O472" s="2" t="n">
-        <v>8.130000000000001</v>
+        <v>8.65</v>
       </c>
     </row>
     <row r="473">
       <c r="A473" s="2" t="inlineStr">
         <is>
-          <t>NOR0032323</t>
+          <t>NOR0032321</t>
         </is>
       </c>
       <c r="B473" s="3" t="inlineStr">
         <is>
-          <t>RECTANGULAR 100 X 50 X 1.5</t>
+          <t>RECTANGULAR 150 X 20 X 1.5</t>
         </is>
       </c>
       <c r="C473" s="2" t="inlineStr">
@@ -27188,19 +27188,19 @@
         </is>
       </c>
       <c r="D473" s="2" t="n">
-        <v>100</v>
+        <v>150</v>
       </c>
       <c r="E473" s="2" t="n">
-        <v>50</v>
+        <v>20</v>
       </c>
       <c r="F473" s="2" t="n">
         <v>1.5</v>
       </c>
       <c r="G473" s="2" t="n">
-        <v>7</v>
+        <v>6.4</v>
       </c>
       <c r="H473" s="2" t="n">
-        <v>1.195</v>
+        <v>1.353</v>
       </c>
       <c r="I473" s="2" t="inlineStr">
         <is>
@@ -27208,16 +27208,16 @@
         </is>
       </c>
       <c r="J473" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K473" s="2" t="n">
         <v>0</v>
       </c>
       <c r="L473" s="2" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="M473" s="2" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="N473" s="5" t="inlineStr">
         <is>
@@ -27225,18 +27225,18 @@
         </is>
       </c>
       <c r="O473" s="2" t="n">
-        <v>8.130000000000001</v>
+        <v>9.199999999999999</v>
       </c>
     </row>
     <row r="474">
       <c r="A474" s="2" t="inlineStr">
         <is>
-          <t>NOR0032324</t>
+          <t>NOR0032323</t>
         </is>
       </c>
       <c r="B474" s="3" t="inlineStr">
         <is>
-          <t>RECTANGULAR 100 X 60 X 1.8</t>
+          <t>RECTANGULAR 100 X 50 X 1.5</t>
         </is>
       </c>
       <c r="C474" s="2" t="inlineStr">
@@ -27248,16 +27248,16 @@
         <v>100</v>
       </c>
       <c r="E474" s="2" t="n">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="F474" s="2" t="n">
-        <v>1.8</v>
+        <v>1.5</v>
       </c>
       <c r="G474" s="2" t="n">
-        <v>6.5</v>
+        <v>6.4</v>
       </c>
       <c r="H474" s="2" t="n">
-        <v>1.526</v>
+        <v>1.195</v>
       </c>
       <c r="I474" s="2" t="inlineStr">
         <is>
@@ -27268,13 +27268,13 @@
         <v>0</v>
       </c>
       <c r="K474" s="2" t="n">
-        <v>38</v>
+        <v>43</v>
       </c>
       <c r="L474" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M474" s="2" t="n">
-        <v>39</v>
+        <v>43</v>
       </c>
       <c r="N474" s="6" t="inlineStr">
         <is>
@@ -27282,39 +27282,39 @@
         </is>
       </c>
       <c r="O474" s="2" t="n">
-        <v>10.38</v>
+        <v>8.130000000000001</v>
       </c>
     </row>
     <row r="475">
       <c r="A475" s="2" t="inlineStr">
         <is>
-          <t>NOR0032401</t>
+          <t>NOR0032323</t>
         </is>
       </c>
       <c r="B475" s="3" t="inlineStr">
         <is>
-          <t>TUBO REDONDO 16 X 1,2</t>
+          <t>RECTANGULAR 100 X 50 X 1.5</t>
         </is>
       </c>
       <c r="C475" s="2" t="inlineStr">
         <is>
-          <t>TUBO REDONDO</t>
+          <t>TUBO RECTANGULAR</t>
         </is>
       </c>
       <c r="D475" s="2" t="n">
-        <v>16</v>
+        <v>100</v>
       </c>
       <c r="E475" s="2" t="n">
-        <v>16</v>
+        <v>50</v>
       </c>
       <c r="F475" s="2" t="n">
-        <v>1.2</v>
+        <v>1.5</v>
       </c>
       <c r="G475" s="2" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="H475" s="2" t="n">
-        <v>0.162</v>
+        <v>1.195</v>
       </c>
       <c r="I475" s="2" t="inlineStr">
         <is>
@@ -27325,53 +27325,53 @@
         <v>0</v>
       </c>
       <c r="K475" s="2" t="n">
-        <v>793</v>
+        <v>0</v>
       </c>
       <c r="L475" s="2" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="M475" s="2" t="n">
-        <v>793</v>
-      </c>
-      <c r="N475" s="6" t="inlineStr">
-        <is>
-          <t>7/10 Días</t>
+        <v>4</v>
+      </c>
+      <c r="N475" s="5" t="inlineStr">
+        <is>
+          <t>Sin stock</t>
         </is>
       </c>
       <c r="O475" s="2" t="n">
-        <v>1.1</v>
+        <v>8.130000000000001</v>
       </c>
     </row>
     <row r="476">
       <c r="A476" s="2" t="inlineStr">
         <is>
-          <t>NOR0032401</t>
+          <t>NOR0032324</t>
         </is>
       </c>
       <c r="B476" s="3" t="inlineStr">
         <is>
-          <t>TUBO REDONDO 16 X 1,2</t>
+          <t>RECTANGULAR 100 X 60 X 1.8</t>
         </is>
       </c>
       <c r="C476" s="2" t="inlineStr">
         <is>
-          <t>TUBO REDONDO</t>
+          <t>TUBO RECTANGULAR</t>
         </is>
       </c>
       <c r="D476" s="2" t="n">
-        <v>16</v>
+        <v>100</v>
       </c>
       <c r="E476" s="2" t="n">
-        <v>16</v>
+        <v>60</v>
       </c>
       <c r="F476" s="2" t="n">
-        <v>1.2</v>
+        <v>1.8</v>
       </c>
       <c r="G476" s="2" t="n">
-        <v>6.4</v>
+        <v>6.5</v>
       </c>
       <c r="H476" s="2" t="n">
-        <v>0.162</v>
+        <v>1.526</v>
       </c>
       <c r="I476" s="2" t="inlineStr">
         <is>
@@ -27379,35 +27379,35 @@
         </is>
       </c>
       <c r="J476" s="2" t="n">
-        <v>29</v>
+        <v>0</v>
       </c>
       <c r="K476" s="2" t="n">
-        <v>0</v>
+        <v>38</v>
       </c>
       <c r="L476" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M476" s="2" t="n">
-        <v>29</v>
-      </c>
-      <c r="N476" s="4" t="inlineStr">
-        <is>
-          <t>Stock</t>
+        <v>39</v>
+      </c>
+      <c r="N476" s="6" t="inlineStr">
+        <is>
+          <t>7/10 Días</t>
         </is>
       </c>
       <c r="O476" s="2" t="n">
-        <v>1.1</v>
+        <v>10.38</v>
       </c>
     </row>
     <row r="477">
       <c r="A477" s="2" t="inlineStr">
         <is>
-          <t>NOR0032403</t>
+          <t>NOR0032401</t>
         </is>
       </c>
       <c r="B477" s="3" t="inlineStr">
         <is>
-          <t>TUBO REDONDO 20 X 1.2</t>
+          <t>TUBO REDONDO 16 X 1,2</t>
         </is>
       </c>
       <c r="C477" s="2" t="inlineStr">
@@ -27416,10 +27416,10 @@
         </is>
       </c>
       <c r="D477" s="2" t="n">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="E477" s="2" t="n">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="F477" s="2" t="n">
         <v>1.2</v>
@@ -27428,7 +27428,7 @@
         <v>6</v>
       </c>
       <c r="H477" s="2" t="n">
-        <v>0.1915</v>
+        <v>0.162</v>
       </c>
       <c r="I477" s="2" t="inlineStr">
         <is>
@@ -27439,13 +27439,13 @@
         <v>0</v>
       </c>
       <c r="K477" s="2" t="n">
-        <v>0</v>
+        <v>793</v>
       </c>
       <c r="L477" s="2" t="n">
-        <v>238</v>
+        <v>0</v>
       </c>
       <c r="M477" s="2" t="n">
-        <v>238</v>
+        <v>793</v>
       </c>
       <c r="N477" s="6" t="inlineStr">
         <is>
@@ -27453,18 +27453,18 @@
         </is>
       </c>
       <c r="O477" s="2" t="n">
-        <v>1.3</v>
+        <v>1.1</v>
       </c>
     </row>
     <row r="478">
       <c r="A478" s="2" t="inlineStr">
         <is>
-          <t>NOR0032403</t>
+          <t>NOR0032401</t>
         </is>
       </c>
       <c r="B478" s="3" t="inlineStr">
         <is>
-          <t>TUBO REDONDO 20 X 1.2</t>
+          <t>TUBO REDONDO 16 X 1,2</t>
         </is>
       </c>
       <c r="C478" s="2" t="inlineStr">
@@ -27473,10 +27473,10 @@
         </is>
       </c>
       <c r="D478" s="2" t="n">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="E478" s="2" t="n">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="F478" s="2" t="n">
         <v>1.2</v>
@@ -27485,7 +27485,7 @@
         <v>6.4</v>
       </c>
       <c r="H478" s="2" t="n">
-        <v>0.1915</v>
+        <v>0.162</v>
       </c>
       <c r="I478" s="2" t="inlineStr">
         <is>
@@ -27493,16 +27493,16 @@
         </is>
       </c>
       <c r="J478" s="2" t="n">
-        <v>117</v>
+        <v>29</v>
       </c>
       <c r="K478" s="2" t="n">
-        <v>37</v>
+        <v>0</v>
       </c>
       <c r="L478" s="2" t="n">
-        <v>330</v>
+        <v>0</v>
       </c>
       <c r="M478" s="2" t="n">
-        <v>484</v>
+        <v>29</v>
       </c>
       <c r="N478" s="4" t="inlineStr">
         <is>
@@ -27510,18 +27510,18 @@
         </is>
       </c>
       <c r="O478" s="2" t="n">
-        <v>1.3</v>
+        <v>1.1</v>
       </c>
     </row>
     <row r="479">
       <c r="A479" s="2" t="inlineStr">
         <is>
-          <t>NOR0032405</t>
+          <t>NOR0032403</t>
         </is>
       </c>
       <c r="B479" s="3" t="inlineStr">
         <is>
-          <t>TUBO REDONDO 30 X 1,2</t>
+          <t>TUBO REDONDO 20 X 1.2</t>
         </is>
       </c>
       <c r="C479" s="2" t="inlineStr">
@@ -27530,19 +27530,19 @@
         </is>
       </c>
       <c r="D479" s="2" t="n">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="E479" s="2" t="n">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="F479" s="2" t="n">
         <v>1.2</v>
       </c>
       <c r="G479" s="2" t="n">
-        <v>6.4</v>
+        <v>6</v>
       </c>
       <c r="H479" s="2" t="n">
-        <v>0.2945</v>
+        <v>0.1915</v>
       </c>
       <c r="I479" s="2" t="inlineStr">
         <is>
@@ -27553,13 +27553,13 @@
         <v>0</v>
       </c>
       <c r="K479" s="2" t="n">
-        <v>120</v>
+        <v>0</v>
       </c>
       <c r="L479" s="2" t="n">
-        <v>23</v>
+        <v>238</v>
       </c>
       <c r="M479" s="2" t="n">
-        <v>143</v>
+        <v>238</v>
       </c>
       <c r="N479" s="6" t="inlineStr">
         <is>
@@ -27567,18 +27567,18 @@
         </is>
       </c>
       <c r="O479" s="2" t="n">
-        <v>2</v>
+        <v>1.3</v>
       </c>
     </row>
     <row r="480">
       <c r="A480" s="2" t="inlineStr">
         <is>
-          <t>NOR0032406</t>
+          <t>NOR0032403</t>
         </is>
       </c>
       <c r="B480" s="3" t="inlineStr">
         <is>
-          <t>TUBO REDONDO 40 X 1,3</t>
+          <t>TUBO REDONDO 20 X 1.2</t>
         </is>
       </c>
       <c r="C480" s="2" t="inlineStr">
@@ -27587,19 +27587,19 @@
         </is>
       </c>
       <c r="D480" s="2" t="n">
-        <v>40</v>
+        <v>20</v>
       </c>
       <c r="E480" s="2" t="n">
-        <v>40</v>
+        <v>20</v>
       </c>
       <c r="F480" s="2" t="n">
-        <v>1.3</v>
+        <v>1.2</v>
       </c>
       <c r="G480" s="2" t="n">
         <v>6.4</v>
       </c>
       <c r="H480" s="2" t="n">
-        <v>0.427</v>
+        <v>0.1915</v>
       </c>
       <c r="I480" s="2" t="inlineStr">
         <is>
@@ -27607,35 +27607,35 @@
         </is>
       </c>
       <c r="J480" s="2" t="n">
-        <v>3</v>
+        <v>117</v>
       </c>
       <c r="K480" s="2" t="n">
-        <v>0</v>
+        <v>37</v>
       </c>
       <c r="L480" s="2" t="n">
-        <v>50</v>
+        <v>330</v>
       </c>
       <c r="M480" s="2" t="n">
-        <v>53</v>
-      </c>
-      <c r="N480" s="6" t="inlineStr">
-        <is>
-          <t>7/10 Días</t>
+        <v>484</v>
+      </c>
+      <c r="N480" s="4" t="inlineStr">
+        <is>
+          <t>Stock</t>
         </is>
       </c>
       <c r="O480" s="2" t="n">
-        <v>2.9</v>
+        <v>1.3</v>
       </c>
     </row>
     <row r="481">
       <c r="A481" s="2" t="inlineStr">
         <is>
-          <t>NOR0032407</t>
+          <t>NOR0032405</t>
         </is>
       </c>
       <c r="B481" s="3" t="inlineStr">
         <is>
-          <t>TUBO REDONDO 50 X 1,5</t>
+          <t>TUBO REDONDO 30 X 1,2</t>
         </is>
       </c>
       <c r="C481" s="2" t="inlineStr">
@@ -27644,19 +27644,19 @@
         </is>
       </c>
       <c r="D481" s="2" t="n">
-        <v>50</v>
+        <v>30</v>
       </c>
       <c r="E481" s="2" t="n">
-        <v>50</v>
+        <v>30</v>
       </c>
       <c r="F481" s="2" t="n">
-        <v>1.5</v>
+        <v>1.2</v>
       </c>
       <c r="G481" s="2" t="n">
         <v>6.4</v>
       </c>
       <c r="H481" s="2" t="n">
-        <v>0.6185</v>
+        <v>0.2945</v>
       </c>
       <c r="I481" s="2" t="inlineStr">
         <is>
@@ -27664,16 +27664,16 @@
         </is>
       </c>
       <c r="J481" s="2" t="n">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="K481" s="2" t="n">
-        <v>33</v>
+        <v>120</v>
       </c>
       <c r="L481" s="2" t="n">
-        <v>0</v>
+        <v>23</v>
       </c>
       <c r="M481" s="2" t="n">
-        <v>41</v>
+        <v>143</v>
       </c>
       <c r="N481" s="6" t="inlineStr">
         <is>
@@ -27681,18 +27681,18 @@
         </is>
       </c>
       <c r="O481" s="2" t="n">
-        <v>4.21</v>
+        <v>2</v>
       </c>
     </row>
     <row r="482">
       <c r="A482" s="2" t="inlineStr">
         <is>
-          <t>NOR0032408</t>
+          <t>NOR0032406</t>
         </is>
       </c>
       <c r="B482" s="3" t="inlineStr">
         <is>
-          <t>TUBO REDONDO 60 X 1,4</t>
+          <t>TUBO REDONDO 40 X 1,3</t>
         </is>
       </c>
       <c r="C482" s="2" t="inlineStr">
@@ -27701,19 +27701,19 @@
         </is>
       </c>
       <c r="D482" s="2" t="n">
-        <v>60</v>
+        <v>40</v>
       </c>
       <c r="E482" s="2" t="n">
-        <v>60</v>
+        <v>40</v>
       </c>
       <c r="F482" s="2" t="n">
-        <v>1.4</v>
+        <v>1.3</v>
       </c>
       <c r="G482" s="2" t="n">
-        <v>6</v>
+        <v>6.4</v>
       </c>
       <c r="H482" s="2" t="n">
-        <v>0.6966</v>
+        <v>0.427</v>
       </c>
       <c r="I482" s="2" t="inlineStr">
         <is>
@@ -27721,35 +27721,35 @@
         </is>
       </c>
       <c r="J482" s="2" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="K482" s="2" t="n">
-        <v>1</v>
+        <v>195</v>
       </c>
       <c r="L482" s="2" t="n">
-        <v>0</v>
+        <v>50</v>
       </c>
       <c r="M482" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="N482" s="5" t="inlineStr">
-        <is>
-          <t>Sin stock</t>
+        <v>248</v>
+      </c>
+      <c r="N482" s="6" t="inlineStr">
+        <is>
+          <t>7/10 Días</t>
         </is>
       </c>
       <c r="O482" s="2" t="n">
-        <v>4.74</v>
+        <v>2.9</v>
       </c>
     </row>
     <row r="483">
       <c r="A483" s="2" t="inlineStr">
         <is>
-          <t>NOR0032408</t>
+          <t>NOR0032407</t>
         </is>
       </c>
       <c r="B483" s="3" t="inlineStr">
         <is>
-          <t>TUBO REDONDO 60 X 1,4</t>
+          <t>TUBO REDONDO 50 X 1,5</t>
         </is>
       </c>
       <c r="C483" s="2" t="inlineStr">
@@ -27758,19 +27758,19 @@
         </is>
       </c>
       <c r="D483" s="2" t="n">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="E483" s="2" t="n">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="F483" s="2" t="n">
-        <v>1.4</v>
+        <v>1.5</v>
       </c>
       <c r="G483" s="2" t="n">
         <v>6.4</v>
       </c>
       <c r="H483" s="2" t="n">
-        <v>0.6966</v>
+        <v>0.6185</v>
       </c>
       <c r="I483" s="2" t="inlineStr">
         <is>
@@ -27778,16 +27778,16 @@
         </is>
       </c>
       <c r="J483" s="2" t="n">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="K483" s="2" t="n">
-        <v>18</v>
+        <v>33</v>
       </c>
       <c r="L483" s="2" t="n">
-        <v>46</v>
+        <v>0</v>
       </c>
       <c r="M483" s="2" t="n">
-        <v>66</v>
+        <v>41</v>
       </c>
       <c r="N483" s="6" t="inlineStr">
         <is>
@@ -27795,18 +27795,18 @@
         </is>
       </c>
       <c r="O483" s="2" t="n">
-        <v>4.74</v>
+        <v>4.21</v>
       </c>
     </row>
     <row r="484">
       <c r="A484" s="2" t="inlineStr">
         <is>
-          <t>NOR0032409</t>
+          <t>NOR0032408</t>
         </is>
       </c>
       <c r="B484" s="3" t="inlineStr">
         <is>
-          <t>TUBO REDONDO 80 X 1.6</t>
+          <t>TUBO REDONDO 60 X 1,4</t>
         </is>
       </c>
       <c r="C484" s="2" t="inlineStr">
@@ -27815,19 +27815,19 @@
         </is>
       </c>
       <c r="D484" s="2" t="n">
-        <v>80</v>
+        <v>60</v>
       </c>
       <c r="E484" s="2" t="n">
-        <v>80</v>
+        <v>60</v>
       </c>
       <c r="F484" s="2" t="n">
-        <v>1.6</v>
+        <v>1.4</v>
       </c>
       <c r="G484" s="2" t="n">
         <v>6</v>
       </c>
       <c r="H484" s="2" t="n">
-        <v>1.065</v>
+        <v>0.6966</v>
       </c>
       <c r="I484" s="2" t="inlineStr">
         <is>
@@ -27838,13 +27838,13 @@
         <v>0</v>
       </c>
       <c r="K484" s="2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="L484" s="2" t="n">
         <v>0</v>
       </c>
       <c r="M484" s="2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="N484" s="5" t="inlineStr">
         <is>
@@ -27852,18 +27852,18 @@
         </is>
       </c>
       <c r="O484" s="2" t="n">
-        <v>7.24</v>
+        <v>4.74</v>
       </c>
     </row>
     <row r="485">
       <c r="A485" s="2" t="inlineStr">
         <is>
-          <t>NOR0032409</t>
+          <t>NOR0032408</t>
         </is>
       </c>
       <c r="B485" s="3" t="inlineStr">
         <is>
-          <t>TUBO REDONDO 80 X 1.6</t>
+          <t>TUBO REDONDO 60 X 1,4</t>
         </is>
       </c>
       <c r="C485" s="2" t="inlineStr">
@@ -27872,19 +27872,19 @@
         </is>
       </c>
       <c r="D485" s="2" t="n">
-        <v>80</v>
+        <v>60</v>
       </c>
       <c r="E485" s="2" t="n">
-        <v>80</v>
+        <v>60</v>
       </c>
       <c r="F485" s="2" t="n">
-        <v>1.6</v>
+        <v>1.4</v>
       </c>
       <c r="G485" s="2" t="n">
         <v>6.4</v>
       </c>
       <c r="H485" s="2" t="n">
-        <v>1.065</v>
+        <v>0.6966</v>
       </c>
       <c r="I485" s="2" t="inlineStr">
         <is>
@@ -27892,16 +27892,16 @@
         </is>
       </c>
       <c r="J485" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K485" s="2" t="n">
-        <v>110</v>
+        <v>18</v>
       </c>
       <c r="L485" s="2" t="n">
-        <v>26</v>
+        <v>46</v>
       </c>
       <c r="M485" s="2" t="n">
-        <v>136</v>
+        <v>66</v>
       </c>
       <c r="N485" s="6" t="inlineStr">
         <is>
@@ -27909,18 +27909,18 @@
         </is>
       </c>
       <c r="O485" s="2" t="n">
-        <v>7.24</v>
+        <v>4.74</v>
       </c>
     </row>
     <row r="486">
       <c r="A486" s="2" t="inlineStr">
         <is>
-          <t>NOR0032410</t>
+          <t>NOR0032409</t>
         </is>
       </c>
       <c r="B486" s="3" t="inlineStr">
         <is>
-          <t>TUBO REDONDO 70 X 1,5</t>
+          <t>TUBO REDONDO 80 X 1.6</t>
         </is>
       </c>
       <c r="C486" s="2" t="inlineStr">
@@ -27929,19 +27929,19 @@
         </is>
       </c>
       <c r="D486" s="2" t="n">
-        <v>70</v>
+        <v>80</v>
       </c>
       <c r="E486" s="2" t="n">
-        <v>70</v>
+        <v>80</v>
       </c>
       <c r="F486" s="2" t="n">
-        <v>1.5</v>
+        <v>1.6</v>
       </c>
       <c r="G486" s="2" t="n">
-        <v>6.4</v>
+        <v>6</v>
       </c>
       <c r="H486" s="2" t="n">
-        <v>0.8721</v>
+        <v>1.065</v>
       </c>
       <c r="I486" s="2" t="inlineStr">
         <is>
@@ -27949,85 +27949,256 @@
         </is>
       </c>
       <c r="J486" s="2" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="K486" s="2" t="n">
-        <v>30</v>
+        <v>3</v>
       </c>
       <c r="L486" s="2" t="n">
-        <v>30</v>
+        <v>0</v>
       </c>
       <c r="M486" s="2" t="n">
-        <v>67</v>
-      </c>
-      <c r="N486" s="6" t="inlineStr">
-        <is>
-          <t>7/10 Días</t>
+        <v>3</v>
+      </c>
+      <c r="N486" s="5" t="inlineStr">
+        <is>
+          <t>Sin stock</t>
         </is>
       </c>
       <c r="O486" s="2" t="n">
-        <v>5.93</v>
+        <v>7.24</v>
       </c>
     </row>
     <row r="487">
       <c r="A487" s="2" t="inlineStr">
         <is>
+          <t>NOR0032409</t>
+        </is>
+      </c>
+      <c r="B487" s="3" t="inlineStr">
+        <is>
+          <t>TUBO REDONDO 80 X 1.6</t>
+        </is>
+      </c>
+      <c r="C487" s="2" t="inlineStr">
+        <is>
+          <t>TUBO REDONDO</t>
+        </is>
+      </c>
+      <c r="D487" s="2" t="n">
+        <v>80</v>
+      </c>
+      <c r="E487" s="2" t="n">
+        <v>80</v>
+      </c>
+      <c r="F487" s="2" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="G487" s="2" t="n">
+        <v>6.4</v>
+      </c>
+      <c r="H487" s="2" t="n">
+        <v>1.065</v>
+      </c>
+      <c r="I487" s="2" t="inlineStr">
+        <is>
+          <t>BRUTO</t>
+        </is>
+      </c>
+      <c r="J487" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K487" s="2" t="n">
+        <v>110</v>
+      </c>
+      <c r="L487" s="2" t="n">
+        <v>26</v>
+      </c>
+      <c r="M487" s="2" t="n">
+        <v>136</v>
+      </c>
+      <c r="N487" s="6" t="inlineStr">
+        <is>
+          <t>7/10 Días</t>
+        </is>
+      </c>
+      <c r="O487" s="2" t="n">
+        <v>7.24</v>
+      </c>
+    </row>
+    <row r="488">
+      <c r="A488" s="2" t="inlineStr">
+        <is>
+          <t>NOR0032410</t>
+        </is>
+      </c>
+      <c r="B488" s="3" t="inlineStr">
+        <is>
+          <t>TUBO REDONDO 70 X 1,5</t>
+        </is>
+      </c>
+      <c r="C488" s="2" t="inlineStr">
+        <is>
+          <t>TUBO REDONDO</t>
+        </is>
+      </c>
+      <c r="D488" s="2" t="n">
+        <v>70</v>
+      </c>
+      <c r="E488" s="2" t="n">
+        <v>70</v>
+      </c>
+      <c r="F488" s="2" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="G488" s="2" t="n">
+        <v>6.4</v>
+      </c>
+      <c r="H488" s="2" t="n">
+        <v>0.8721</v>
+      </c>
+      <c r="I488" s="2" t="inlineStr">
+        <is>
+          <t>BRUTO</t>
+        </is>
+      </c>
+      <c r="J488" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="K488" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="L488" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="M488" s="2" t="n">
+        <v>67</v>
+      </c>
+      <c r="N488" s="6" t="inlineStr">
+        <is>
+          <t>7/10 Días</t>
+        </is>
+      </c>
+      <c r="O488" s="2" t="n">
+        <v>5.93</v>
+      </c>
+    </row>
+    <row r="489">
+      <c r="A489" s="2" t="inlineStr">
+        <is>
           <t>NOR0032414</t>
         </is>
       </c>
-      <c r="B487" s="3" t="inlineStr">
+      <c r="B489" s="3" t="inlineStr">
         <is>
           <t>T - 30 X 30 X 1.5</t>
         </is>
       </c>
-      <c r="C487" s="2" t="inlineStr">
+      <c r="C489" s="2" t="inlineStr">
         <is>
           <t>PERFIL T</t>
         </is>
       </c>
-      <c r="D487" s="2" t="n">
+      <c r="D489" s="2" t="n">
         <v>30</v>
       </c>
-      <c r="E487" s="2" t="n">
+      <c r="E489" s="2" t="n">
         <v>30</v>
       </c>
-      <c r="F487" s="2" t="n">
+      <c r="F489" s="2" t="n">
         <v>1.5</v>
       </c>
-      <c r="G487" s="2" t="n">
-        <v>6</v>
-      </c>
-      <c r="H487" s="2" t="n">
+      <c r="G489" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="H489" s="2" t="n">
         <v>0.237</v>
       </c>
-      <c r="I487" s="2" t="inlineStr">
-        <is>
-          <t>BRUTO</t>
-        </is>
-      </c>
-      <c r="J487" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="K487" s="2" t="n">
+      <c r="I489" s="2" t="inlineStr">
+        <is>
+          <t>BRUTO</t>
+        </is>
+      </c>
+      <c r="J489" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K489" s="2" t="n">
         <v>19</v>
       </c>
-      <c r="L487" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="M487" s="2" t="n">
+      <c r="L489" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M489" s="2" t="n">
         <v>19</v>
       </c>
-      <c r="N487" s="6" t="inlineStr">
+      <c r="N489" s="6" t="inlineStr">
         <is>
           <t>7/10 Días</t>
         </is>
       </c>
-      <c r="O487" s="2" t="n">
+      <c r="O489" s="2" t="n">
         <v>1.61</v>
       </c>
     </row>
+    <row r="490">
+      <c r="A490" s="2" t="inlineStr">
+        <is>
+          <t>NOR0032414</t>
+        </is>
+      </c>
+      <c r="B490" s="3" t="inlineStr">
+        <is>
+          <t>T - 30 X 30 X 1.5</t>
+        </is>
+      </c>
+      <c r="C490" s="2" t="inlineStr">
+        <is>
+          <t>PERFIL T</t>
+        </is>
+      </c>
+      <c r="D490" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="E490" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="F490" s="2" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="G490" s="2" t="n">
+        <v>6.4</v>
+      </c>
+      <c r="H490" s="2" t="n">
+        <v>0.237</v>
+      </c>
+      <c r="I490" s="2" t="inlineStr">
+        <is>
+          <t>BRUTO</t>
+        </is>
+      </c>
+      <c r="J490" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K490" s="2" t="n">
+        <v>168</v>
+      </c>
+      <c r="L490" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M490" s="2" t="n">
+        <v>168</v>
+      </c>
+      <c r="N490" s="6" t="inlineStr">
+        <is>
+          <t>7/10 Días</t>
+        </is>
+      </c>
+      <c r="O490" s="2" t="n">
+        <v>1.61</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:O487"/>
+  <autoFilter ref="A1:O490"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update inventario_expandido.xlsx — 03/07/2026
</commit_message>
<xml_diff>
--- a/inventario_expandido.xlsx
+++ b/inventario_expandido.xlsx
@@ -618,13 +618,13 @@
         <v>45</v>
       </c>
       <c r="K2" s="2" t="n">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="L2" s="2" t="n">
         <v>25</v>
       </c>
       <c r="M2" s="2" t="n">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="N2" s="4" t="inlineStr">
         <is>
@@ -1547,13 +1547,13 @@
         <v>99</v>
       </c>
       <c r="K19" s="2" t="n">
-        <v>128</v>
+        <v>125</v>
       </c>
       <c r="L19" s="2" t="n">
         <v>87</v>
       </c>
       <c r="M19" s="2" t="n">
-        <v>314</v>
+        <v>311</v>
       </c>
       <c r="N19" s="4" t="inlineStr">
         <is>
@@ -1600,13 +1600,13 @@
         <v>31</v>
       </c>
       <c r="K20" s="2" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="L20" s="2" t="n">
         <v>88</v>
       </c>
       <c r="M20" s="2" t="n">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="N20" s="4" t="inlineStr">
         <is>
@@ -1650,16 +1650,16 @@
         </is>
       </c>
       <c r="J21" s="2" t="n">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="K21" s="2" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="L21" s="2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="M21" s="2" t="n">
-        <v>40</v>
+        <v>33</v>
       </c>
       <c r="N21" s="4" t="inlineStr">
         <is>
@@ -1809,16 +1809,16 @@
         </is>
       </c>
       <c r="J24" s="2" t="n">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="K24" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L24" s="2" t="n">
         <v>47</v>
       </c>
-      <c r="L24" s="2" t="n">
-        <v>0</v>
-      </c>
       <c r="M24" s="2" t="n">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="N24" s="4" t="inlineStr">
         <is>
@@ -1971,13 +1971,13 @@
         <v>320</v>
       </c>
       <c r="K27" s="2" t="n">
-        <v>63</v>
+        <v>13</v>
       </c>
       <c r="L27" s="2" t="n">
         <v>324</v>
       </c>
       <c r="M27" s="2" t="n">
-        <v>707</v>
+        <v>657</v>
       </c>
       <c r="N27" s="4" t="inlineStr">
         <is>
@@ -2132,13 +2132,13 @@
         <v>318</v>
       </c>
       <c r="K30" s="2" t="n">
-        <v>437</v>
+        <v>399</v>
       </c>
       <c r="L30" s="2" t="n">
         <v>526</v>
       </c>
       <c r="M30" s="2" t="n">
-        <v>1281</v>
+        <v>1243</v>
       </c>
       <c r="N30" s="4" t="inlineStr">
         <is>
@@ -2297,13 +2297,13 @@
         <v>349</v>
       </c>
       <c r="K33" s="2" t="n">
-        <v>174</v>
+        <v>170</v>
       </c>
       <c r="L33" s="2" t="n">
         <v>183</v>
       </c>
       <c r="M33" s="2" t="n">
-        <v>706</v>
+        <v>702</v>
       </c>
       <c r="N33" s="4" t="inlineStr">
         <is>
@@ -2404,7 +2404,7 @@
         </is>
       </c>
       <c r="J35" s="2" t="n">
-        <v>123</v>
+        <v>99</v>
       </c>
       <c r="K35" s="2" t="n">
         <v>79</v>
@@ -2413,7 +2413,7 @@
         <v>1</v>
       </c>
       <c r="M35" s="2" t="n">
-        <v>203</v>
+        <v>179</v>
       </c>
       <c r="N35" s="4" t="inlineStr">
         <is>
@@ -2682,13 +2682,13 @@
         <v>15</v>
       </c>
       <c r="K40" s="2" t="n">
-        <v>342</v>
+        <v>341</v>
       </c>
       <c r="L40" s="2" t="n">
         <v>17</v>
       </c>
       <c r="M40" s="2" t="n">
-        <v>374</v>
+        <v>373</v>
       </c>
       <c r="N40" s="4" t="inlineStr">
         <is>
@@ -3064,7 +3064,7 @@
         </is>
       </c>
       <c r="J47" s="2" t="n">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="K47" s="2" t="n">
         <v>201</v>
@@ -3073,7 +3073,7 @@
         <v>118</v>
       </c>
       <c r="M47" s="2" t="n">
-        <v>385</v>
+        <v>383</v>
       </c>
       <c r="N47" s="4" t="inlineStr">
         <is>
@@ -3510,10 +3510,10 @@
         <v>78</v>
       </c>
       <c r="L55" s="2" t="n">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="M55" s="2" t="n">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="N55" s="4" t="inlineStr">
         <is>
@@ -3617,13 +3617,13 @@
         <v>0</v>
       </c>
       <c r="K57" s="2" t="n">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="L57" s="2" t="n">
         <v>0</v>
       </c>
       <c r="M57" s="2" t="n">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="N57" s="6" t="inlineStr">
         <is>
@@ -3672,13 +3672,13 @@
         <v>28</v>
       </c>
       <c r="K58" s="2" t="n">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="L58" s="2" t="n">
         <v>25</v>
       </c>
       <c r="M58" s="2" t="n">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="N58" s="4" t="inlineStr">
         <is>
@@ -3892,13 +3892,13 @@
         <v>28</v>
       </c>
       <c r="K62" s="2" t="n">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="L62" s="2" t="n">
         <v>54</v>
       </c>
       <c r="M62" s="2" t="n">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="N62" s="4" t="inlineStr">
         <is>
@@ -4497,13 +4497,13 @@
         <v>42</v>
       </c>
       <c r="K73" s="2" t="n">
-        <v>339</v>
+        <v>337</v>
       </c>
       <c r="L73" s="2" t="n">
         <v>0</v>
       </c>
       <c r="M73" s="2" t="n">
-        <v>381</v>
+        <v>379</v>
       </c>
       <c r="N73" s="4" t="inlineStr">
         <is>
@@ -4604,16 +4604,16 @@
         </is>
       </c>
       <c r="J75" s="2" t="n">
-        <v>205</v>
+        <v>151</v>
       </c>
       <c r="K75" s="2" t="n">
-        <v>0</v>
+        <v>66</v>
       </c>
       <c r="L75" s="2" t="n">
         <v>267</v>
       </c>
       <c r="M75" s="2" t="n">
-        <v>472</v>
+        <v>484</v>
       </c>
       <c r="N75" s="4" t="inlineStr">
         <is>
@@ -4717,13 +4717,13 @@
         <v>117</v>
       </c>
       <c r="K77" s="2" t="n">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="L77" s="2" t="n">
         <v>5</v>
       </c>
       <c r="M77" s="2" t="n">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="N77" s="4" t="inlineStr">
         <is>
@@ -5264,7 +5264,7 @@
         </is>
       </c>
       <c r="J87" s="2" t="n">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="K87" s="2" t="n">
         <v>42</v>
@@ -5273,7 +5273,7 @@
         <v>50</v>
       </c>
       <c r="M87" s="2" t="n">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="N87" s="4" t="inlineStr">
         <is>
@@ -6477,13 +6477,13 @@
         <v>8</v>
       </c>
       <c r="K109" s="2" t="n">
-        <v>76</v>
+        <v>60</v>
       </c>
       <c r="L109" s="2" t="n">
         <v>0</v>
       </c>
       <c r="M109" s="2" t="n">
-        <v>84</v>
+        <v>68</v>
       </c>
       <c r="N109" s="6" t="inlineStr">
         <is>
@@ -6587,13 +6587,13 @@
         <v>0</v>
       </c>
       <c r="K111" s="2" t="n">
-        <v>81</v>
+        <v>51</v>
       </c>
       <c r="L111" s="2" t="n">
         <v>0</v>
       </c>
       <c r="M111" s="2" t="n">
-        <v>81</v>
+        <v>51</v>
       </c>
       <c r="N111" s="6" t="inlineStr">
         <is>
@@ -7665,16 +7665,16 @@
         </is>
       </c>
       <c r="J130" s="2" t="n">
-        <v>132</v>
+        <v>32</v>
       </c>
       <c r="K130" s="2" t="n">
         <v>92</v>
       </c>
       <c r="L130" s="2" t="n">
-        <v>296</v>
+        <v>90</v>
       </c>
       <c r="M130" s="2" t="n">
-        <v>520</v>
+        <v>214</v>
       </c>
       <c r="N130" s="4" t="inlineStr">
         <is>
@@ -7953,13 +7953,13 @@
         <v>29</v>
       </c>
       <c r="K135" s="2" t="n">
-        <v>94</v>
+        <v>19</v>
       </c>
       <c r="L135" s="2" t="n">
         <v>187</v>
       </c>
       <c r="M135" s="2" t="n">
-        <v>310</v>
+        <v>235</v>
       </c>
       <c r="N135" s="4" t="inlineStr">
         <is>
@@ -8124,13 +8124,13 @@
         <v>53</v>
       </c>
       <c r="K138" s="2" t="n">
-        <v>458</v>
+        <v>332</v>
       </c>
       <c r="L138" s="2" t="n">
         <v>37</v>
       </c>
       <c r="M138" s="2" t="n">
-        <v>548</v>
+        <v>422</v>
       </c>
       <c r="N138" s="4" t="inlineStr">
         <is>
@@ -8520,7 +8520,7 @@
         </is>
       </c>
       <c r="J145" s="2" t="n">
-        <v>343</v>
+        <v>342</v>
       </c>
       <c r="K145" s="2" t="n">
         <v>488</v>
@@ -8529,7 +8529,7 @@
         <v>248</v>
       </c>
       <c r="M145" s="2" t="n">
-        <v>1079</v>
+        <v>1078</v>
       </c>
       <c r="N145" s="4" t="inlineStr">
         <is>
@@ -9321,13 +9321,13 @@
         <v>162</v>
       </c>
       <c r="K159" s="2" t="n">
-        <v>236</v>
+        <v>231</v>
       </c>
       <c r="L159" s="2" t="n">
         <v>166</v>
       </c>
       <c r="M159" s="2" t="n">
-        <v>564</v>
+        <v>559</v>
       </c>
       <c r="N159" s="4" t="inlineStr">
         <is>
@@ -9720,13 +9720,13 @@
         <v>112</v>
       </c>
       <c r="K166" s="2" t="n">
-        <v>609</v>
+        <v>604</v>
       </c>
       <c r="L166" s="2" t="n">
         <v>75</v>
       </c>
       <c r="M166" s="2" t="n">
-        <v>796</v>
+        <v>791</v>
       </c>
       <c r="N166" s="4" t="inlineStr">
         <is>
@@ -9780,10 +9780,10 @@
         <v>148</v>
       </c>
       <c r="L167" s="2" t="n">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="M167" s="2" t="n">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="N167" s="4" t="inlineStr">
         <is>
@@ -9951,10 +9951,10 @@
         <v>184</v>
       </c>
       <c r="L170" s="2" t="n">
-        <v>45</v>
+        <v>32</v>
       </c>
       <c r="M170" s="2" t="n">
-        <v>486</v>
+        <v>473</v>
       </c>
       <c r="N170" s="4" t="inlineStr">
         <is>
@@ -10176,13 +10176,13 @@
         <v>71</v>
       </c>
       <c r="K174" s="2" t="n">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="L174" s="2" t="n">
         <v>373</v>
       </c>
       <c r="M174" s="2" t="n">
-        <v>494</v>
+        <v>491</v>
       </c>
       <c r="N174" s="4" t="inlineStr">
         <is>
@@ -11202,13 +11202,13 @@
         <v>192</v>
       </c>
       <c r="K192" s="2" t="n">
-        <v>144</v>
+        <v>140</v>
       </c>
       <c r="L192" s="2" t="n">
         <v>20</v>
       </c>
       <c r="M192" s="2" t="n">
-        <v>356</v>
+        <v>352</v>
       </c>
       <c r="N192" s="4" t="inlineStr">
         <is>
@@ -11313,7 +11313,7 @@
         </is>
       </c>
       <c r="J194" s="2" t="n">
-        <v>206</v>
+        <v>204</v>
       </c>
       <c r="K194" s="2" t="n">
         <v>69</v>
@@ -11322,7 +11322,7 @@
         <v>0</v>
       </c>
       <c r="M194" s="2" t="n">
-        <v>275</v>
+        <v>273</v>
       </c>
       <c r="N194" s="4" t="inlineStr">
         <is>
@@ -11715,13 +11715,13 @@
         <v>193</v>
       </c>
       <c r="K201" s="2" t="n">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="L201" s="2" t="n">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="M201" s="2" t="n">
-        <v>309</v>
+        <v>304</v>
       </c>
       <c r="N201" s="4" t="inlineStr">
         <is>
@@ -11886,13 +11886,13 @@
         <v>182</v>
       </c>
       <c r="K204" s="2" t="n">
-        <v>0</v>
+        <v>333</v>
       </c>
       <c r="L204" s="2" t="n">
         <v>238</v>
       </c>
       <c r="M204" s="2" t="n">
-        <v>420</v>
+        <v>753</v>
       </c>
       <c r="N204" s="4" t="inlineStr">
         <is>
@@ -11943,13 +11943,13 @@
         <v>80</v>
       </c>
       <c r="K205" s="2" t="n">
-        <v>302</v>
+        <v>296</v>
       </c>
       <c r="L205" s="2" t="n">
         <v>0</v>
       </c>
       <c r="M205" s="2" t="n">
-        <v>382</v>
+        <v>376</v>
       </c>
       <c r="N205" s="4" t="inlineStr">
         <is>
@@ -12225,7 +12225,7 @@
         </is>
       </c>
       <c r="J210" s="2" t="n">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="K210" s="2" t="n">
         <v>65</v>
@@ -12234,7 +12234,7 @@
         <v>54</v>
       </c>
       <c r="M210" s="2" t="n">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="N210" s="4" t="inlineStr">
         <is>
@@ -12285,13 +12285,13 @@
         <v>0</v>
       </c>
       <c r="K211" s="2" t="n">
-        <v>111</v>
+        <v>45</v>
       </c>
       <c r="L211" s="2" t="n">
         <v>0</v>
       </c>
       <c r="M211" s="2" t="n">
-        <v>111</v>
+        <v>45</v>
       </c>
       <c r="N211" s="6" t="inlineStr">
         <is>
@@ -12513,13 +12513,13 @@
         <v>1</v>
       </c>
       <c r="K215" s="2" t="n">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="L215" s="2" t="n">
         <v>0</v>
       </c>
       <c r="M215" s="2" t="n">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="N215" s="6" t="inlineStr">
         <is>
@@ -12855,13 +12855,13 @@
         <v>7</v>
       </c>
       <c r="K221" s="2" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="L221" s="2" t="n">
         <v>0</v>
       </c>
       <c r="M221" s="2" t="n">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="N221" s="6" t="inlineStr">
         <is>
@@ -13767,13 +13767,13 @@
         <v>62</v>
       </c>
       <c r="K237" s="2" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="L237" s="2" t="n">
         <v>49</v>
       </c>
       <c r="M237" s="2" t="n">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="N237" s="4" t="inlineStr">
         <is>
@@ -13992,7 +13992,7 @@
         </is>
       </c>
       <c r="J241" s="2" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="K241" s="2" t="n">
         <v>68</v>
@@ -14001,7 +14001,7 @@
         <v>0</v>
       </c>
       <c r="M241" s="2" t="n">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="N241" s="6" t="inlineStr">
         <is>
@@ -14619,16 +14619,16 @@
         </is>
       </c>
       <c r="J252" s="2" t="n">
-        <v>64</v>
+        <v>53</v>
       </c>
       <c r="K252" s="2" t="n">
         <v>0</v>
       </c>
       <c r="L252" s="2" t="n">
-        <v>222</v>
+        <v>211</v>
       </c>
       <c r="M252" s="2" t="n">
-        <v>286</v>
+        <v>264</v>
       </c>
       <c r="N252" s="4" t="inlineStr">
         <is>
@@ -14682,10 +14682,10 @@
         <v>259</v>
       </c>
       <c r="L253" s="2" t="n">
-        <v>183</v>
+        <v>181</v>
       </c>
       <c r="M253" s="2" t="n">
-        <v>638</v>
+        <v>636</v>
       </c>
       <c r="N253" s="4" t="inlineStr">
         <is>
@@ -14847,7 +14847,7 @@
         </is>
       </c>
       <c r="J256" s="2" t="n">
-        <v>101</v>
+        <v>86</v>
       </c>
       <c r="K256" s="2" t="n">
         <v>228</v>
@@ -14856,7 +14856,7 @@
         <v>295</v>
       </c>
       <c r="M256" s="2" t="n">
-        <v>624</v>
+        <v>609</v>
       </c>
       <c r="N256" s="4" t="inlineStr">
         <is>
@@ -14910,10 +14910,10 @@
         <v>204</v>
       </c>
       <c r="L257" s="2" t="n">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="M257" s="2" t="n">
-        <v>379</v>
+        <v>378</v>
       </c>
       <c r="N257" s="4" t="inlineStr">
         <is>
@@ -14964,13 +14964,13 @@
         <v>65</v>
       </c>
       <c r="K258" s="2" t="n">
-        <v>166</v>
+        <v>158</v>
       </c>
       <c r="L258" s="2" t="n">
         <v>79</v>
       </c>
       <c r="M258" s="2" t="n">
-        <v>310</v>
+        <v>302</v>
       </c>
       <c r="N258" s="4" t="inlineStr">
         <is>
@@ -15078,13 +15078,13 @@
         <v>71</v>
       </c>
       <c r="K260" s="2" t="n">
-        <v>61</v>
+        <v>51</v>
       </c>
       <c r="L260" s="2" t="n">
         <v>44</v>
       </c>
       <c r="M260" s="2" t="n">
-        <v>176</v>
+        <v>166</v>
       </c>
       <c r="N260" s="4" t="inlineStr">
         <is>
@@ -15192,13 +15192,13 @@
         <v>32</v>
       </c>
       <c r="K262" s="2" t="n">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="L262" s="2" t="n">
         <v>50</v>
       </c>
       <c r="M262" s="2" t="n">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="N262" s="4" t="inlineStr">
         <is>
@@ -15249,13 +15249,13 @@
         <v>57</v>
       </c>
       <c r="K263" s="2" t="n">
-        <v>48</v>
+        <v>42</v>
       </c>
       <c r="L263" s="2" t="n">
-        <v>142</v>
+        <v>125</v>
       </c>
       <c r="M263" s="2" t="n">
-        <v>247</v>
+        <v>224</v>
       </c>
       <c r="N263" s="4" t="inlineStr">
         <is>
@@ -15645,16 +15645,16 @@
         </is>
       </c>
       <c r="J270" s="2" t="n">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="K270" s="2" t="n">
         <v>227</v>
       </c>
       <c r="L270" s="2" t="n">
-        <v>179</v>
+        <v>166</v>
       </c>
       <c r="M270" s="2" t="n">
-        <v>458</v>
+        <v>444</v>
       </c>
       <c r="N270" s="4" t="inlineStr">
         <is>
@@ -16221,10 +16221,10 @@
         <v>511</v>
       </c>
       <c r="L280" s="2" t="n">
-        <v>54</v>
+        <v>14</v>
       </c>
       <c r="M280" s="2" t="n">
-        <v>592</v>
+        <v>552</v>
       </c>
       <c r="N280" s="4" t="inlineStr">
         <is>
@@ -16902,13 +16902,13 @@
         <v>15</v>
       </c>
       <c r="K292" s="2" t="n">
-        <v>30</v>
+        <v>19</v>
       </c>
       <c r="L292" s="2" t="n">
         <v>0</v>
       </c>
       <c r="M292" s="2" t="n">
-        <v>45</v>
+        <v>34</v>
       </c>
       <c r="N292" s="4" t="inlineStr">
         <is>
@@ -17076,10 +17076,10 @@
         <v>6</v>
       </c>
       <c r="L295" s="2" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="M295" s="2" t="n">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="N295" s="5" t="inlineStr">
         <is>
@@ -17187,13 +17187,13 @@
         <v>76</v>
       </c>
       <c r="K297" s="2" t="n">
-        <v>197</v>
+        <v>191</v>
       </c>
       <c r="L297" s="2" t="n">
         <v>171</v>
       </c>
       <c r="M297" s="2" t="n">
-        <v>444</v>
+        <v>438</v>
       </c>
       <c r="N297" s="4" t="inlineStr">
         <is>
@@ -17700,13 +17700,13 @@
         <v>43</v>
       </c>
       <c r="K306" s="2" t="n">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="L306" s="2" t="n">
         <v>92</v>
       </c>
       <c r="M306" s="2" t="n">
-        <v>312</v>
+        <v>310</v>
       </c>
       <c r="N306" s="4" t="inlineStr">
         <is>
@@ -17868,7 +17868,7 @@
         </is>
       </c>
       <c r="J309" s="2" t="n">
-        <v>179</v>
+        <v>175</v>
       </c>
       <c r="K309" s="2" t="n">
         <v>1</v>
@@ -17877,7 +17877,7 @@
         <v>127</v>
       </c>
       <c r="M309" s="2" t="n">
-        <v>307</v>
+        <v>303</v>
       </c>
       <c r="N309" s="4" t="inlineStr">
         <is>
@@ -18042,13 +18042,13 @@
         <v>0</v>
       </c>
       <c r="K312" s="2" t="n">
-        <v>44</v>
+        <v>30</v>
       </c>
       <c r="L312" s="2" t="n">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="M312" s="2" t="n">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="N312" s="6" t="inlineStr">
         <is>
@@ -18381,20 +18381,20 @@
         </is>
       </c>
       <c r="J318" s="2" t="n">
-        <v>12</v>
+        <v>0</v>
       </c>
       <c r="K318" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L318" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="L318" s="2" t="n">
-        <v>0</v>
-      </c>
       <c r="M318" s="2" t="n">
-        <v>14</v>
-      </c>
-      <c r="N318" s="4" t="inlineStr">
-        <is>
-          <t>Stock</t>
+        <v>2</v>
+      </c>
+      <c r="N318" s="5" t="inlineStr">
+        <is>
+          <t>Sin stock</t>
         </is>
       </c>
       <c r="O318" s="2" t="n">
@@ -18441,13 +18441,13 @@
         <v>87</v>
       </c>
       <c r="K319" s="2" t="n">
-        <v>164</v>
+        <v>162</v>
       </c>
       <c r="L319" s="2" t="n">
         <v>52</v>
       </c>
       <c r="M319" s="2" t="n">
-        <v>303</v>
+        <v>301</v>
       </c>
       <c r="N319" s="4" t="inlineStr">
         <is>
@@ -19239,13 +19239,13 @@
         <v>56</v>
       </c>
       <c r="K333" s="2" t="n">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="L333" s="2" t="n">
         <v>155</v>
       </c>
       <c r="M333" s="2" t="n">
-        <v>296</v>
+        <v>294</v>
       </c>
       <c r="N333" s="4" t="inlineStr">
         <is>
@@ -19863,16 +19863,16 @@
         </is>
       </c>
       <c r="J344" s="2" t="n">
-        <v>27</v>
+        <v>63</v>
       </c>
       <c r="K344" s="2" t="n">
-        <v>331</v>
+        <v>289</v>
       </c>
       <c r="L344" s="2" t="n">
         <v>4</v>
       </c>
       <c r="M344" s="2" t="n">
-        <v>362</v>
+        <v>356</v>
       </c>
       <c r="N344" s="4" t="inlineStr">
         <is>
@@ -19920,20 +19920,20 @@
         </is>
       </c>
       <c r="J345" s="2" t="n">
-        <v>14</v>
+        <v>4</v>
       </c>
       <c r="K345" s="2" t="n">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="L345" s="2" t="n">
-        <v>23</v>
+        <v>18</v>
       </c>
       <c r="M345" s="2" t="n">
-        <v>64</v>
-      </c>
-      <c r="N345" s="4" t="inlineStr">
-        <is>
-          <t>Stock</t>
+        <v>48</v>
+      </c>
+      <c r="N345" s="6" t="inlineStr">
+        <is>
+          <t>7/10 Días</t>
         </is>
       </c>
       <c r="O345" s="2" t="n">
@@ -20205,7 +20205,7 @@
         </is>
       </c>
       <c r="J350" s="2" t="n">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="K350" s="2" t="n">
         <v>135</v>
@@ -20214,11 +20214,11 @@
         <v>32</v>
       </c>
       <c r="M350" s="2" t="n">
-        <v>177</v>
-      </c>
-      <c r="N350" s="4" t="inlineStr">
-        <is>
-          <t>Stock</t>
+        <v>174</v>
+      </c>
+      <c r="N350" s="6" t="inlineStr">
+        <is>
+          <t>7/10 Días</t>
         </is>
       </c>
       <c r="O350" s="2" t="n">
@@ -20490,20 +20490,20 @@
         </is>
       </c>
       <c r="J355" s="2" t="n">
-        <v>0</v>
+        <v>13</v>
       </c>
       <c r="K355" s="2" t="n">
         <v>1</v>
       </c>
       <c r="L355" s="2" t="n">
-        <v>42</v>
+        <v>21</v>
       </c>
       <c r="M355" s="2" t="n">
-        <v>43</v>
-      </c>
-      <c r="N355" s="6" t="inlineStr">
-        <is>
-          <t>7/10 Días</t>
+        <v>35</v>
+      </c>
+      <c r="N355" s="4" t="inlineStr">
+        <is>
+          <t>Stock</t>
         </is>
       </c>
       <c r="O355" s="2" t="n">
@@ -21123,10 +21123,10 @@
         <v>2</v>
       </c>
       <c r="L366" s="2" t="n">
-        <v>10</v>
+        <v>40</v>
       </c>
       <c r="M366" s="2" t="n">
-        <v>12</v>
+        <v>42</v>
       </c>
       <c r="N366" s="6" t="inlineStr">
         <is>
@@ -21237,10 +21237,10 @@
         <v>51</v>
       </c>
       <c r="L368" s="2" t="n">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="M368" s="2" t="n">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="N368" s="4" t="inlineStr">
         <is>
@@ -21351,10 +21351,10 @@
         <v>75</v>
       </c>
       <c r="L370" s="2" t="n">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="M370" s="2" t="n">
-        <v>160</v>
+        <v>157</v>
       </c>
       <c r="N370" s="4" t="inlineStr">
         <is>
@@ -21573,13 +21573,13 @@
         </is>
       </c>
       <c r="J374" s="2" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="K374" s="2" t="n">
-        <v>57</v>
+        <v>45</v>
       </c>
       <c r="L374" s="2" t="n">
-        <v>9</v>
+        <v>15</v>
       </c>
       <c r="M374" s="2" t="n">
         <v>69</v>
@@ -21747,13 +21747,13 @@
         <v>0</v>
       </c>
       <c r="K377" s="2" t="n">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="L377" s="2" t="n">
         <v>22</v>
       </c>
       <c r="M377" s="2" t="n">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="N377" s="6" t="inlineStr">
         <is>
@@ -22716,13 +22716,13 @@
         <v>118</v>
       </c>
       <c r="K394" s="2" t="n">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="L394" s="2" t="n">
         <v>0</v>
       </c>
       <c r="M394" s="2" t="n">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="N394" s="4" t="inlineStr">
         <is>
@@ -23050,13 +23050,13 @@
         <v>178</v>
       </c>
       <c r="K400" s="2" t="n">
-        <v>302</v>
+        <v>294</v>
       </c>
       <c r="L400" s="2" t="n">
         <v>93</v>
       </c>
       <c r="M400" s="2" t="n">
-        <v>573</v>
+        <v>565</v>
       </c>
       <c r="N400" s="4" t="inlineStr">
         <is>
@@ -23446,7 +23446,7 @@
         </is>
       </c>
       <c r="J407" s="2" t="n">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="K407" s="2" t="n">
         <v>0</v>
@@ -23455,7 +23455,7 @@
         <v>0</v>
       </c>
       <c r="M407" s="2" t="n">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="N407" s="4" t="inlineStr">
         <is>
@@ -23509,10 +23509,10 @@
         <v>91</v>
       </c>
       <c r="L408" s="2" t="n">
-        <v>1260</v>
+        <v>908</v>
       </c>
       <c r="M408" s="2" t="n">
-        <v>1424</v>
+        <v>1072</v>
       </c>
       <c r="N408" s="4" t="inlineStr">
         <is>
@@ -23677,13 +23677,13 @@
         <v>201</v>
       </c>
       <c r="K411" s="2" t="n">
-        <v>1280</v>
+        <v>1258</v>
       </c>
       <c r="L411" s="2" t="n">
         <v>0</v>
       </c>
       <c r="M411" s="2" t="n">
-        <v>1481</v>
+        <v>1459</v>
       </c>
       <c r="N411" s="4" t="inlineStr">
         <is>
@@ -23731,16 +23731,16 @@
         </is>
       </c>
       <c r="J412" s="2" t="n">
-        <v>399</v>
+        <v>397</v>
       </c>
       <c r="K412" s="2" t="n">
-        <v>1957</v>
+        <v>1948</v>
       </c>
       <c r="L412" s="2" t="n">
         <v>695</v>
       </c>
       <c r="M412" s="2" t="n">
-        <v>3051</v>
+        <v>3040</v>
       </c>
       <c r="N412" s="4" t="inlineStr">
         <is>
@@ -24076,13 +24076,13 @@
         <v>79</v>
       </c>
       <c r="K418" s="2" t="n">
-        <v>494</v>
+        <v>488</v>
       </c>
       <c r="L418" s="2" t="n">
         <v>274</v>
       </c>
       <c r="M418" s="2" t="n">
-        <v>847</v>
+        <v>841</v>
       </c>
       <c r="N418" s="4" t="inlineStr">
         <is>
@@ -24190,13 +24190,13 @@
         <v>128</v>
       </c>
       <c r="K420" s="2" t="n">
-        <v>282</v>
+        <v>280</v>
       </c>
       <c r="L420" s="2" t="n">
         <v>83</v>
       </c>
       <c r="M420" s="2" t="n">
-        <v>493</v>
+        <v>491</v>
       </c>
       <c r="N420" s="4" t="inlineStr">
         <is>
@@ -24304,13 +24304,13 @@
         <v>85</v>
       </c>
       <c r="K422" s="2" t="n">
-        <v>202</v>
+        <v>176</v>
       </c>
       <c r="L422" s="2" t="n">
         <v>69</v>
       </c>
       <c r="M422" s="2" t="n">
-        <v>356</v>
+        <v>330</v>
       </c>
       <c r="N422" s="4" t="inlineStr">
         <is>
@@ -24475,13 +24475,13 @@
         <v>179</v>
       </c>
       <c r="K425" s="2" t="n">
-        <v>224</v>
+        <v>222</v>
       </c>
       <c r="L425" s="2" t="n">
         <v>226</v>
       </c>
       <c r="M425" s="2" t="n">
-        <v>629</v>
+        <v>627</v>
       </c>
       <c r="N425" s="4" t="inlineStr">
         <is>
@@ -24586,7 +24586,7 @@
         </is>
       </c>
       <c r="J427" s="2" t="n">
-        <v>191</v>
+        <v>0</v>
       </c>
       <c r="K427" s="2" t="n">
         <v>205</v>
@@ -24595,11 +24595,11 @@
         <v>60</v>
       </c>
       <c r="M427" s="2" t="n">
-        <v>456</v>
-      </c>
-      <c r="N427" s="4" t="inlineStr">
-        <is>
-          <t>Stock</t>
+        <v>265</v>
+      </c>
+      <c r="N427" s="6" t="inlineStr">
+        <is>
+          <t>7/10 Días</t>
         </is>
       </c>
       <c r="O427" s="2" t="n">
@@ -24643,7 +24643,7 @@
         </is>
       </c>
       <c r="J428" s="2" t="n">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="K428" s="2" t="n">
         <v>40</v>
@@ -24652,7 +24652,7 @@
         <v>120</v>
       </c>
       <c r="M428" s="2" t="n">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="N428" s="4" t="inlineStr">
         <is>
@@ -24874,13 +24874,13 @@
         <v>137</v>
       </c>
       <c r="K432" s="2" t="n">
-        <v>500</v>
+        <v>479</v>
       </c>
       <c r="L432" s="2" t="n">
         <v>81</v>
       </c>
       <c r="M432" s="2" t="n">
-        <v>718</v>
+        <v>697</v>
       </c>
       <c r="N432" s="4" t="inlineStr">
         <is>
@@ -24988,13 +24988,13 @@
         <v>0</v>
       </c>
       <c r="K434" s="2" t="n">
-        <v>330</v>
+        <v>325</v>
       </c>
       <c r="L434" s="2" t="n">
         <v>157</v>
       </c>
       <c r="M434" s="2" t="n">
-        <v>487</v>
+        <v>482</v>
       </c>
       <c r="N434" s="6" t="inlineStr">
         <is>
@@ -25159,13 +25159,13 @@
         <v>0</v>
       </c>
       <c r="K437" s="2" t="n">
-        <v>262</v>
+        <v>260</v>
       </c>
       <c r="L437" s="2" t="n">
         <v>104</v>
       </c>
       <c r="M437" s="2" t="n">
-        <v>366</v>
+        <v>364</v>
       </c>
       <c r="N437" s="6" t="inlineStr">
         <is>
@@ -25216,13 +25216,13 @@
         <v>169</v>
       </c>
       <c r="K438" s="2" t="n">
-        <v>22</v>
+        <v>198</v>
       </c>
       <c r="L438" s="2" t="n">
         <v>191</v>
       </c>
       <c r="M438" s="2" t="n">
-        <v>382</v>
+        <v>558</v>
       </c>
       <c r="N438" s="4" t="inlineStr">
         <is>
@@ -25615,13 +25615,13 @@
         <v>11</v>
       </c>
       <c r="K445" s="2" t="n">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="L445" s="2" t="n">
         <v>6</v>
       </c>
       <c r="M445" s="2" t="n">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="N445" s="4" t="inlineStr">
         <is>
@@ -25954,7 +25954,7 @@
         </is>
       </c>
       <c r="J451" s="2" t="n">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="K451" s="2" t="n">
         <v>343</v>
@@ -25963,7 +25963,7 @@
         <v>463</v>
       </c>
       <c r="M451" s="2" t="n">
-        <v>885</v>
+        <v>883</v>
       </c>
       <c r="N451" s="4" t="inlineStr">
         <is>
@@ -26071,13 +26071,13 @@
         <v>42</v>
       </c>
       <c r="K453" s="2" t="n">
-        <v>118</v>
+        <v>108</v>
       </c>
       <c r="L453" s="2" t="n">
         <v>257</v>
       </c>
       <c r="M453" s="2" t="n">
-        <v>417</v>
+        <v>407</v>
       </c>
       <c r="N453" s="4" t="inlineStr">
         <is>
@@ -26128,13 +26128,13 @@
         <v>1</v>
       </c>
       <c r="K454" s="2" t="n">
-        <v>78</v>
+        <v>56</v>
       </c>
       <c r="L454" s="2" t="n">
-        <v>180</v>
+        <v>140</v>
       </c>
       <c r="M454" s="2" t="n">
-        <v>259</v>
+        <v>197</v>
       </c>
       <c r="N454" s="6" t="inlineStr">
         <is>
@@ -26245,10 +26245,10 @@
         <v>117</v>
       </c>
       <c r="L456" s="2" t="n">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="M456" s="2" t="n">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="N456" s="4" t="inlineStr">
         <is>
@@ -26356,13 +26356,13 @@
         <v>1</v>
       </c>
       <c r="K458" s="2" t="n">
-        <v>56</v>
+        <v>34</v>
       </c>
       <c r="L458" s="2" t="n">
         <v>95</v>
       </c>
       <c r="M458" s="2" t="n">
-        <v>152</v>
+        <v>130</v>
       </c>
       <c r="N458" s="6" t="inlineStr">
         <is>
@@ -26698,13 +26698,13 @@
         <v>0</v>
       </c>
       <c r="K464" s="2" t="n">
+        <v>125</v>
+      </c>
+      <c r="L464" s="2" t="n">
         <v>127</v>
       </c>
-      <c r="L464" s="2" t="n">
-        <v>130</v>
-      </c>
       <c r="M464" s="2" t="n">
-        <v>257</v>
+        <v>252</v>
       </c>
       <c r="N464" s="6" t="inlineStr">
         <is>
@@ -27211,13 +27211,13 @@
         <v>1</v>
       </c>
       <c r="K473" s="2" t="n">
-        <v>72</v>
+        <v>33</v>
       </c>
       <c r="L473" s="2" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="M473" s="2" t="n">
-        <v>73</v>
+        <v>37</v>
       </c>
       <c r="N473" s="6" t="inlineStr">
         <is>
@@ -27439,13 +27439,13 @@
         <v>0</v>
       </c>
       <c r="K477" s="2" t="n">
-        <v>456</v>
+        <v>453</v>
       </c>
       <c r="L477" s="2" t="n">
         <v>0</v>
       </c>
       <c r="M477" s="2" t="n">
-        <v>456</v>
+        <v>453</v>
       </c>
       <c r="N477" s="6" t="inlineStr">
         <is>
@@ -27781,13 +27781,13 @@
         <v>8</v>
       </c>
       <c r="K483" s="2" t="n">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="L483" s="2" t="n">
         <v>0</v>
       </c>
       <c r="M483" s="2" t="n">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="N483" s="6" t="inlineStr">
         <is>
@@ -27895,13 +27895,13 @@
         <v>2</v>
       </c>
       <c r="K485" s="2" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="L485" s="2" t="n">
         <v>46</v>
       </c>
       <c r="M485" s="2" t="n">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="N485" s="6" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Update inventario_expandido.xlsx — 10/07/2026 (+6 refs nuevas)
</commit_message>
<xml_diff>
--- a/inventario_expandido.xlsx
+++ b/inventario_expandido.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Inventario" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Inventario'!$A$1:$O$490</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Inventario'!$A$1:$O$496</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -481,7 +481,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O490"/>
+  <dimension ref="A1:O496"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -729,7 +729,7 @@
         </is>
       </c>
       <c r="J4" s="2" t="n">
-        <v>12</v>
+        <v>347</v>
       </c>
       <c r="K4" s="2" t="n">
         <v>11</v>
@@ -738,7 +738,7 @@
         <v>0</v>
       </c>
       <c r="M4" s="2" t="n">
-        <v>23</v>
+        <v>358</v>
       </c>
       <c r="N4" s="4" t="inlineStr">
         <is>
@@ -787,13 +787,13 @@
         <v>300</v>
       </c>
       <c r="K5" s="2" t="n">
-        <v>437</v>
+        <v>427</v>
       </c>
       <c r="L5" s="2" t="n">
         <v>567</v>
       </c>
       <c r="M5" s="2" t="n">
-        <v>1304</v>
+        <v>1294</v>
       </c>
       <c r="N5" s="4" t="inlineStr">
         <is>
@@ -1385,7 +1385,7 @@
         </is>
       </c>
       <c r="J16" s="2" t="n">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="K16" s="2" t="n">
         <v>345</v>
@@ -1394,7 +1394,7 @@
         <v>56</v>
       </c>
       <c r="M16" s="2" t="n">
-        <v>545</v>
+        <v>543</v>
       </c>
       <c r="N16" s="4" t="inlineStr">
         <is>
@@ -1547,13 +1547,13 @@
         <v>99</v>
       </c>
       <c r="K19" s="2" t="n">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="L19" s="2" t="n">
         <v>87</v>
       </c>
       <c r="M19" s="2" t="n">
-        <v>311</v>
+        <v>309</v>
       </c>
       <c r="N19" s="4" t="inlineStr">
         <is>
@@ -2349,16 +2349,16 @@
         </is>
       </c>
       <c r="J34" s="2" t="n">
-        <v>289</v>
+        <v>279</v>
       </c>
       <c r="K34" s="2" t="n">
         <v>0</v>
       </c>
       <c r="L34" s="2" t="n">
-        <v>273</v>
+        <v>198</v>
       </c>
       <c r="M34" s="2" t="n">
-        <v>562</v>
+        <v>477</v>
       </c>
       <c r="N34" s="4" t="inlineStr">
         <is>
@@ -2407,13 +2407,13 @@
         <v>99</v>
       </c>
       <c r="K35" s="2" t="n">
-        <v>79</v>
+        <v>12</v>
       </c>
       <c r="L35" s="2" t="n">
         <v>1</v>
       </c>
       <c r="M35" s="2" t="n">
-        <v>179</v>
+        <v>112</v>
       </c>
       <c r="N35" s="4" t="inlineStr">
         <is>
@@ -2462,13 +2462,13 @@
         <v>90</v>
       </c>
       <c r="K36" s="2" t="n">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="L36" s="2" t="n">
         <v>184</v>
       </c>
       <c r="M36" s="2" t="n">
-        <v>525</v>
+        <v>524</v>
       </c>
       <c r="N36" s="4" t="inlineStr">
         <is>
@@ -2624,7 +2624,7 @@
         </is>
       </c>
       <c r="J39" s="2" t="n">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="K39" s="2" t="n">
         <v>502</v>
@@ -2633,7 +2633,7 @@
         <v>176</v>
       </c>
       <c r="M39" s="2" t="n">
-        <v>753</v>
+        <v>751</v>
       </c>
       <c r="N39" s="4" t="inlineStr">
         <is>
@@ -2734,7 +2734,7 @@
         </is>
       </c>
       <c r="J41" s="2" t="n">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="K41" s="2" t="n">
         <v>17</v>
@@ -2743,7 +2743,7 @@
         <v>80</v>
       </c>
       <c r="M41" s="2" t="n">
-        <v>275</v>
+        <v>273</v>
       </c>
       <c r="N41" s="4" t="inlineStr">
         <is>
@@ -2847,13 +2847,13 @@
         <v>10</v>
       </c>
       <c r="K43" s="2" t="n">
-        <v>203</v>
+        <v>199</v>
       </c>
       <c r="L43" s="2" t="n">
         <v>42</v>
       </c>
       <c r="M43" s="2" t="n">
-        <v>255</v>
+        <v>251</v>
       </c>
       <c r="N43" s="4" t="inlineStr">
         <is>
@@ -3009,7 +3009,7 @@
         </is>
       </c>
       <c r="J46" s="2" t="n">
-        <v>177</v>
+        <v>172</v>
       </c>
       <c r="K46" s="2" t="n">
         <v>23</v>
@@ -3018,7 +3018,7 @@
         <v>24</v>
       </c>
       <c r="M46" s="2" t="n">
-        <v>224</v>
+        <v>219</v>
       </c>
       <c r="N46" s="4" t="inlineStr">
         <is>
@@ -3180,10 +3180,10 @@
         <v>73</v>
       </c>
       <c r="L49" s="2" t="n">
-        <v>26</v>
+        <v>18</v>
       </c>
       <c r="M49" s="2" t="n">
-        <v>149</v>
+        <v>141</v>
       </c>
       <c r="N49" s="4" t="inlineStr">
         <is>
@@ -3617,13 +3617,13 @@
         <v>0</v>
       </c>
       <c r="K57" s="2" t="n">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="L57" s="2" t="n">
         <v>0</v>
       </c>
       <c r="M57" s="2" t="n">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="N57" s="6" t="inlineStr">
         <is>
@@ -3672,13 +3672,13 @@
         <v>28</v>
       </c>
       <c r="K58" s="2" t="n">
-        <v>23</v>
+        <v>13</v>
       </c>
       <c r="L58" s="2" t="n">
         <v>25</v>
       </c>
       <c r="M58" s="2" t="n">
-        <v>76</v>
+        <v>66</v>
       </c>
       <c r="N58" s="4" t="inlineStr">
         <is>
@@ -4332,13 +4332,13 @@
         <v>13</v>
       </c>
       <c r="K70" s="2" t="n">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="L70" s="2" t="n">
         <v>0</v>
       </c>
       <c r="M70" s="2" t="n">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="N70" s="4" t="inlineStr">
         <is>
@@ -4497,13 +4497,13 @@
         <v>42</v>
       </c>
       <c r="K73" s="2" t="n">
-        <v>337</v>
+        <v>335</v>
       </c>
       <c r="L73" s="2" t="n">
         <v>0</v>
       </c>
       <c r="M73" s="2" t="n">
-        <v>379</v>
+        <v>377</v>
       </c>
       <c r="N73" s="4" t="inlineStr">
         <is>
@@ -4552,13 +4552,13 @@
         <v>85</v>
       </c>
       <c r="K74" s="2" t="n">
-        <v>241</v>
+        <v>238</v>
       </c>
       <c r="L74" s="2" t="n">
         <v>92</v>
       </c>
       <c r="M74" s="2" t="n">
-        <v>418</v>
+        <v>415</v>
       </c>
       <c r="N74" s="4" t="inlineStr">
         <is>
@@ -5270,10 +5270,10 @@
         <v>42</v>
       </c>
       <c r="L87" s="2" t="n">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="M87" s="2" t="n">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="N87" s="4" t="inlineStr">
         <is>
@@ -5429,7 +5429,7 @@
         </is>
       </c>
       <c r="J90" s="2" t="n">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="K90" s="2" t="n">
         <v>0</v>
@@ -5438,7 +5438,7 @@
         <v>97</v>
       </c>
       <c r="M90" s="2" t="n">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="N90" s="4" t="inlineStr">
         <is>
@@ -5869,7 +5869,7 @@
         </is>
       </c>
       <c r="J98" s="2" t="n">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="K98" s="2" t="n">
         <v>97</v>
@@ -5878,7 +5878,7 @@
         <v>0</v>
       </c>
       <c r="M98" s="2" t="n">
-        <v>188</v>
+        <v>186</v>
       </c>
       <c r="N98" s="4" t="inlineStr">
         <is>
@@ -6870,13 +6870,13 @@
         <v>23</v>
       </c>
       <c r="K116" s="2" t="n">
-        <v>115</v>
+        <v>192</v>
       </c>
       <c r="L116" s="2" t="n">
         <v>0</v>
       </c>
       <c r="M116" s="2" t="n">
-        <v>138</v>
+        <v>215</v>
       </c>
       <c r="N116" s="4" t="inlineStr">
         <is>
@@ -7671,10 +7671,10 @@
         <v>92</v>
       </c>
       <c r="L130" s="2" t="n">
-        <v>90</v>
+        <v>85</v>
       </c>
       <c r="M130" s="2" t="n">
-        <v>214</v>
+        <v>209</v>
       </c>
       <c r="N130" s="4" t="inlineStr">
         <is>
@@ -7953,13 +7953,13 @@
         <v>29</v>
       </c>
       <c r="K135" s="2" t="n">
-        <v>19</v>
+        <v>334</v>
       </c>
       <c r="L135" s="2" t="n">
         <v>187</v>
       </c>
       <c r="M135" s="2" t="n">
-        <v>235</v>
+        <v>550</v>
       </c>
       <c r="N135" s="4" t="inlineStr">
         <is>
@@ -8520,16 +8520,16 @@
         </is>
       </c>
       <c r="J145" s="2" t="n">
-        <v>342</v>
+        <v>335</v>
       </c>
       <c r="K145" s="2" t="n">
-        <v>488</v>
+        <v>468</v>
       </c>
       <c r="L145" s="2" t="n">
         <v>248</v>
       </c>
       <c r="M145" s="2" t="n">
-        <v>1078</v>
+        <v>1051</v>
       </c>
       <c r="N145" s="4" t="inlineStr">
         <is>
@@ -8694,13 +8694,13 @@
         <v>0</v>
       </c>
       <c r="K148" s="2" t="n">
-        <v>385</v>
+        <v>377</v>
       </c>
       <c r="L148" s="2" t="n">
         <v>22</v>
       </c>
       <c r="M148" s="2" t="n">
-        <v>407</v>
+        <v>399</v>
       </c>
       <c r="N148" s="6" t="inlineStr">
         <is>
@@ -9090,7 +9090,7 @@
         </is>
       </c>
       <c r="J155" s="2" t="n">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="K155" s="2" t="n">
         <v>0</v>
@@ -9099,7 +9099,7 @@
         <v>82</v>
       </c>
       <c r="M155" s="2" t="n">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="N155" s="4" t="inlineStr">
         <is>
@@ -9720,13 +9720,13 @@
         <v>112</v>
       </c>
       <c r="K166" s="2" t="n">
-        <v>604</v>
+        <v>596</v>
       </c>
       <c r="L166" s="2" t="n">
         <v>75</v>
       </c>
       <c r="M166" s="2" t="n">
-        <v>791</v>
+        <v>783</v>
       </c>
       <c r="N166" s="4" t="inlineStr">
         <is>
@@ -10347,13 +10347,13 @@
         <v>0</v>
       </c>
       <c r="K177" s="2" t="n">
-        <v>118</v>
+        <v>0</v>
       </c>
       <c r="L177" s="2" t="n">
         <v>48</v>
       </c>
       <c r="M177" s="2" t="n">
-        <v>166</v>
+        <v>48</v>
       </c>
       <c r="N177" s="6" t="inlineStr">
         <is>
@@ -10404,13 +10404,13 @@
         <v>169</v>
       </c>
       <c r="K178" s="2" t="n">
-        <v>0</v>
+        <v>149</v>
       </c>
       <c r="L178" s="2" t="n">
         <v>70</v>
       </c>
       <c r="M178" s="2" t="n">
-        <v>239</v>
+        <v>388</v>
       </c>
       <c r="N178" s="4" t="inlineStr">
         <is>
@@ -10518,13 +10518,13 @@
         <v>9</v>
       </c>
       <c r="K180" s="2" t="n">
-        <v>17</v>
+        <v>10</v>
       </c>
       <c r="L180" s="2" t="n">
         <v>0</v>
       </c>
       <c r="M180" s="2" t="n">
-        <v>26</v>
+        <v>19</v>
       </c>
       <c r="N180" s="6" t="inlineStr">
         <is>
@@ -10689,13 +10689,13 @@
         <v>0</v>
       </c>
       <c r="K183" s="2" t="n">
-        <v>87</v>
+        <v>302</v>
       </c>
       <c r="L183" s="2" t="n">
         <v>100</v>
       </c>
       <c r="M183" s="2" t="n">
-        <v>187</v>
+        <v>402</v>
       </c>
       <c r="N183" s="6" t="inlineStr">
         <is>
@@ -11544,13 +11544,13 @@
         <v>106</v>
       </c>
       <c r="K198" s="2" t="n">
-        <v>361</v>
+        <v>321</v>
       </c>
       <c r="L198" s="2" t="n">
         <v>180</v>
       </c>
       <c r="M198" s="2" t="n">
-        <v>647</v>
+        <v>607</v>
       </c>
       <c r="N198" s="4" t="inlineStr">
         <is>
@@ -11769,16 +11769,16 @@
         </is>
       </c>
       <c r="J202" s="2" t="n">
-        <v>197</v>
+        <v>195</v>
       </c>
       <c r="K202" s="2" t="n">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="L202" s="2" t="n">
         <v>120</v>
       </c>
       <c r="M202" s="2" t="n">
-        <v>474</v>
+        <v>470</v>
       </c>
       <c r="N202" s="4" t="inlineStr">
         <is>
@@ -12000,13 +12000,13 @@
         <v>147</v>
       </c>
       <c r="K206" s="2" t="n">
-        <v>63</v>
+        <v>56</v>
       </c>
       <c r="L206" s="2" t="n">
         <v>96</v>
       </c>
       <c r="M206" s="2" t="n">
-        <v>306</v>
+        <v>299</v>
       </c>
       <c r="N206" s="4" t="inlineStr">
         <is>
@@ -12057,13 +12057,13 @@
         <v>116</v>
       </c>
       <c r="K207" s="2" t="n">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="L207" s="2" t="n">
         <v>46</v>
       </c>
       <c r="M207" s="2" t="n">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="N207" s="4" t="inlineStr">
         <is>
@@ -12342,13 +12342,13 @@
         <v>129</v>
       </c>
       <c r="K212" s="2" t="n">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="L212" s="2" t="n">
         <v>41</v>
       </c>
       <c r="M212" s="2" t="n">
-        <v>231</v>
+        <v>229</v>
       </c>
       <c r="N212" s="4" t="inlineStr">
         <is>
@@ -12399,13 +12399,13 @@
         <v>0</v>
       </c>
       <c r="K213" s="2" t="n">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="L213" s="2" t="n">
         <v>35</v>
       </c>
       <c r="M213" s="2" t="n">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="N213" s="6" t="inlineStr">
         <is>
@@ -13485,10 +13485,10 @@
         <v>179</v>
       </c>
       <c r="L232" s="2" t="n">
-        <v>12</v>
+        <v>7</v>
       </c>
       <c r="M232" s="2" t="n">
-        <v>267</v>
+        <v>262</v>
       </c>
       <c r="N232" s="4" t="inlineStr">
         <is>
@@ -13596,13 +13596,13 @@
         <v>6</v>
       </c>
       <c r="K234" s="2" t="n">
-        <v>17</v>
+        <v>85</v>
       </c>
       <c r="L234" s="2" t="n">
         <v>22</v>
       </c>
       <c r="M234" s="2" t="n">
-        <v>45</v>
+        <v>113</v>
       </c>
       <c r="N234" s="6" t="inlineStr">
         <is>
@@ -14625,10 +14625,10 @@
         <v>0</v>
       </c>
       <c r="L252" s="2" t="n">
-        <v>211</v>
+        <v>151</v>
       </c>
       <c r="M252" s="2" t="n">
-        <v>264</v>
+        <v>204</v>
       </c>
       <c r="N252" s="4" t="inlineStr">
         <is>
@@ -14676,16 +14676,16 @@
         </is>
       </c>
       <c r="J253" s="2" t="n">
-        <v>196</v>
+        <v>193</v>
       </c>
       <c r="K253" s="2" t="n">
-        <v>259</v>
+        <v>242</v>
       </c>
       <c r="L253" s="2" t="n">
         <v>181</v>
       </c>
       <c r="M253" s="2" t="n">
-        <v>636</v>
+        <v>616</v>
       </c>
       <c r="N253" s="4" t="inlineStr">
         <is>
@@ -14736,13 +14736,13 @@
         <v>0</v>
       </c>
       <c r="K254" s="2" t="n">
-        <v>287</v>
+        <v>284</v>
       </c>
       <c r="L254" s="2" t="n">
         <v>45</v>
       </c>
       <c r="M254" s="2" t="n">
-        <v>332</v>
+        <v>329</v>
       </c>
       <c r="N254" s="6" t="inlineStr">
         <is>
@@ -14961,16 +14961,16 @@
         </is>
       </c>
       <c r="J258" s="2" t="n">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="K258" s="2" t="n">
-        <v>158</v>
+        <v>148</v>
       </c>
       <c r="L258" s="2" t="n">
         <v>79</v>
       </c>
       <c r="M258" s="2" t="n">
-        <v>302</v>
+        <v>290</v>
       </c>
       <c r="N258" s="4" t="inlineStr">
         <is>
@@ -15078,13 +15078,13 @@
         <v>71</v>
       </c>
       <c r="K260" s="2" t="n">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="L260" s="2" t="n">
         <v>44</v>
       </c>
       <c r="M260" s="2" t="n">
-        <v>166</v>
+        <v>164</v>
       </c>
       <c r="N260" s="4" t="inlineStr">
         <is>
@@ -15138,10 +15138,10 @@
         <v>103</v>
       </c>
       <c r="L261" s="2" t="n">
-        <v>116</v>
+        <v>100</v>
       </c>
       <c r="M261" s="2" t="n">
-        <v>313</v>
+        <v>297</v>
       </c>
       <c r="N261" s="4" t="inlineStr">
         <is>
@@ -15477,13 +15477,13 @@
         <v>4</v>
       </c>
       <c r="K267" s="2" t="n">
-        <v>34</v>
+        <v>26</v>
       </c>
       <c r="L267" s="2" t="n">
         <v>12</v>
       </c>
       <c r="M267" s="2" t="n">
-        <v>50</v>
+        <v>42</v>
       </c>
       <c r="N267" s="6" t="inlineStr">
         <is>
@@ -15591,13 +15591,13 @@
         <v>39</v>
       </c>
       <c r="K269" s="2" t="n">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="L269" s="2" t="n">
         <v>10</v>
       </c>
       <c r="M269" s="2" t="n">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="N269" s="4" t="inlineStr">
         <is>
@@ -15645,16 +15645,16 @@
         </is>
       </c>
       <c r="J270" s="2" t="n">
-        <v>51</v>
+        <v>40</v>
       </c>
       <c r="K270" s="2" t="n">
-        <v>227</v>
+        <v>222</v>
       </c>
       <c r="L270" s="2" t="n">
-        <v>166</v>
+        <v>115</v>
       </c>
       <c r="M270" s="2" t="n">
-        <v>444</v>
+        <v>377</v>
       </c>
       <c r="N270" s="4" t="inlineStr">
         <is>
@@ -16161,13 +16161,13 @@
         <v>81</v>
       </c>
       <c r="K279" s="2" t="n">
-        <v>95</v>
+        <v>89</v>
       </c>
       <c r="L279" s="2" t="n">
         <v>69</v>
       </c>
       <c r="M279" s="2" t="n">
-        <v>245</v>
+        <v>239</v>
       </c>
       <c r="N279" s="4" t="inlineStr">
         <is>
@@ -16392,10 +16392,10 @@
         <v>246</v>
       </c>
       <c r="L283" s="2" t="n">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="M283" s="2" t="n">
-        <v>323</v>
+        <v>321</v>
       </c>
       <c r="N283" s="6" t="inlineStr">
         <is>
@@ -16734,10 +16734,10 @@
         <v>6</v>
       </c>
       <c r="L289" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M289" s="2" t="n">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="N289" s="4" t="inlineStr">
         <is>
@@ -17184,16 +17184,16 @@
         </is>
       </c>
       <c r="J297" s="2" t="n">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="K297" s="2" t="n">
-        <v>191</v>
+        <v>145</v>
       </c>
       <c r="L297" s="2" t="n">
-        <v>171</v>
+        <v>163</v>
       </c>
       <c r="M297" s="2" t="n">
-        <v>438</v>
+        <v>383</v>
       </c>
       <c r="N297" s="4" t="inlineStr">
         <is>
@@ -17301,13 +17301,13 @@
         <v>0</v>
       </c>
       <c r="K299" s="2" t="n">
-        <v>13</v>
+        <v>93</v>
       </c>
       <c r="L299" s="2" t="n">
         <v>69</v>
       </c>
       <c r="M299" s="2" t="n">
-        <v>82</v>
+        <v>162</v>
       </c>
       <c r="N299" s="6" t="inlineStr">
         <is>
@@ -17532,10 +17532,10 @@
         <v>135</v>
       </c>
       <c r="L303" s="2" t="n">
-        <v>58</v>
+        <v>52</v>
       </c>
       <c r="M303" s="2" t="n">
-        <v>247</v>
+        <v>241</v>
       </c>
       <c r="N303" s="4" t="inlineStr">
         <is>
@@ -17700,13 +17700,13 @@
         <v>43</v>
       </c>
       <c r="K306" s="2" t="n">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="L306" s="2" t="n">
-        <v>92</v>
+        <v>87</v>
       </c>
       <c r="M306" s="2" t="n">
-        <v>310</v>
+        <v>304</v>
       </c>
       <c r="N306" s="4" t="inlineStr">
         <is>
@@ -17760,10 +17760,10 @@
         <v>67</v>
       </c>
       <c r="L307" s="2" t="n">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="M307" s="2" t="n">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="N307" s="4" t="inlineStr">
         <is>
@@ -17985,13 +17985,13 @@
         <v>13</v>
       </c>
       <c r="K311" s="2" t="n">
-        <v>35</v>
+        <v>28</v>
       </c>
       <c r="L311" s="2" t="n">
         <v>0</v>
       </c>
       <c r="M311" s="2" t="n">
-        <v>48</v>
+        <v>41</v>
       </c>
       <c r="N311" s="4" t="inlineStr">
         <is>
@@ -18441,13 +18441,13 @@
         <v>87</v>
       </c>
       <c r="K319" s="2" t="n">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="L319" s="2" t="n">
         <v>52</v>
       </c>
       <c r="M319" s="2" t="n">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="N319" s="4" t="inlineStr">
         <is>
@@ -19752,13 +19752,13 @@
         <v>83</v>
       </c>
       <c r="K342" s="2" t="n">
-        <v>103</v>
+        <v>96</v>
       </c>
       <c r="L342" s="2" t="n">
-        <v>34</v>
+        <v>28</v>
       </c>
       <c r="M342" s="2" t="n">
-        <v>220</v>
+        <v>207</v>
       </c>
       <c r="N342" s="4" t="inlineStr">
         <is>
@@ -20037,13 +20037,13 @@
         <v>115</v>
       </c>
       <c r="K347" s="2" t="n">
-        <v>309</v>
+        <v>299</v>
       </c>
       <c r="L347" s="2" t="n">
         <v>187</v>
       </c>
       <c r="M347" s="2" t="n">
-        <v>611</v>
+        <v>601</v>
       </c>
       <c r="N347" s="4" t="inlineStr">
         <is>
@@ -20208,13 +20208,13 @@
         <v>7</v>
       </c>
       <c r="K350" s="2" t="n">
-        <v>135</v>
+        <v>126</v>
       </c>
       <c r="L350" s="2" t="n">
         <v>32</v>
       </c>
       <c r="M350" s="2" t="n">
-        <v>174</v>
+        <v>165</v>
       </c>
       <c r="N350" s="6" t="inlineStr">
         <is>
@@ -20949,13 +20949,13 @@
         <v>0</v>
       </c>
       <c r="K363" s="2" t="n">
-        <v>27</v>
+        <v>22</v>
       </c>
       <c r="L363" s="2" t="n">
         <v>0</v>
       </c>
       <c r="M363" s="2" t="n">
-        <v>27</v>
+        <v>22</v>
       </c>
       <c r="N363" s="6" t="inlineStr">
         <is>
@@ -21348,13 +21348,13 @@
         <v>38</v>
       </c>
       <c r="K370" s="2" t="n">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="L370" s="2" t="n">
         <v>44</v>
       </c>
       <c r="M370" s="2" t="n">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="N370" s="4" t="inlineStr">
         <is>
@@ -21636,10 +21636,10 @@
         <v>30</v>
       </c>
       <c r="L375" s="2" t="n">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="M375" s="2" t="n">
-        <v>39</v>
+        <v>35</v>
       </c>
       <c r="N375" s="6" t="inlineStr">
         <is>
@@ -21747,13 +21747,13 @@
         <v>0</v>
       </c>
       <c r="K377" s="2" t="n">
-        <v>99</v>
+        <v>62</v>
       </c>
       <c r="L377" s="2" t="n">
         <v>22</v>
       </c>
       <c r="M377" s="2" t="n">
-        <v>121</v>
+        <v>84</v>
       </c>
       <c r="N377" s="6" t="inlineStr">
         <is>
@@ -21807,10 +21807,10 @@
         <v>7</v>
       </c>
       <c r="L378" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="M378" s="2" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="N378" s="5" t="inlineStr">
         <is>
@@ -21915,7 +21915,7 @@
         </is>
       </c>
       <c r="J380" s="2" t="n">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="K380" s="2" t="n">
         <v>138</v>
@@ -21924,7 +21924,7 @@
         <v>25</v>
       </c>
       <c r="M380" s="2" t="n">
-        <v>233</v>
+        <v>231</v>
       </c>
       <c r="N380" s="4" t="inlineStr">
         <is>
@@ -21975,13 +21975,13 @@
         <v>58</v>
       </c>
       <c r="K381" s="2" t="n">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="L381" s="2" t="n">
         <v>0</v>
       </c>
       <c r="M381" s="2" t="n">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="N381" s="4" t="inlineStr">
         <is>
@@ -23050,13 +23050,13 @@
         <v>178</v>
       </c>
       <c r="K400" s="2" t="n">
-        <v>294</v>
+        <v>286</v>
       </c>
       <c r="L400" s="2" t="n">
         <v>93</v>
       </c>
       <c r="M400" s="2" t="n">
-        <v>565</v>
+        <v>557</v>
       </c>
       <c r="N400" s="4" t="inlineStr">
         <is>
@@ -23677,13 +23677,13 @@
         <v>201</v>
       </c>
       <c r="K411" s="2" t="n">
-        <v>1258</v>
+        <v>1185</v>
       </c>
       <c r="L411" s="2" t="n">
         <v>0</v>
       </c>
       <c r="M411" s="2" t="n">
-        <v>1459</v>
+        <v>1386</v>
       </c>
       <c r="N411" s="4" t="inlineStr">
         <is>
@@ -23731,16 +23731,16 @@
         </is>
       </c>
       <c r="J412" s="2" t="n">
-        <v>397</v>
+        <v>395</v>
       </c>
       <c r="K412" s="2" t="n">
-        <v>1948</v>
+        <v>1947</v>
       </c>
       <c r="L412" s="2" t="n">
         <v>695</v>
       </c>
       <c r="M412" s="2" t="n">
-        <v>3040</v>
+        <v>3037</v>
       </c>
       <c r="N412" s="4" t="inlineStr">
         <is>
@@ -23905,13 +23905,13 @@
         <v>279</v>
       </c>
       <c r="K415" s="2" t="n">
-        <v>769</v>
+        <v>766</v>
       </c>
       <c r="L415" s="2" t="n">
         <v>66</v>
       </c>
       <c r="M415" s="2" t="n">
-        <v>1114</v>
+        <v>1111</v>
       </c>
       <c r="N415" s="4" t="inlineStr">
         <is>
@@ -24073,16 +24073,16 @@
         </is>
       </c>
       <c r="J418" s="2" t="n">
-        <v>79</v>
+        <v>67</v>
       </c>
       <c r="K418" s="2" t="n">
-        <v>488</v>
+        <v>477</v>
       </c>
       <c r="L418" s="2" t="n">
         <v>274</v>
       </c>
       <c r="M418" s="2" t="n">
-        <v>841</v>
+        <v>818</v>
       </c>
       <c r="N418" s="4" t="inlineStr">
         <is>
@@ -24247,13 +24247,13 @@
         <v>0</v>
       </c>
       <c r="K421" s="2" t="n">
-        <v>188</v>
+        <v>182</v>
       </c>
       <c r="L421" s="2" t="n">
         <v>109</v>
       </c>
       <c r="M421" s="2" t="n">
-        <v>297</v>
+        <v>291</v>
       </c>
       <c r="N421" s="6" t="inlineStr">
         <is>
@@ -24475,13 +24475,13 @@
         <v>179</v>
       </c>
       <c r="K425" s="2" t="n">
-        <v>222</v>
+        <v>215</v>
       </c>
       <c r="L425" s="2" t="n">
         <v>226</v>
       </c>
       <c r="M425" s="2" t="n">
-        <v>627</v>
+        <v>620</v>
       </c>
       <c r="N425" s="4" t="inlineStr">
         <is>
@@ -24760,13 +24760,13 @@
         <v>65</v>
       </c>
       <c r="K430" s="2" t="n">
-        <v>281</v>
+        <v>69</v>
       </c>
       <c r="L430" s="2" t="n">
         <v>31</v>
       </c>
       <c r="M430" s="2" t="n">
-        <v>377</v>
+        <v>165</v>
       </c>
       <c r="N430" s="4" t="inlineStr">
         <is>
@@ -24871,16 +24871,16 @@
         </is>
       </c>
       <c r="J432" s="2" t="n">
-        <v>137</v>
+        <v>49</v>
       </c>
       <c r="K432" s="2" t="n">
-        <v>479</v>
+        <v>403</v>
       </c>
       <c r="L432" s="2" t="n">
         <v>81</v>
       </c>
       <c r="M432" s="2" t="n">
-        <v>697</v>
+        <v>533</v>
       </c>
       <c r="N432" s="4" t="inlineStr">
         <is>
@@ -24991,10 +24991,10 @@
         <v>325</v>
       </c>
       <c r="L434" s="2" t="n">
-        <v>157</v>
+        <v>117</v>
       </c>
       <c r="M434" s="2" t="n">
-        <v>482</v>
+        <v>442</v>
       </c>
       <c r="N434" s="6" t="inlineStr">
         <is>
@@ -25102,13 +25102,13 @@
         <v>218</v>
       </c>
       <c r="K436" s="2" t="n">
-        <v>239</v>
+        <v>219</v>
       </c>
       <c r="L436" s="2" t="n">
-        <v>24</v>
+        <v>4</v>
       </c>
       <c r="M436" s="2" t="n">
-        <v>481</v>
+        <v>441</v>
       </c>
       <c r="N436" s="4" t="inlineStr">
         <is>
@@ -25159,13 +25159,13 @@
         <v>0</v>
       </c>
       <c r="K437" s="2" t="n">
-        <v>260</v>
+        <v>256</v>
       </c>
       <c r="L437" s="2" t="n">
         <v>104</v>
       </c>
       <c r="M437" s="2" t="n">
-        <v>364</v>
+        <v>360</v>
       </c>
       <c r="N437" s="6" t="inlineStr">
         <is>
@@ -25216,13 +25216,13 @@
         <v>169</v>
       </c>
       <c r="K438" s="2" t="n">
-        <v>198</v>
+        <v>272</v>
       </c>
       <c r="L438" s="2" t="n">
         <v>191</v>
       </c>
       <c r="M438" s="2" t="n">
-        <v>558</v>
+        <v>632</v>
       </c>
       <c r="N438" s="4" t="inlineStr">
         <is>
@@ -25330,13 +25330,13 @@
         <v>0</v>
       </c>
       <c r="K440" s="2" t="n">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="L440" s="2" t="n">
         <v>59</v>
       </c>
       <c r="M440" s="2" t="n">
-        <v>197</v>
+        <v>195</v>
       </c>
       <c r="N440" s="6" t="inlineStr">
         <is>
@@ -25444,13 +25444,13 @@
         <v>19</v>
       </c>
       <c r="K442" s="2" t="n">
-        <v>67</v>
+        <v>59</v>
       </c>
       <c r="L442" s="2" t="n">
         <v>61</v>
       </c>
       <c r="M442" s="2" t="n">
-        <v>147</v>
+        <v>139</v>
       </c>
       <c r="N442" s="4" t="inlineStr">
         <is>
@@ -25729,13 +25729,13 @@
         <v>0</v>
       </c>
       <c r="K447" s="2" t="n">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="L447" s="2" t="n">
         <v>2</v>
       </c>
       <c r="M447" s="2" t="n">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="N447" s="6" t="inlineStr">
         <is>
@@ -25786,13 +25786,13 @@
         <v>4</v>
       </c>
       <c r="K448" s="2" t="n">
-        <v>80</v>
+        <v>55</v>
       </c>
       <c r="L448" s="2" t="n">
         <v>260</v>
       </c>
       <c r="M448" s="2" t="n">
-        <v>344</v>
+        <v>319</v>
       </c>
       <c r="N448" s="6" t="inlineStr">
         <is>
@@ -25957,13 +25957,13 @@
         <v>77</v>
       </c>
       <c r="K451" s="2" t="n">
-        <v>343</v>
+        <v>313</v>
       </c>
       <c r="L451" s="2" t="n">
         <v>463</v>
       </c>
       <c r="M451" s="2" t="n">
-        <v>883</v>
+        <v>853</v>
       </c>
       <c r="N451" s="4" t="inlineStr">
         <is>
@@ -26074,10 +26074,10 @@
         <v>108</v>
       </c>
       <c r="L453" s="2" t="n">
-        <v>257</v>
+        <v>242</v>
       </c>
       <c r="M453" s="2" t="n">
-        <v>407</v>
+        <v>392</v>
       </c>
       <c r="N453" s="4" t="inlineStr">
         <is>
@@ -26128,13 +26128,13 @@
         <v>1</v>
       </c>
       <c r="K454" s="2" t="n">
-        <v>56</v>
+        <v>413</v>
       </c>
       <c r="L454" s="2" t="n">
-        <v>140</v>
+        <v>130</v>
       </c>
       <c r="M454" s="2" t="n">
-        <v>197</v>
+        <v>544</v>
       </c>
       <c r="N454" s="6" t="inlineStr">
         <is>
@@ -26185,13 +26185,13 @@
         <v>54</v>
       </c>
       <c r="K455" s="2" t="n">
-        <v>29</v>
+        <v>19</v>
       </c>
       <c r="L455" s="2" t="n">
         <v>24</v>
       </c>
       <c r="M455" s="2" t="n">
-        <v>107</v>
+        <v>97</v>
       </c>
       <c r="N455" s="4" t="inlineStr">
         <is>
@@ -26242,13 +26242,13 @@
         <v>98</v>
       </c>
       <c r="K456" s="2" t="n">
-        <v>117</v>
+        <v>112</v>
       </c>
       <c r="L456" s="2" t="n">
         <v>82</v>
       </c>
       <c r="M456" s="2" t="n">
-        <v>297</v>
+        <v>292</v>
       </c>
       <c r="N456" s="4" t="inlineStr">
         <is>
@@ -26356,13 +26356,13 @@
         <v>1</v>
       </c>
       <c r="K458" s="2" t="n">
-        <v>34</v>
+        <v>115</v>
       </c>
       <c r="L458" s="2" t="n">
         <v>95</v>
       </c>
       <c r="M458" s="2" t="n">
-        <v>130</v>
+        <v>211</v>
       </c>
       <c r="N458" s="6" t="inlineStr">
         <is>
@@ -26470,13 +26470,13 @@
         <v>8</v>
       </c>
       <c r="K460" s="2" t="n">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="L460" s="2" t="n">
         <v>55</v>
       </c>
       <c r="M460" s="2" t="n">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="N460" s="6" t="inlineStr">
         <is>
@@ -26641,13 +26641,13 @@
         <v>11</v>
       </c>
       <c r="K463" s="2" t="n">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="L463" s="2" t="n">
         <v>45</v>
       </c>
       <c r="M463" s="2" t="n">
-        <v>205</v>
+        <v>203</v>
       </c>
       <c r="N463" s="4" t="inlineStr">
         <is>
@@ -26701,10 +26701,10 @@
         <v>125</v>
       </c>
       <c r="L464" s="2" t="n">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="M464" s="2" t="n">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="N464" s="6" t="inlineStr">
         <is>
@@ -26812,13 +26812,13 @@
         <v>25</v>
       </c>
       <c r="K466" s="2" t="n">
-        <v>121</v>
+        <v>116</v>
       </c>
       <c r="L466" s="2" t="n">
         <v>78</v>
       </c>
       <c r="M466" s="2" t="n">
-        <v>224</v>
+        <v>219</v>
       </c>
       <c r="N466" s="4" t="inlineStr">
         <is>
@@ -26869,13 +26869,13 @@
         <v>16</v>
       </c>
       <c r="K467" s="2" t="n">
-        <v>319</v>
+        <v>316</v>
       </c>
       <c r="L467" s="2" t="n">
         <v>148</v>
       </c>
       <c r="M467" s="2" t="n">
-        <v>483</v>
+        <v>480</v>
       </c>
       <c r="N467" s="4" t="inlineStr">
         <is>
@@ -26926,13 +26926,13 @@
         <v>11</v>
       </c>
       <c r="K468" s="2" t="n">
-        <v>335</v>
+        <v>334</v>
       </c>
       <c r="L468" s="2" t="n">
         <v>44</v>
       </c>
       <c r="M468" s="2" t="n">
-        <v>390</v>
+        <v>389</v>
       </c>
       <c r="N468" s="4" t="inlineStr">
         <is>
@@ -27727,10 +27727,10 @@
         <v>195</v>
       </c>
       <c r="L482" s="2" t="n">
-        <v>50</v>
+        <v>20</v>
       </c>
       <c r="M482" s="2" t="n">
-        <v>248</v>
+        <v>218</v>
       </c>
       <c r="N482" s="6" t="inlineStr">
         <is>
@@ -28197,8 +28197,348 @@
         <v>1.66</v>
       </c>
     </row>
+    <row r="491">
+      <c r="A491" s="2" t="inlineStr">
+        <is>
+          <t>NOI0088753</t>
+        </is>
+      </c>
+      <c r="B491" s="3" t="inlineStr">
+        <is>
+          <t>TUBO REDONDO 30 X 1.5 (30/27)</t>
+        </is>
+      </c>
+      <c r="C491" s="2" t="inlineStr">
+        <is>
+          <t>TUBO REDONDO</t>
+        </is>
+      </c>
+      <c r="D491" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="E491" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="F491" s="2" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="G491" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="H491" s="2" t="n">
+        <v>0.363</v>
+      </c>
+      <c r="I491" s="2" t="inlineStr">
+        <is>
+          <t>BRUTO</t>
+        </is>
+      </c>
+      <c r="J491" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K491" s="2" t="n">
+        <v>272</v>
+      </c>
+      <c r="L491" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M491" s="2" t="n">
+        <v>272</v>
+      </c>
+      <c r="N491" s="6" t="inlineStr">
+        <is>
+          <t>7/10 Días</t>
+        </is>
+      </c>
+      <c r="O491" s="2" t="n">
+        <v>2.54</v>
+      </c>
+    </row>
+    <row r="492">
+      <c r="A492" s="2" t="inlineStr">
+        <is>
+          <t>NOR0032108</t>
+        </is>
+      </c>
+      <c r="B492" s="3" t="inlineStr">
+        <is>
+          <t>ANGULO 20 X 10 X 1.5</t>
+        </is>
+      </c>
+      <c r="C492" s="2" t="inlineStr">
+        <is>
+          <t>ANGULO</t>
+        </is>
+      </c>
+      <c r="D492" s="2" t="n">
+        <v>20</v>
+      </c>
+      <c r="E492" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="F492" s="2" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="G492" s="2" t="n">
+        <v>6.4</v>
+      </c>
+      <c r="H492" s="2" t="n">
+        <v>0.101</v>
+      </c>
+      <c r="I492" s="2" t="inlineStr">
+        <is>
+          <t>BRUTO</t>
+        </is>
+      </c>
+      <c r="J492" s="2" t="n">
+        <v>534</v>
+      </c>
+      <c r="K492" s="2" t="n">
+        <v>357</v>
+      </c>
+      <c r="L492" s="2" t="n">
+        <v>191</v>
+      </c>
+      <c r="M492" s="2" t="n">
+        <v>1082</v>
+      </c>
+      <c r="N492" s="4" t="inlineStr">
+        <is>
+          <t>Stock</t>
+        </is>
+      </c>
+      <c r="O492" s="2" t="n">
+        <v>0.71</v>
+      </c>
+    </row>
+    <row r="493">
+      <c r="A493" s="2" t="inlineStr">
+        <is>
+          <t>NOR0032002</t>
+        </is>
+      </c>
+      <c r="B493" s="3" t="inlineStr">
+        <is>
+          <t>PLETINA 30 X 4</t>
+        </is>
+      </c>
+      <c r="C493" s="2" t="inlineStr">
+        <is>
+          <t>PLETINA</t>
+        </is>
+      </c>
+      <c r="D493" s="2" t="inlineStr"/>
+      <c r="E493" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="F493" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="G493" s="2" t="n">
+        <v>6.4</v>
+      </c>
+      <c r="H493" s="2" t="n">
+        <v>0.324</v>
+      </c>
+      <c r="I493" s="2" t="inlineStr">
+        <is>
+          <t>BRUTO</t>
+        </is>
+      </c>
+      <c r="J493" s="2" t="n">
+        <v>201</v>
+      </c>
+      <c r="K493" s="2" t="n">
+        <v>221</v>
+      </c>
+      <c r="L493" s="2" t="n">
+        <v>280</v>
+      </c>
+      <c r="M493" s="2" t="n">
+        <v>702</v>
+      </c>
+      <c r="N493" s="4" t="inlineStr">
+        <is>
+          <t>Stock</t>
+        </is>
+      </c>
+      <c r="O493" s="2" t="n">
+        <v>2.27</v>
+      </c>
+    </row>
+    <row r="494">
+      <c r="A494" s="2" t="inlineStr">
+        <is>
+          <t>NOR0032402</t>
+        </is>
+      </c>
+      <c r="B494" s="3" t="inlineStr">
+        <is>
+          <t>TUBO REDONDO 18 X 1.5</t>
+        </is>
+      </c>
+      <c r="C494" s="2" t="inlineStr">
+        <is>
+          <t>TUBO REDONDO</t>
+        </is>
+      </c>
+      <c r="D494" s="2" t="n">
+        <v>18</v>
+      </c>
+      <c r="E494" s="2" t="n">
+        <v>18</v>
+      </c>
+      <c r="F494" s="2" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="G494" s="2" t="n">
+        <v>6.4</v>
+      </c>
+      <c r="H494" s="2" t="n">
+        <v>0.211</v>
+      </c>
+      <c r="I494" s="2" t="inlineStr">
+        <is>
+          <t>BRUTO</t>
+        </is>
+      </c>
+      <c r="J494" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K494" s="2" t="n">
+        <v>390</v>
+      </c>
+      <c r="L494" s="2" t="n">
+        <v>41</v>
+      </c>
+      <c r="M494" s="2" t="n">
+        <v>431</v>
+      </c>
+      <c r="N494" s="6" t="inlineStr">
+        <is>
+          <t>7/10 Días</t>
+        </is>
+      </c>
+      <c r="O494" s="2" t="n">
+        <v>1.48</v>
+      </c>
+    </row>
+    <row r="495">
+      <c r="A495" s="2" t="inlineStr">
+        <is>
+          <t>NOI0088717</t>
+        </is>
+      </c>
+      <c r="B495" s="3" t="inlineStr">
+        <is>
+          <t>TUBO REDONDO 110 X 5 (110/100)</t>
+        </is>
+      </c>
+      <c r="C495" s="2" t="inlineStr">
+        <is>
+          <t>TUBO REDONDO</t>
+        </is>
+      </c>
+      <c r="D495" s="2" t="n">
+        <v>110</v>
+      </c>
+      <c r="E495" s="2" t="n">
+        <v>110</v>
+      </c>
+      <c r="F495" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="G495" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="H495" s="2" t="n">
+        <v>4.452</v>
+      </c>
+      <c r="I495" s="2" t="inlineStr">
+        <is>
+          <t>BRUTO</t>
+        </is>
+      </c>
+      <c r="J495" s="2" t="n">
+        <v>14</v>
+      </c>
+      <c r="K495" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="L495" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M495" s="2" t="n">
+        <v>23</v>
+      </c>
+      <c r="N495" s="4" t="inlineStr">
+        <is>
+          <t>Stock</t>
+        </is>
+      </c>
+      <c r="O495" s="2" t="n">
+        <v>31.16</v>
+      </c>
+    </row>
+    <row r="496">
+      <c r="A496" s="2" t="inlineStr">
+        <is>
+          <t>NOR0032404</t>
+        </is>
+      </c>
+      <c r="B496" s="3" t="inlineStr">
+        <is>
+          <t>TUBO REDONDO 25 X 1,3</t>
+        </is>
+      </c>
+      <c r="C496" s="2" t="inlineStr">
+        <is>
+          <t>TUBO REDONDO</t>
+        </is>
+      </c>
+      <c r="D496" s="2" t="n">
+        <v>25</v>
+      </c>
+      <c r="E496" s="2" t="n">
+        <v>25</v>
+      </c>
+      <c r="F496" s="2" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="G496" s="2" t="n">
+        <v>6.4</v>
+      </c>
+      <c r="H496" s="2" t="n">
+        <v>0.261</v>
+      </c>
+      <c r="I496" s="2" t="inlineStr">
+        <is>
+          <t>BRUTO</t>
+        </is>
+      </c>
+      <c r="J496" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K496" s="2" t="n">
+        <v>175</v>
+      </c>
+      <c r="L496" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M496" s="2" t="n">
+        <v>175</v>
+      </c>
+      <c r="N496" s="6" t="inlineStr">
+        <is>
+          <t>7/10 Días</t>
+        </is>
+      </c>
+      <c r="O496" s="2" t="n">
+        <v>1.83</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:O490"/>
+  <autoFilter ref="A1:O496"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update inventario_expandido.xlsx — 28/07/2026
</commit_message>
<xml_diff>
--- a/inventario_expandido.xlsx
+++ b/inventario_expandido.xlsx
@@ -618,13 +618,13 @@
         <v>45</v>
       </c>
       <c r="K2" s="2" t="n">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="L2" s="2" t="n">
         <v>25</v>
       </c>
       <c r="M2" s="2" t="n">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="N2" s="4" t="inlineStr">
         <is>
@@ -897,13 +897,13 @@
         <v>48</v>
       </c>
       <c r="K7" s="2" t="n">
-        <v>104</v>
+        <v>92</v>
       </c>
       <c r="L7" s="2" t="n">
         <v>8</v>
       </c>
       <c r="M7" s="2" t="n">
-        <v>160</v>
+        <v>148</v>
       </c>
       <c r="N7" s="4" t="inlineStr">
         <is>
@@ -1391,10 +1391,10 @@
         <v>345</v>
       </c>
       <c r="L16" s="2" t="n">
-        <v>56</v>
+        <v>44</v>
       </c>
       <c r="M16" s="2" t="n">
-        <v>543</v>
+        <v>531</v>
       </c>
       <c r="N16" s="4" t="inlineStr">
         <is>
@@ -1547,13 +1547,13 @@
         <v>99</v>
       </c>
       <c r="K19" s="2" t="n">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="L19" s="2" t="n">
         <v>87</v>
       </c>
       <c r="M19" s="2" t="n">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="N19" s="4" t="inlineStr">
         <is>
@@ -1597,7 +1597,7 @@
         </is>
       </c>
       <c r="J20" s="2" t="n">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="K20" s="2" t="n">
         <v>6</v>
@@ -1606,7 +1606,7 @@
         <v>88</v>
       </c>
       <c r="M20" s="2" t="n">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="N20" s="4" t="inlineStr">
         <is>
@@ -1809,7 +1809,7 @@
         </is>
       </c>
       <c r="J24" s="2" t="n">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="K24" s="2" t="n">
         <v>0</v>
@@ -1818,7 +1818,7 @@
         <v>16</v>
       </c>
       <c r="M24" s="2" t="n">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="N24" s="4" t="inlineStr">
         <is>
@@ -2132,13 +2132,13 @@
         <v>318</v>
       </c>
       <c r="K30" s="2" t="n">
-        <v>396</v>
+        <v>1045</v>
       </c>
       <c r="L30" s="2" t="n">
         <v>525</v>
       </c>
       <c r="M30" s="2" t="n">
-        <v>1239</v>
+        <v>1888</v>
       </c>
       <c r="N30" s="4" t="inlineStr">
         <is>
@@ -2297,13 +2297,13 @@
         <v>348</v>
       </c>
       <c r="K33" s="2" t="n">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="L33" s="2" t="n">
         <v>183</v>
       </c>
       <c r="M33" s="2" t="n">
-        <v>701</v>
+        <v>698</v>
       </c>
       <c r="N33" s="4" t="inlineStr">
         <is>
@@ -2630,10 +2630,10 @@
         <v>496</v>
       </c>
       <c r="L39" s="2" t="n">
-        <v>176</v>
+        <v>174</v>
       </c>
       <c r="M39" s="2" t="n">
-        <v>745</v>
+        <v>743</v>
       </c>
       <c r="N39" s="4" t="inlineStr">
         <is>
@@ -2682,13 +2682,13 @@
         <v>15</v>
       </c>
       <c r="K40" s="2" t="n">
-        <v>341</v>
+        <v>333</v>
       </c>
       <c r="L40" s="2" t="n">
         <v>17</v>
       </c>
       <c r="M40" s="2" t="n">
-        <v>373</v>
+        <v>365</v>
       </c>
       <c r="N40" s="4" t="inlineStr">
         <is>
@@ -2792,13 +2792,13 @@
         <v>64</v>
       </c>
       <c r="K42" s="2" t="n">
-        <v>62</v>
+        <v>52</v>
       </c>
       <c r="L42" s="2" t="n">
         <v>57</v>
       </c>
       <c r="M42" s="2" t="n">
-        <v>183</v>
+        <v>173</v>
       </c>
       <c r="N42" s="4" t="inlineStr">
         <is>
@@ -3015,10 +3015,10 @@
         <v>23</v>
       </c>
       <c r="L46" s="2" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="M46" s="2" t="n">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="N46" s="4" t="inlineStr">
         <is>
@@ -3125,10 +3125,10 @@
         <v>150</v>
       </c>
       <c r="L48" s="2" t="n">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="M48" s="2" t="n">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="N48" s="4" t="inlineStr">
         <is>
@@ -3287,13 +3287,13 @@
         <v>8</v>
       </c>
       <c r="K51" s="2" t="n">
-        <v>190</v>
+        <v>185</v>
       </c>
       <c r="L51" s="2" t="n">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="M51" s="2" t="n">
-        <v>248</v>
+        <v>241</v>
       </c>
       <c r="N51" s="6" t="inlineStr">
         <is>
@@ -3342,13 +3342,13 @@
         <v>50</v>
       </c>
       <c r="K52" s="2" t="n">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="L52" s="2" t="n">
         <v>42</v>
       </c>
       <c r="M52" s="2" t="n">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="N52" s="4" t="inlineStr">
         <is>
@@ -3617,13 +3617,13 @@
         <v>0</v>
       </c>
       <c r="K57" s="2" t="n">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="L57" s="2" t="n">
         <v>0</v>
       </c>
       <c r="M57" s="2" t="n">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="N57" s="6" t="inlineStr">
         <is>
@@ -3672,13 +3672,13 @@
         <v>28</v>
       </c>
       <c r="K58" s="2" t="n">
-        <v>13</v>
+        <v>5</v>
       </c>
       <c r="L58" s="2" t="n">
         <v>25</v>
       </c>
       <c r="M58" s="2" t="n">
-        <v>66</v>
+        <v>58</v>
       </c>
       <c r="N58" s="4" t="inlineStr">
         <is>
@@ -4662,13 +4662,13 @@
         <v>401</v>
       </c>
       <c r="K76" s="2" t="n">
-        <v>191</v>
+        <v>179</v>
       </c>
       <c r="L76" s="2" t="n">
         <v>8</v>
       </c>
       <c r="M76" s="2" t="n">
-        <v>600</v>
+        <v>588</v>
       </c>
       <c r="N76" s="4" t="inlineStr">
         <is>
@@ -4772,13 +4772,13 @@
         <v>87</v>
       </c>
       <c r="K78" s="2" t="n">
-        <v>22</v>
+        <v>16</v>
       </c>
       <c r="L78" s="2" t="n">
         <v>272</v>
       </c>
       <c r="M78" s="2" t="n">
-        <v>381</v>
+        <v>375</v>
       </c>
       <c r="N78" s="4" t="inlineStr">
         <is>
@@ -4827,13 +4827,13 @@
         <v>80</v>
       </c>
       <c r="K79" s="2" t="n">
-        <v>175</v>
+        <v>173</v>
       </c>
       <c r="L79" s="2" t="n">
         <v>83</v>
       </c>
       <c r="M79" s="2" t="n">
-        <v>338</v>
+        <v>336</v>
       </c>
       <c r="N79" s="4" t="inlineStr">
         <is>
@@ -5487,13 +5487,13 @@
         <v>14</v>
       </c>
       <c r="K91" s="2" t="n">
-        <v>508</v>
+        <v>506</v>
       </c>
       <c r="L91" s="2" t="n">
         <v>0</v>
       </c>
       <c r="M91" s="2" t="n">
-        <v>522</v>
+        <v>520</v>
       </c>
       <c r="N91" s="4" t="inlineStr">
         <is>
@@ -7953,13 +7953,13 @@
         <v>28</v>
       </c>
       <c r="K135" s="2" t="n">
-        <v>332</v>
+        <v>331</v>
       </c>
       <c r="L135" s="2" t="n">
         <v>187</v>
       </c>
       <c r="M135" s="2" t="n">
-        <v>547</v>
+        <v>546</v>
       </c>
       <c r="N135" s="4" t="inlineStr">
         <is>
@@ -8010,13 +8010,13 @@
         <v>62</v>
       </c>
       <c r="K136" s="2" t="n">
-        <v>385</v>
+        <v>372</v>
       </c>
       <c r="L136" s="2" t="n">
         <v>2</v>
       </c>
       <c r="M136" s="2" t="n">
-        <v>449</v>
+        <v>436</v>
       </c>
       <c r="N136" s="4" t="inlineStr">
         <is>
@@ -8238,13 +8238,13 @@
         <v>0</v>
       </c>
       <c r="K140" s="2" t="n">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="L140" s="2" t="n">
         <v>2</v>
       </c>
       <c r="M140" s="2" t="n">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="N140" s="6" t="inlineStr">
         <is>
@@ -8520,16 +8520,16 @@
         </is>
       </c>
       <c r="J145" s="2" t="n">
-        <v>334</v>
+        <v>333</v>
       </c>
       <c r="K145" s="2" t="n">
-        <v>468</v>
+        <v>434</v>
       </c>
       <c r="L145" s="2" t="n">
         <v>248</v>
       </c>
       <c r="M145" s="2" t="n">
-        <v>1050</v>
+        <v>1015</v>
       </c>
       <c r="N145" s="4" t="inlineStr">
         <is>
@@ -9375,7 +9375,7 @@
         </is>
       </c>
       <c r="J160" s="2" t="n">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="K160" s="2" t="n">
         <v>111</v>
@@ -9384,7 +9384,7 @@
         <v>156</v>
       </c>
       <c r="M160" s="2" t="n">
-        <v>408</v>
+        <v>407</v>
       </c>
       <c r="N160" s="4" t="inlineStr">
         <is>
@@ -9777,13 +9777,13 @@
         <v>102</v>
       </c>
       <c r="K167" s="2" t="n">
-        <v>144</v>
+        <v>140</v>
       </c>
       <c r="L167" s="2" t="n">
         <v>84</v>
       </c>
       <c r="M167" s="2" t="n">
-        <v>330</v>
+        <v>326</v>
       </c>
       <c r="N167" s="4" t="inlineStr">
         <is>
@@ -10005,13 +10005,13 @@
         <v>116</v>
       </c>
       <c r="K171" s="2" t="n">
-        <v>74</v>
+        <v>70</v>
       </c>
       <c r="L171" s="2" t="n">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="M171" s="2" t="n">
-        <v>273</v>
+        <v>268</v>
       </c>
       <c r="N171" s="4" t="inlineStr">
         <is>
@@ -10347,13 +10347,13 @@
         <v>0</v>
       </c>
       <c r="K177" s="2" t="n">
-        <v>27</v>
+        <v>0</v>
       </c>
       <c r="L177" s="2" t="n">
-        <v>21</v>
+        <v>42</v>
       </c>
       <c r="M177" s="2" t="n">
-        <v>48</v>
+        <v>42</v>
       </c>
       <c r="N177" s="6" t="inlineStr">
         <is>
@@ -11886,13 +11886,13 @@
         <v>182</v>
       </c>
       <c r="K204" s="2" t="n">
-        <v>333</v>
+        <v>328</v>
       </c>
       <c r="L204" s="2" t="n">
         <v>238</v>
       </c>
       <c r="M204" s="2" t="n">
-        <v>753</v>
+        <v>748</v>
       </c>
       <c r="N204" s="4" t="inlineStr">
         <is>
@@ -12000,13 +12000,13 @@
         <v>147</v>
       </c>
       <c r="K206" s="2" t="n">
-        <v>56</v>
+        <v>31</v>
       </c>
       <c r="L206" s="2" t="n">
         <v>96</v>
       </c>
       <c r="M206" s="2" t="n">
-        <v>299</v>
+        <v>274</v>
       </c>
       <c r="N206" s="4" t="inlineStr">
         <is>
@@ -12054,16 +12054,16 @@
         </is>
       </c>
       <c r="J207" s="2" t="n">
-        <v>116</v>
+        <v>112</v>
       </c>
       <c r="K207" s="2" t="n">
-        <v>145</v>
+        <v>124</v>
       </c>
       <c r="L207" s="2" t="n">
         <v>41</v>
       </c>
       <c r="M207" s="2" t="n">
-        <v>302</v>
+        <v>277</v>
       </c>
       <c r="N207" s="4" t="inlineStr">
         <is>
@@ -12171,13 +12171,13 @@
         <v>4</v>
       </c>
       <c r="K209" s="2" t="n">
-        <v>70</v>
+        <v>64</v>
       </c>
       <c r="L209" s="2" t="n">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="M209" s="2" t="n">
-        <v>167</v>
+        <v>159</v>
       </c>
       <c r="N209" s="6" t="inlineStr">
         <is>
@@ -13539,13 +13539,13 @@
         <v>76</v>
       </c>
       <c r="K233" s="2" t="n">
-        <v>179</v>
+        <v>164</v>
       </c>
       <c r="L233" s="2" t="n">
         <v>7</v>
       </c>
       <c r="M233" s="2" t="n">
-        <v>262</v>
+        <v>247</v>
       </c>
       <c r="N233" s="4" t="inlineStr">
         <is>
@@ -13824,13 +13824,13 @@
         <v>42</v>
       </c>
       <c r="K238" s="2" t="n">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="L238" s="2" t="n">
         <v>49</v>
       </c>
       <c r="M238" s="2" t="n">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="N238" s="4" t="inlineStr">
         <is>
@@ -14508,13 +14508,13 @@
         <v>18</v>
       </c>
       <c r="K250" s="2" t="n">
-        <v>27</v>
+        <v>20</v>
       </c>
       <c r="L250" s="2" t="n">
         <v>26</v>
       </c>
       <c r="M250" s="2" t="n">
-        <v>71</v>
+        <v>64</v>
       </c>
       <c r="N250" s="4" t="inlineStr">
         <is>
@@ -14676,7 +14676,7 @@
         </is>
       </c>
       <c r="J253" s="2" t="n">
-        <v>53</v>
+        <v>41</v>
       </c>
       <c r="K253" s="2" t="n">
         <v>0</v>
@@ -14685,7 +14685,7 @@
         <v>151</v>
       </c>
       <c r="M253" s="2" t="n">
-        <v>204</v>
+        <v>192</v>
       </c>
       <c r="N253" s="4" t="inlineStr">
         <is>
@@ -14736,13 +14736,13 @@
         <v>193</v>
       </c>
       <c r="K254" s="2" t="n">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="L254" s="2" t="n">
         <v>181</v>
       </c>
       <c r="M254" s="2" t="n">
-        <v>616</v>
+        <v>615</v>
       </c>
       <c r="N254" s="4" t="inlineStr">
         <is>
@@ -14793,13 +14793,13 @@
         <v>0</v>
       </c>
       <c r="K255" s="2" t="n">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="L255" s="2" t="n">
         <v>45</v>
       </c>
       <c r="M255" s="2" t="n">
-        <v>329</v>
+        <v>328</v>
       </c>
       <c r="N255" s="6" t="inlineStr">
         <is>
@@ -14964,13 +14964,13 @@
         <v>139</v>
       </c>
       <c r="K258" s="2" t="n">
-        <v>204</v>
+        <v>198</v>
       </c>
       <c r="L258" s="2" t="n">
         <v>35</v>
       </c>
       <c r="M258" s="2" t="n">
-        <v>378</v>
+        <v>372</v>
       </c>
       <c r="N258" s="4" t="inlineStr">
         <is>
@@ -15021,13 +15021,13 @@
         <v>63</v>
       </c>
       <c r="K259" s="2" t="n">
-        <v>146</v>
+        <v>119</v>
       </c>
       <c r="L259" s="2" t="n">
-        <v>74</v>
+        <v>68</v>
       </c>
       <c r="M259" s="2" t="n">
-        <v>283</v>
+        <v>250</v>
       </c>
       <c r="N259" s="4" t="inlineStr">
         <is>
@@ -15192,13 +15192,13 @@
         <v>94</v>
       </c>
       <c r="K262" s="2" t="n">
-        <v>103</v>
+        <v>100</v>
       </c>
       <c r="L262" s="2" t="n">
         <v>100</v>
       </c>
       <c r="M262" s="2" t="n">
-        <v>297</v>
+        <v>294</v>
       </c>
       <c r="N262" s="4" t="inlineStr">
         <is>
@@ -15249,13 +15249,13 @@
         <v>32</v>
       </c>
       <c r="K263" s="2" t="n">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="L263" s="2" t="n">
         <v>50</v>
       </c>
       <c r="M263" s="2" t="n">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="N263" s="4" t="inlineStr">
         <is>
@@ -15363,13 +15363,13 @@
         <v>38</v>
       </c>
       <c r="K265" s="2" t="n">
-        <v>47</v>
+        <v>27</v>
       </c>
       <c r="L265" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M265" s="2" t="n">
-        <v>86</v>
+        <v>65</v>
       </c>
       <c r="N265" s="4" t="inlineStr">
         <is>
@@ -15762,13 +15762,13 @@
         <v>96</v>
       </c>
       <c r="K272" s="2" t="n">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="L272" s="2" t="n">
         <v>114</v>
       </c>
       <c r="M272" s="2" t="n">
-        <v>273</v>
+        <v>269</v>
       </c>
       <c r="N272" s="4" t="inlineStr">
         <is>
@@ -16278,10 +16278,10 @@
         <v>511</v>
       </c>
       <c r="L281" s="2" t="n">
-        <v>14</v>
+        <v>0</v>
       </c>
       <c r="M281" s="2" t="n">
-        <v>552</v>
+        <v>538</v>
       </c>
       <c r="N281" s="4" t="inlineStr">
         <is>
@@ -16671,7 +16671,7 @@
         </is>
       </c>
       <c r="J288" s="2" t="n">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="K288" s="2" t="n">
         <v>72</v>
@@ -16680,7 +16680,7 @@
         <v>54</v>
       </c>
       <c r="M288" s="2" t="n">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="N288" s="4" t="inlineStr">
         <is>
@@ -17241,16 +17241,16 @@
         </is>
       </c>
       <c r="J298" s="2" t="n">
-        <v>75</v>
+        <v>71</v>
       </c>
       <c r="K298" s="2" t="n">
-        <v>145</v>
+        <v>136</v>
       </c>
       <c r="L298" s="2" t="n">
-        <v>163</v>
+        <v>121</v>
       </c>
       <c r="M298" s="2" t="n">
-        <v>383</v>
+        <v>328</v>
       </c>
       <c r="N298" s="4" t="inlineStr">
         <is>
@@ -17526,16 +17526,16 @@
         </is>
       </c>
       <c r="J303" s="2" t="n">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="K303" s="2" t="n">
         <v>7</v>
       </c>
       <c r="L303" s="2" t="n">
-        <v>82</v>
+        <v>42</v>
       </c>
       <c r="M303" s="2" t="n">
-        <v>127</v>
+        <v>86</v>
       </c>
       <c r="N303" s="4" t="inlineStr">
         <is>
@@ -17589,10 +17589,10 @@
         <v>135</v>
       </c>
       <c r="L304" s="2" t="n">
-        <v>52</v>
+        <v>39</v>
       </c>
       <c r="M304" s="2" t="n">
-        <v>241</v>
+        <v>228</v>
       </c>
       <c r="N304" s="4" t="inlineStr">
         <is>
@@ -17754,16 +17754,16 @@
         </is>
       </c>
       <c r="J307" s="2" t="n">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="K307" s="2" t="n">
-        <v>172</v>
+        <v>158</v>
       </c>
       <c r="L307" s="2" t="n">
-        <v>87</v>
+        <v>77</v>
       </c>
       <c r="M307" s="2" t="n">
-        <v>302</v>
+        <v>276</v>
       </c>
       <c r="N307" s="4" t="inlineStr">
         <is>
@@ -17817,10 +17817,10 @@
         <v>62</v>
       </c>
       <c r="L308" s="2" t="n">
-        <v>29</v>
+        <v>18</v>
       </c>
       <c r="M308" s="2" t="n">
-        <v>133</v>
+        <v>122</v>
       </c>
       <c r="N308" s="4" t="inlineStr">
         <is>
@@ -17925,7 +17925,7 @@
         </is>
       </c>
       <c r="J310" s="2" t="n">
-        <v>175</v>
+        <v>173</v>
       </c>
       <c r="K310" s="2" t="n">
         <v>1</v>
@@ -17934,7 +17934,7 @@
         <v>127</v>
       </c>
       <c r="M310" s="2" t="n">
-        <v>303</v>
+        <v>301</v>
       </c>
       <c r="N310" s="4" t="inlineStr">
         <is>
@@ -18327,13 +18327,13 @@
         <v>93</v>
       </c>
       <c r="K317" s="2" t="n">
-        <v>11</v>
+        <v>4</v>
       </c>
       <c r="L317" s="2" t="n">
         <v>74</v>
       </c>
       <c r="M317" s="2" t="n">
-        <v>178</v>
+        <v>171</v>
       </c>
       <c r="N317" s="4" t="inlineStr">
         <is>
@@ -18381,7 +18381,7 @@
         </is>
       </c>
       <c r="J318" s="2" t="n">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="K318" s="2" t="n">
         <v>77</v>
@@ -18390,7 +18390,7 @@
         <v>38</v>
       </c>
       <c r="M318" s="2" t="n">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="N318" s="4" t="inlineStr">
         <is>
@@ -18669,13 +18669,13 @@
         <v>14</v>
       </c>
       <c r="K323" s="2" t="n">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="L323" s="2" t="n">
         <v>17</v>
       </c>
       <c r="M323" s="2" t="n">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="N323" s="4" t="inlineStr">
         <is>
@@ -19182,13 +19182,13 @@
         <v>7</v>
       </c>
       <c r="K332" s="2" t="n">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="L332" s="2" t="n">
         <v>0</v>
       </c>
       <c r="M332" s="2" t="n">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="N332" s="6" t="inlineStr">
         <is>
@@ -19353,13 +19353,13 @@
         <v>22</v>
       </c>
       <c r="K335" s="2" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="L335" s="2" t="n">
         <v>32</v>
       </c>
       <c r="M335" s="2" t="n">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="N335" s="4" t="inlineStr">
         <is>
@@ -19752,13 +19752,13 @@
         <v>83</v>
       </c>
       <c r="K342" s="2" t="n">
-        <v>96</v>
+        <v>92</v>
       </c>
       <c r="L342" s="2" t="n">
         <v>28</v>
       </c>
       <c r="M342" s="2" t="n">
-        <v>207</v>
+        <v>203</v>
       </c>
       <c r="N342" s="4" t="inlineStr">
         <is>
@@ -19923,13 +19923,13 @@
         <v>4</v>
       </c>
       <c r="K345" s="2" t="n">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="L345" s="2" t="n">
         <v>18</v>
       </c>
       <c r="M345" s="2" t="n">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="N345" s="6" t="inlineStr">
         <is>
@@ -20262,10 +20262,10 @@
         </is>
       </c>
       <c r="J351" s="2" t="n">
-        <v>0</v>
+        <v>56</v>
       </c>
       <c r="K351" s="2" t="n">
-        <v>240</v>
+        <v>184</v>
       </c>
       <c r="L351" s="2" t="n">
         <v>26</v>
@@ -20273,9 +20273,9 @@
       <c r="M351" s="2" t="n">
         <v>266</v>
       </c>
-      <c r="N351" s="6" t="inlineStr">
-        <is>
-          <t>7/10 Días</t>
+      <c r="N351" s="4" t="inlineStr">
+        <is>
+          <t>Stock</t>
         </is>
       </c>
       <c r="O351" s="2" t="n">
@@ -21177,13 +21177,13 @@
         <v>3</v>
       </c>
       <c r="K367" s="2" t="n">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="L367" s="2" t="n">
         <v>7</v>
       </c>
       <c r="M367" s="2" t="n">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="N367" s="6" t="inlineStr">
         <is>
@@ -21237,10 +21237,10 @@
         <v>51</v>
       </c>
       <c r="L368" s="2" t="n">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="M368" s="2" t="n">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="N368" s="4" t="inlineStr">
         <is>
@@ -21462,13 +21462,13 @@
         <v>0</v>
       </c>
       <c r="K372" s="2" t="n">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="L372" s="2" t="n">
         <v>0</v>
       </c>
       <c r="M372" s="2" t="n">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="N372" s="6" t="inlineStr">
         <is>
@@ -22488,13 +22488,13 @@
         <v>27</v>
       </c>
       <c r="K390" s="2" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="L390" s="2" t="n">
         <v>57</v>
       </c>
       <c r="M390" s="2" t="n">
-        <v>103</v>
+        <v>100</v>
       </c>
       <c r="N390" s="4" t="inlineStr">
         <is>
@@ -22713,7 +22713,7 @@
         </is>
       </c>
       <c r="J394" s="2" t="n">
-        <v>114</v>
+        <v>110</v>
       </c>
       <c r="K394" s="2" t="n">
         <v>46</v>
@@ -22722,7 +22722,7 @@
         <v>0</v>
       </c>
       <c r="M394" s="2" t="n">
-        <v>160</v>
+        <v>156</v>
       </c>
       <c r="N394" s="4" t="inlineStr">
         <is>
@@ -22882,7 +22882,7 @@
         </is>
       </c>
       <c r="J397" s="2" t="n">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="K397" s="2" t="n">
         <v>0</v>
@@ -22891,7 +22891,7 @@
         <v>854</v>
       </c>
       <c r="M397" s="2" t="n">
-        <v>1008</v>
+        <v>1007</v>
       </c>
       <c r="N397" s="4" t="inlineStr">
         <is>
@@ -23105,13 +23105,13 @@
         <v>178</v>
       </c>
       <c r="K401" s="2" t="n">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="L401" s="2" t="n">
         <v>91</v>
       </c>
       <c r="M401" s="2" t="n">
-        <v>548</v>
+        <v>547</v>
       </c>
       <c r="N401" s="4" t="inlineStr">
         <is>
@@ -23615,16 +23615,16 @@
         </is>
       </c>
       <c r="J410" s="2" t="n">
-        <v>371</v>
+        <v>370</v>
       </c>
       <c r="K410" s="2" t="n">
-        <v>234</v>
+        <v>213</v>
       </c>
       <c r="L410" s="2" t="n">
         <v>49</v>
       </c>
       <c r="M410" s="2" t="n">
-        <v>654</v>
+        <v>632</v>
       </c>
       <c r="N410" s="4" t="inlineStr">
         <is>
@@ -23732,13 +23732,13 @@
         <v>201</v>
       </c>
       <c r="K412" s="2" t="n">
-        <v>1185</v>
+        <v>1172</v>
       </c>
       <c r="L412" s="2" t="n">
         <v>0</v>
       </c>
       <c r="M412" s="2" t="n">
-        <v>1386</v>
+        <v>1373</v>
       </c>
       <c r="N412" s="4" t="inlineStr">
         <is>
@@ -23789,13 +23789,13 @@
         <v>395</v>
       </c>
       <c r="K413" s="2" t="n">
-        <v>1939</v>
+        <v>1933</v>
       </c>
       <c r="L413" s="2" t="n">
         <v>695</v>
       </c>
       <c r="M413" s="2" t="n">
-        <v>3029</v>
+        <v>3023</v>
       </c>
       <c r="N413" s="4" t="inlineStr">
         <is>
@@ -23846,13 +23846,13 @@
         <v>189</v>
       </c>
       <c r="K414" s="2" t="n">
-        <v>753</v>
+        <v>727</v>
       </c>
       <c r="L414" s="2" t="n">
         <v>91</v>
       </c>
       <c r="M414" s="2" t="n">
-        <v>1033</v>
+        <v>1007</v>
       </c>
       <c r="N414" s="4" t="inlineStr">
         <is>
@@ -23960,13 +23960,13 @@
         <v>279</v>
       </c>
       <c r="K416" s="2" t="n">
-        <v>766</v>
+        <v>754</v>
       </c>
       <c r="L416" s="2" t="n">
-        <v>58</v>
+        <v>43</v>
       </c>
       <c r="M416" s="2" t="n">
-        <v>1103</v>
+        <v>1076</v>
       </c>
       <c r="N416" s="4" t="inlineStr">
         <is>
@@ -24131,13 +24131,13 @@
         <v>67</v>
       </c>
       <c r="K419" s="2" t="n">
-        <v>474</v>
+        <v>454</v>
       </c>
       <c r="L419" s="2" t="n">
-        <v>274</v>
+        <v>259</v>
       </c>
       <c r="M419" s="2" t="n">
-        <v>815</v>
+        <v>780</v>
       </c>
       <c r="N419" s="4" t="inlineStr">
         <is>
@@ -24245,13 +24245,13 @@
         <v>128</v>
       </c>
       <c r="K421" s="2" t="n">
-        <v>280</v>
+        <v>276</v>
       </c>
       <c r="L421" s="2" t="n">
         <v>83</v>
       </c>
       <c r="M421" s="2" t="n">
-        <v>491</v>
+        <v>487</v>
       </c>
       <c r="N421" s="4" t="inlineStr">
         <is>
@@ -24416,13 +24416,13 @@
         <v>85</v>
       </c>
       <c r="K424" s="2" t="n">
-        <v>182</v>
+        <v>177</v>
       </c>
       <c r="L424" s="2" t="n">
-        <v>69</v>
+        <v>35</v>
       </c>
       <c r="M424" s="2" t="n">
-        <v>336</v>
+        <v>297</v>
       </c>
       <c r="N424" s="4" t="inlineStr">
         <is>
@@ -24590,10 +24590,10 @@
         <v>214</v>
       </c>
       <c r="L427" s="2" t="n">
-        <v>226</v>
+        <v>224</v>
       </c>
       <c r="M427" s="2" t="n">
-        <v>619</v>
+        <v>617</v>
       </c>
       <c r="N427" s="4" t="inlineStr">
         <is>
@@ -24704,10 +24704,10 @@
         <v>205</v>
       </c>
       <c r="L429" s="2" t="n">
-        <v>60</v>
+        <v>35</v>
       </c>
       <c r="M429" s="2" t="n">
-        <v>265</v>
+        <v>240</v>
       </c>
       <c r="N429" s="6" t="inlineStr">
         <is>
@@ -24758,13 +24758,13 @@
         <v>141</v>
       </c>
       <c r="K430" s="2" t="n">
-        <v>40</v>
+        <v>30</v>
       </c>
       <c r="L430" s="2" t="n">
         <v>120</v>
       </c>
       <c r="M430" s="2" t="n">
-        <v>301</v>
+        <v>291</v>
       </c>
       <c r="N430" s="4" t="inlineStr">
         <is>
@@ -24872,13 +24872,13 @@
         <v>60</v>
       </c>
       <c r="K432" s="2" t="n">
-        <v>69</v>
+        <v>35</v>
       </c>
       <c r="L432" s="2" t="n">
         <v>31</v>
       </c>
       <c r="M432" s="2" t="n">
-        <v>160</v>
+        <v>126</v>
       </c>
       <c r="N432" s="4" t="inlineStr">
         <is>
@@ -24986,13 +24986,13 @@
         <v>49</v>
       </c>
       <c r="K434" s="2" t="n">
-        <v>401</v>
+        <v>366</v>
       </c>
       <c r="L434" s="2" t="n">
         <v>81</v>
       </c>
       <c r="M434" s="2" t="n">
-        <v>531</v>
+        <v>496</v>
       </c>
       <c r="N434" s="4" t="inlineStr">
         <is>
@@ -25100,13 +25100,13 @@
         <v>0</v>
       </c>
       <c r="K436" s="2" t="n">
-        <v>304</v>
+        <v>302</v>
       </c>
       <c r="L436" s="2" t="n">
         <v>117</v>
       </c>
       <c r="M436" s="2" t="n">
-        <v>421</v>
+        <v>419</v>
       </c>
       <c r="N436" s="6" t="inlineStr">
         <is>
@@ -25271,13 +25271,13 @@
         <v>0</v>
       </c>
       <c r="K439" s="2" t="n">
-        <v>256</v>
+        <v>250</v>
       </c>
       <c r="L439" s="2" t="n">
         <v>94</v>
       </c>
       <c r="M439" s="2" t="n">
-        <v>350</v>
+        <v>344</v>
       </c>
       <c r="N439" s="6" t="inlineStr">
         <is>
@@ -25328,13 +25328,13 @@
         <v>169</v>
       </c>
       <c r="K440" s="2" t="n">
-        <v>272</v>
+        <v>261</v>
       </c>
       <c r="L440" s="2" t="n">
-        <v>176</v>
+        <v>136</v>
       </c>
       <c r="M440" s="2" t="n">
-        <v>617</v>
+        <v>566</v>
       </c>
       <c r="N440" s="4" t="inlineStr">
         <is>
@@ -25442,13 +25442,13 @@
         <v>0</v>
       </c>
       <c r="K442" s="2" t="n">
-        <v>136</v>
+        <v>112</v>
       </c>
       <c r="L442" s="2" t="n">
         <v>59</v>
       </c>
       <c r="M442" s="2" t="n">
-        <v>195</v>
+        <v>171</v>
       </c>
       <c r="N442" s="6" t="inlineStr">
         <is>
@@ -25841,13 +25841,13 @@
         <v>0</v>
       </c>
       <c r="K449" s="2" t="n">
-        <v>39</v>
+        <v>35</v>
       </c>
       <c r="L449" s="2" t="n">
         <v>2</v>
       </c>
       <c r="M449" s="2" t="n">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="N449" s="6" t="inlineStr">
         <is>
@@ -26126,13 +26126,13 @@
         <v>7</v>
       </c>
       <c r="K454" s="2" t="n">
-        <v>303</v>
+        <v>293</v>
       </c>
       <c r="L454" s="2" t="n">
-        <v>233</v>
+        <v>230</v>
       </c>
       <c r="M454" s="2" t="n">
-        <v>543</v>
+        <v>530</v>
       </c>
       <c r="N454" s="6" t="inlineStr">
         <is>
@@ -26183,13 +26183,13 @@
         <v>42</v>
       </c>
       <c r="K455" s="2" t="n">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="L455" s="2" t="n">
         <v>241</v>
       </c>
       <c r="M455" s="2" t="n">
-        <v>361</v>
+        <v>358</v>
       </c>
       <c r="N455" s="4" t="inlineStr">
         <is>
@@ -26240,13 +26240,13 @@
         <v>1</v>
       </c>
       <c r="K456" s="2" t="n">
-        <v>391</v>
+        <v>507</v>
       </c>
       <c r="L456" s="2" t="n">
-        <v>130</v>
+        <v>120</v>
       </c>
       <c r="M456" s="2" t="n">
-        <v>522</v>
+        <v>628</v>
       </c>
       <c r="N456" s="6" t="inlineStr">
         <is>
@@ -26297,13 +26297,13 @@
         <v>51</v>
       </c>
       <c r="K457" s="2" t="n">
-        <v>19</v>
+        <v>3</v>
       </c>
       <c r="L457" s="2" t="n">
         <v>24</v>
       </c>
       <c r="M457" s="2" t="n">
-        <v>94</v>
+        <v>78</v>
       </c>
       <c r="N457" s="4" t="inlineStr">
         <is>
@@ -26354,13 +26354,13 @@
         <v>98</v>
       </c>
       <c r="K458" s="2" t="n">
-        <v>112</v>
+        <v>108</v>
       </c>
       <c r="L458" s="2" t="n">
         <v>82</v>
       </c>
       <c r="M458" s="2" t="n">
-        <v>292</v>
+        <v>288</v>
       </c>
       <c r="N458" s="4" t="inlineStr">
         <is>
@@ -26468,13 +26468,13 @@
         <v>1</v>
       </c>
       <c r="K460" s="2" t="n">
-        <v>115</v>
+        <v>112</v>
       </c>
       <c r="L460" s="2" t="n">
         <v>95</v>
       </c>
       <c r="M460" s="2" t="n">
-        <v>211</v>
+        <v>208</v>
       </c>
       <c r="N460" s="6" t="inlineStr">
         <is>
@@ -26753,13 +26753,13 @@
         <v>11</v>
       </c>
       <c r="K465" s="2" t="n">
-        <v>147</v>
+        <v>95</v>
       </c>
       <c r="L465" s="2" t="n">
         <v>45</v>
       </c>
       <c r="M465" s="2" t="n">
-        <v>203</v>
+        <v>151</v>
       </c>
       <c r="N465" s="4" t="inlineStr">
         <is>
@@ -27038,13 +27038,13 @@
         <v>11</v>
       </c>
       <c r="K470" s="2" t="n">
-        <v>351</v>
+        <v>405</v>
       </c>
       <c r="L470" s="2" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="M470" s="2" t="n">
-        <v>379</v>
+        <v>432</v>
       </c>
       <c r="N470" s="4" t="inlineStr">
         <is>
@@ -27605,7 +27605,7 @@
         </is>
       </c>
       <c r="J480" s="2" t="n">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="K480" s="2" t="n">
         <v>0</v>
@@ -27614,7 +27614,7 @@
         <v>0</v>
       </c>
       <c r="M480" s="2" t="n">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="N480" s="4" t="inlineStr">
         <is>
@@ -27665,13 +27665,13 @@
         <v>0</v>
       </c>
       <c r="K481" s="2" t="n">
-        <v>390</v>
+        <v>389</v>
       </c>
       <c r="L481" s="2" t="n">
         <v>41</v>
       </c>
       <c r="M481" s="2" t="n">
-        <v>431</v>
+        <v>430</v>
       </c>
       <c r="N481" s="6" t="inlineStr">
         <is>
@@ -27779,13 +27779,13 @@
         <v>117</v>
       </c>
       <c r="K483" s="2" t="n">
-        <v>37</v>
+        <v>33</v>
       </c>
       <c r="L483" s="2" t="n">
         <v>330</v>
       </c>
       <c r="M483" s="2" t="n">
-        <v>484</v>
+        <v>480</v>
       </c>
       <c r="N483" s="4" t="inlineStr">
         <is>
@@ -28007,13 +28007,13 @@
         <v>8</v>
       </c>
       <c r="K487" s="2" t="n">
-        <v>32</v>
+        <v>26</v>
       </c>
       <c r="L487" s="2" t="n">
         <v>0</v>
       </c>
       <c r="M487" s="2" t="n">
-        <v>40</v>
+        <v>34</v>
       </c>
       <c r="N487" s="6" t="inlineStr">
         <is>
@@ -28292,13 +28292,13 @@
         <v>7</v>
       </c>
       <c r="K492" s="2" t="n">
-        <v>30</v>
+        <v>24</v>
       </c>
       <c r="L492" s="2" t="n">
         <v>30</v>
       </c>
       <c r="M492" s="2" t="n">
-        <v>67</v>
+        <v>61</v>
       </c>
       <c r="N492" s="6" t="inlineStr">
         <is>

</xml_diff>